<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-18
</commit_message>
<xml_diff>
--- a/output/profile_1_civil_vias_sst_tracker.xlsx
+++ b/output/profile_1_civil_vias_sst_tracker.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K637"/>
+  <dimension ref="A1:K640"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -25399,26 +25399,26 @@
     <row r="530" ht="22" customHeight="1">
       <c r="A530" s="2" t="inlineStr">
         <is>
-          <t>4426b2c17306f519</t>
+          <t>b55954435d797fc0</t>
         </is>
       </c>
       <c r="B530" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 05:09</t>
+          <t>2026-10-18 14:24</t>
         </is>
       </c>
       <c r="C530" s="3" t="inlineStr">
         <is>
-          <t>Residente de Seguridad y Salud en el trabajo</t>
+          <t>Proyectista civil - semi senior</t>
         </is>
       </c>
       <c r="D530" s="3" t="inlineStr">
         <is>
-          <t>Cal y Mayor y Asociados S.C</t>
-        </is>
-      </c>
-      <c r="E530" s="8" t="n">
-        <v>0.48</v>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E530" s="7" t="n">
+        <v>0.5</v>
       </c>
       <c r="F530" s="2" t="inlineStr">
         <is>
@@ -25426,17 +25426,13 @@
         </is>
       </c>
       <c r="G530" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-residente-de-seguridad-y-salud-en-el-trabajo-sst-sst-en-bogota-dc-D67E64C3D53E0D6961373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H530" s="6" t="inlineStr">
-        <is>
-          <t>$ 4.200.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/proyectista-civil-semi-senior-1886736963", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H530" s="6" t="inlineStr"/>
       <c r="I530" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J530" s="2" t="inlineStr">
@@ -25449,26 +25445,26 @@
     <row r="531" ht="22" customHeight="1">
       <c r="A531" s="2" t="inlineStr">
         <is>
-          <t>83015d6afb890f1d</t>
+          <t>eaecdc7883c5c946</t>
         </is>
       </c>
       <c r="B531" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 05:09</t>
+          <t>2026-10-18 14:24</t>
         </is>
       </c>
       <c r="C531" s="3" t="inlineStr">
         <is>
-          <t>Analista/profesional HSEQ / SST Sesquile o Alrededores</t>
+          <t>Analista de aplicaciones e infraestructura ti</t>
         </is>
       </c>
       <c r="D531" s="3" t="inlineStr">
         <is>
-          <t>ACTIVOS S A S</t>
-        </is>
-      </c>
-      <c r="E531" s="8" t="n">
-        <v>0.48</v>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E531" s="7" t="n">
+        <v>0.5</v>
       </c>
       <c r="F531" s="2" t="inlineStr">
         <is>
@@ -25476,17 +25472,13 @@
         </is>
       </c>
       <c r="G531" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analistaprofesional-hseq-sst-sesquile-o-alrededores-sector-consumo-masivo-en-sesquile-632A9566338A59E361373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H531" s="6" t="inlineStr">
-        <is>
-          <t>$ 4.000.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-aplicaciones-e-infraestructura-ti-1886763122", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H531" s="6" t="inlineStr"/>
       <c r="I531" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad parcial en infraestructura vial y transporte. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J531" s="2" t="inlineStr">
@@ -25499,26 +25491,26 @@
     <row r="532" ht="22" customHeight="1">
       <c r="A532" s="2" t="inlineStr">
         <is>
-          <t>bc0b38b5129e0905</t>
+          <t>94e5a72874057837</t>
         </is>
       </c>
       <c r="B532" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 05:09</t>
+          <t>2026-10-18 14:24</t>
         </is>
       </c>
       <c r="C532" s="3" t="inlineStr">
         <is>
-          <t>Profesional en seguridad y salud en el trabajo SST</t>
+          <t>Analista de seguridad y salud en el trabajo</t>
         </is>
       </c>
       <c r="D532" s="3" t="inlineStr">
         <is>
-          <t>Seguridad y Vigilancia Exito de Colombia</t>
-        </is>
-      </c>
-      <c r="E532" s="8" t="n">
-        <v>0.48</v>
+          <t>COMFACUNDI</t>
+        </is>
+      </c>
+      <c r="E532" s="7" t="n">
+        <v>0.5</v>
       </c>
       <c r="F532" s="2" t="inlineStr">
         <is>
@@ -25526,17 +25518,13 @@
         </is>
       </c>
       <c r="G532" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-profesional-en-seguridad-y-salud-en-el-trabajo-sst-con-experiencia-y-conocimiento-en-pesv-en-bogota-dc-A7CA6F8805D1C53B61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H532" s="6" t="inlineStr">
-        <is>
-          <t>$ 3.200.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-seguridad-y-salud-en-el-trabajo-1886762763", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H532" s="6" t="inlineStr"/>
       <c r="I532" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J532" s="2" t="inlineStr">
@@ -25549,7 +25537,7 @@
     <row r="533" ht="22" customHeight="1">
       <c r="A533" s="2" t="inlineStr">
         <is>
-          <t>e15ce00dbe5c21b5</t>
+          <t>4426b2c17306f519</t>
         </is>
       </c>
       <c r="B533" s="2" t="inlineStr">
@@ -25559,12 +25547,12 @@
       </c>
       <c r="C533" s="3" t="inlineStr">
         <is>
-          <t>Tecnólogo HSEQ / Seguridad y Salud en el Trabajo</t>
+          <t>Residente de Seguridad y Salud en el trabajo</t>
         </is>
       </c>
       <c r="D533" s="3" t="inlineStr">
         <is>
-          <t>Lighgen Ingeniería Ltda</t>
+          <t>Cal y Mayor y Asociados S.C</t>
         </is>
       </c>
       <c r="E533" s="8" t="n">
@@ -25576,10 +25564,14 @@
         </is>
       </c>
       <c r="G533" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnologo-hseq-seguridad-y-salud-en-el-trabajo-con-experiencia-2-anos-en-bogota-dc-87DB3FCAFEA8E12861373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H533" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-residente-de-seguridad-y-salud-en-el-trabajo-sst-sst-en-bogota-dc-D67E64C3D53E0D6961373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H533" s="6" t="inlineStr">
+        <is>
+          <t>$ 4.200.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I533" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -25595,7 +25587,7 @@
     <row r="534" ht="22" customHeight="1">
       <c r="A534" s="2" t="inlineStr">
         <is>
-          <t>1f3bf8b16a58f0b4</t>
+          <t>83015d6afb890f1d</t>
         </is>
       </c>
       <c r="B534" s="2" t="inlineStr">
@@ -25605,12 +25597,12 @@
       </c>
       <c r="C534" s="3" t="inlineStr">
         <is>
-          <t>Inspector (a) de vias y urbanismo</t>
+          <t>Analista/profesional HSEQ / SST Sesquile o Alrededores</t>
         </is>
       </c>
       <c r="D534" s="3" t="inlineStr">
         <is>
-          <t>METRO LINEA 1 S.A.S.</t>
+          <t>ACTIVOS S A S</t>
         </is>
       </c>
       <c r="E534" s="8" t="n">
@@ -25622,13 +25614,17 @@
         </is>
       </c>
       <c r="G534" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/inspector-a-de-vias-y-urbanismo-1886728733", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H534" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analistaprofesional-hseq-sst-sesquile-o-alrededores-sector-consumo-masivo-en-sesquile-632A9566338A59E361373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H534" s="6" t="inlineStr">
+        <is>
+          <t>$ 4.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I534" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia técnica en infraestructura vial, diseño geométrico y pavimentos. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J534" s="2" t="inlineStr">
@@ -25641,7 +25637,7 @@
     <row r="535" ht="22" customHeight="1">
       <c r="A535" s="2" t="inlineStr">
         <is>
-          <t>8fd843a922654d9e</t>
+          <t>bc0b38b5129e0905</t>
         </is>
       </c>
       <c r="B535" s="2" t="inlineStr">
@@ -25651,12 +25647,12 @@
       </c>
       <c r="C535" s="3" t="inlineStr">
         <is>
-          <t>Oficial de obra</t>
+          <t>Profesional en seguridad y salud en el trabajo SST</t>
         </is>
       </c>
       <c r="D535" s="3" t="inlineStr">
         <is>
-          <t>TERMOTECNICA COINDUSTRIAL SAS</t>
+          <t>Seguridad y Vigilancia Exito de Colombia</t>
         </is>
       </c>
       <c r="E535" s="8" t="n">
@@ -25668,13 +25664,17 @@
         </is>
       </c>
       <c r="G535" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/oficial-de-obra-puentevias-1886766237", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H535" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-profesional-en-seguridad-y-salud-en-el-trabajo-sst-con-experiencia-y-conocimiento-en-pesv-en-bogota-dc-A7CA6F8805D1C53B61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H535" s="6" t="inlineStr">
+        <is>
+          <t>$ 3.200.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I535" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia técnica en infraestructura vial, diseño geométrico y pavimentos. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J535" s="2" t="inlineStr">
@@ -25687,7 +25687,7 @@
     <row r="536" ht="22" customHeight="1">
       <c r="A536" s="2" t="inlineStr">
         <is>
-          <t>03eab73111095faa</t>
+          <t>e15ce00dbe5c21b5</t>
         </is>
       </c>
       <c r="B536" s="2" t="inlineStr">
@@ -25697,12 +25697,12 @@
       </c>
       <c r="C536" s="3" t="inlineStr">
         <is>
-          <t>Residente estructuras</t>
+          <t>Tecnólogo HSEQ / Seguridad y Salud en el Trabajo</t>
         </is>
       </c>
       <c r="D536" s="3" t="inlineStr">
         <is>
-          <t>CONCONCRETO S.A.</t>
+          <t>Lighgen Ingeniería Ltda</t>
         </is>
       </c>
       <c r="E536" s="8" t="n">
@@ -25714,13 +25714,13 @@
         </is>
       </c>
       <c r="G536" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/residente-estructuras-experiencia-en-infraestructura-vial-y-talud-1886757305", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnologo-hseq-seguridad-y-salud-en-el-trabajo-con-experiencia-2-anos-en-bogota-dc-87DB3FCAFEA8E12861373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H536" s="6" t="inlineStr"/>
       <c r="I536" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia técnica en infraestructura vial, diseño geométrico y pavimentos. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J536" s="2" t="inlineStr">
@@ -25733,7 +25733,7 @@
     <row r="537" ht="22" customHeight="1">
       <c r="A537" s="2" t="inlineStr">
         <is>
-          <t>c5911c7562546e3c</t>
+          <t>1f3bf8b16a58f0b4</t>
         </is>
       </c>
       <c r="B537" s="2" t="inlineStr">
@@ -25743,12 +25743,12 @@
       </c>
       <c r="C537" s="3" t="inlineStr">
         <is>
-          <t>Profesional con experiencia en el sector de transporte marítimo y/o por vías navegables</t>
+          <t>Inspector (a) de vias y urbanismo</t>
         </is>
       </c>
       <c r="D537" s="3" t="inlineStr">
         <is>
-          <t>ICONTEC</t>
+          <t>METRO LINEA 1 S.A.S.</t>
         </is>
       </c>
       <c r="E537" s="8" t="n">
@@ -25760,7 +25760,7 @@
         </is>
       </c>
       <c r="G537" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/profesional-con-experiencia-en-el-sector-de-transporte-maritimo-y-o-por-vias-navegables-1886761682", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/inspector-a-de-vias-y-urbanismo-1886728733", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H537" s="6" t="inlineStr"/>
@@ -25779,7 +25779,7 @@
     <row r="538" ht="22" customHeight="1">
       <c r="A538" s="2" t="inlineStr">
         <is>
-          <t>c2903e245a44de39</t>
+          <t>8fd843a922654d9e</t>
         </is>
       </c>
       <c r="B538" s="2" t="inlineStr">
@@ -25789,7 +25789,7 @@
       </c>
       <c r="C538" s="3" t="inlineStr">
         <is>
-          <t>Encargado de obra</t>
+          <t>Oficial de obra</t>
         </is>
       </c>
       <c r="D538" s="3" t="inlineStr">
@@ -25806,7 +25806,7 @@
         </is>
       </c>
       <c r="G538" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/encargado-de-obra-puentes-vias-1886762620", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/oficial-de-obra-puentevias-1886766237", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H538" s="6" t="inlineStr"/>
@@ -25825,7 +25825,7 @@
     <row r="539" ht="22" customHeight="1">
       <c r="A539" s="2" t="inlineStr">
         <is>
-          <t>a5bd833e8b837d34</t>
+          <t>03eab73111095faa</t>
         </is>
       </c>
       <c r="B539" s="2" t="inlineStr">
@@ -25835,12 +25835,12 @@
       </c>
       <c r="C539" s="3" t="inlineStr">
         <is>
-          <t>Residente en seguridad y salud en el trabajo</t>
+          <t>Residente estructuras</t>
         </is>
       </c>
       <c r="D539" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>CONCONCRETO S.A.</t>
         </is>
       </c>
       <c r="E539" s="8" t="n">
@@ -25852,13 +25852,13 @@
         </is>
       </c>
       <c r="G539" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/residente-en-seguridad-y-salud-en-el-trabajo-sst-1886762728", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/residente-estructuras-experiencia-en-infraestructura-vial-y-talud-1886757305", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H539" s="6" t="inlineStr"/>
       <c r="I539" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia técnica en infraestructura vial, diseño geométrico y pavimentos. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J539" s="2" t="inlineStr">
@@ -25871,7 +25871,7 @@
     <row r="540" ht="22" customHeight="1">
       <c r="A540" s="2" t="inlineStr">
         <is>
-          <t>55e7967f3b4afa02</t>
+          <t>c5911c7562546e3c</t>
         </is>
       </c>
       <c r="B540" s="2" t="inlineStr">
@@ -25881,12 +25881,12 @@
       </c>
       <c r="C540" s="3" t="inlineStr">
         <is>
-          <t>Tecnólogo/a en Seguridad y Salud en el Trabajo</t>
+          <t>Profesional con experiencia en el sector de transporte marítimo y/o por vías navegables</t>
         </is>
       </c>
       <c r="D540" s="3" t="inlineStr">
         <is>
-          <t>EOSOL</t>
+          <t>ICONTEC</t>
         </is>
       </c>
       <c r="E540" s="8" t="n">
@@ -25898,13 +25898,13 @@
         </is>
       </c>
       <c r="G540" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/tecn%C3%B3logo-a-en-seguridad-y-salud-en-el-trabajo-sst-at-eosol-4464868638", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/profesional-con-experiencia-en-el-sector-de-transporte-maritimo-y-o-por-vias-navegables-1886761682", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H540" s="6" t="inlineStr"/>
       <c r="I540" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia técnica en infraestructura vial, diseño geométrico y pavimentos. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J540" s="2" t="inlineStr">
@@ -25917,7 +25917,7 @@
     <row r="541" ht="22" customHeight="1">
       <c r="A541" s="2" t="inlineStr">
         <is>
-          <t>6df905e482fe09b1</t>
+          <t>c2903e245a44de39</t>
         </is>
       </c>
       <c r="B541" s="2" t="inlineStr">
@@ -25927,12 +25927,12 @@
       </c>
       <c r="C541" s="3" t="inlineStr">
         <is>
-          <t>Aprendiz SENA - Técnico(a) de Salud Ocupacional o Seguridad y Salud en el Trabajo - Ginebra</t>
+          <t>Encargado de obra</t>
         </is>
       </c>
       <c r="D541" s="3" t="inlineStr">
         <is>
-          <t>Cargill</t>
+          <t>TERMOTECNICA COINDUSTRIAL SAS</t>
         </is>
       </c>
       <c r="E541" s="8" t="n">
@@ -25944,13 +25944,13 @@
         </is>
       </c>
       <c r="G541" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/aprendiz-sena-t%C3%A9cnico-a-de-salud-ocupacional-o-seguridad-y-salud-en-el-trabajo-ginebra-at-cargill-4466994159", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/encargado-de-obra-puentes-vias-1886762620", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H541" s="6" t="inlineStr"/>
       <c r="I541" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia técnica en infraestructura vial, diseño geométrico y pavimentos. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J541" s="2" t="inlineStr">
@@ -25963,7 +25963,7 @@
     <row r="542" ht="22" customHeight="1">
       <c r="A542" s="2" t="inlineStr">
         <is>
-          <t>06656fbb2d452086</t>
+          <t>a5bd833e8b837d34</t>
         </is>
       </c>
       <c r="B542" s="2" t="inlineStr">
@@ -25973,12 +25973,12 @@
       </c>
       <c r="C542" s="3" t="inlineStr">
         <is>
-          <t>Residente de Seguridad y Salud en el trabajo</t>
+          <t>Residente en seguridad y salud en el trabajo</t>
         </is>
       </c>
       <c r="D542" s="3" t="inlineStr">
         <is>
-          <t>Grupo Cal y Mayor</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E542" s="8" t="n">
@@ -25990,7 +25990,7 @@
         </is>
       </c>
       <c r="G542" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/residente-de-seguridad-y-salud-en-el-trabajo-sst-at-cal-y-mayor-4468610572", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/residente-en-seguridad-y-salud-en-el-trabajo-sst-1886762728", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H542" s="6" t="inlineStr"/>
@@ -26009,7 +26009,7 @@
     <row r="543" ht="22" customHeight="1">
       <c r="A543" s="2" t="inlineStr">
         <is>
-          <t>7796e088dce85b5a</t>
+          <t>55e7967f3b4afa02</t>
         </is>
       </c>
       <c r="B543" s="2" t="inlineStr">
@@ -26019,16 +26019,16 @@
       </c>
       <c r="C543" s="3" t="inlineStr">
         <is>
-          <t>Civil Engineer (Fire Sprinkler Design))</t>
+          <t>Tecnólogo/a en Seguridad y Salud en el Trabajo</t>
         </is>
       </c>
       <c r="D543" s="3" t="inlineStr">
         <is>
-          <t>Hyremote</t>
+          <t>EOSOL</t>
         </is>
       </c>
       <c r="E543" s="8" t="n">
-        <v>0.45</v>
+        <v>0.48</v>
       </c>
       <c r="F543" s="2" t="inlineStr">
         <is>
@@ -26036,17 +26036,13 @@
         </is>
       </c>
       <c r="G543" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-civil-engineer-fire-sprinkler-design-english-c1-remote-en-bogota-dc-A2EE61A321FC0D3361373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H543" s="6" t="inlineStr">
-        <is>
-          <t>$ 4.499.993,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/tecn%C3%B3logo-a-en-seguridad-y-salud-en-el-trabajo-sst-at-eosol-4464868638", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H543" s="6" t="inlineStr"/>
       <c r="I543" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J543" s="2" t="inlineStr">
@@ -26059,7 +26055,7 @@
     <row r="544" ht="22" customHeight="1">
       <c r="A544" s="2" t="inlineStr">
         <is>
-          <t>48463526ca7c8ada</t>
+          <t>6df905e482fe09b1</t>
         </is>
       </c>
       <c r="B544" s="2" t="inlineStr">
@@ -26069,16 +26065,16 @@
       </c>
       <c r="C544" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero Civil Especialista en Hidrología e Hidráulica</t>
+          <t>Aprendiz SENA - Técnico(a) de Salud Ocupacional o Seguridad y Salud en el Trabajo - Ginebra</t>
         </is>
       </c>
       <c r="D544" s="3" t="inlineStr">
         <is>
-          <t>ATLAS INFRASTRUCTURE DESIGN LIMITED</t>
+          <t>Cargill</t>
         </is>
       </c>
       <c r="E544" s="8" t="n">
-        <v>0.45</v>
+        <v>0.48</v>
       </c>
       <c r="F544" s="2" t="inlineStr">
         <is>
@@ -26086,17 +26082,13 @@
         </is>
       </c>
       <c r="G544" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingeniero-civil-especialista-en-hidrologia-e-hidraulica-tiempo-completo-en-remoto-y-de-larga-duracion-en-colombia-027FB718364F4C7761373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H544" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/aprendiz-sena-t%C3%A9cnico-a-de-salud-ocupacional-o-seguridad-y-salud-en-el-trabajo-ginebra-at-cargill-4466994159", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H544" s="6" t="inlineStr"/>
       <c r="I544" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J544" s="2" t="inlineStr">
@@ -26109,7 +26101,7 @@
     <row r="545" ht="22" customHeight="1">
       <c r="A545" s="2" t="inlineStr">
         <is>
-          <t>2d406567ceb21bf8</t>
+          <t>06656fbb2d452086</t>
         </is>
       </c>
       <c r="B545" s="2" t="inlineStr">
@@ -26119,16 +26111,16 @@
       </c>
       <c r="C545" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero Civil de Diseño</t>
+          <t>Residente de Seguridad y Salud en el trabajo</t>
         </is>
       </c>
       <c r="D545" s="3" t="inlineStr">
         <is>
-          <t>ATLAS INFRASTRUCTURE DESIGN LIMITED</t>
+          <t>Grupo Cal y Mayor</t>
         </is>
       </c>
       <c r="E545" s="8" t="n">
-        <v>0.45</v>
+        <v>0.48</v>
       </c>
       <c r="F545" s="2" t="inlineStr">
         <is>
@@ -26136,17 +26128,13 @@
         </is>
       </c>
       <c r="G545" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingeniero-civil-de-diseno-tiempo-completo-en-remoto-en-colombia-4CB8F30B6D8FBF7261373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H545" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/residente-de-seguridad-y-salud-en-el-trabajo-sst-at-cal-y-mayor-4468610572", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H545" s="6" t="inlineStr"/>
       <c r="I545" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J545" s="2" t="inlineStr">
@@ -26159,7 +26147,7 @@
     <row r="546" ht="22" customHeight="1">
       <c r="A546" s="2" t="inlineStr">
         <is>
-          <t>4d4013d19591d2a5</t>
+          <t>7796e088dce85b5a</t>
         </is>
       </c>
       <c r="B546" s="2" t="inlineStr">
@@ -26169,12 +26157,12 @@
       </c>
       <c r="C546" s="3" t="inlineStr">
         <is>
-          <t>Especialista en Salud y Seguridad en el trabajo con especialización en medio Ambiente</t>
+          <t>Civil Engineer (Fire Sprinkler Design))</t>
         </is>
       </c>
       <c r="D546" s="3" t="inlineStr">
         <is>
-          <t>DEXTERA S.A.S</t>
+          <t>Hyremote</t>
         </is>
       </c>
       <c r="E546" s="8" t="n">
@@ -26186,10 +26174,14 @@
         </is>
       </c>
       <c r="G546" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-especialista-en-salud-y-seguridad-en-el-trabajo-con-especializacion-en-medio-ambiente-en-bogota-dc-68C95C2F64D6648561373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H546" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-civil-engineer-fire-sprinkler-design-english-c1-remote-en-bogota-dc-A2EE61A321FC0D3361373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H546" s="6" t="inlineStr">
+        <is>
+          <t>$ 4.499.993,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I546" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -26205,7 +26197,7 @@
     <row r="547" ht="22" customHeight="1">
       <c r="A547" s="2" t="inlineStr">
         <is>
-          <t>cf70d2ca6e5c25de</t>
+          <t>48463526ca7c8ada</t>
         </is>
       </c>
       <c r="B547" s="2" t="inlineStr">
@@ -26215,12 +26207,12 @@
       </c>
       <c r="C547" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero civil</t>
+          <t>Ingeniero Civil Especialista en Hidrología e Hidráulica</t>
         </is>
       </c>
       <c r="D547" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>ATLAS INFRASTRUCTURE DESIGN LIMITED</t>
         </is>
       </c>
       <c r="E547" s="8" t="n">
@@ -26232,12 +26224,12 @@
         </is>
       </c>
       <c r="G547" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingeniero-civil-con-experiencia-en-sistemas-fotovoltaicos-en-bogota-dc-8BCBCD7DF8FE589C61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingeniero-civil-especialista-en-hidrologia-e-hidraulica-tiempo-completo-en-remoto-y-de-larga-duracion-en-colombia-027FB718364F4C7761373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H547" s="6" t="inlineStr">
         <is>
-          <t>$ 3.300.000,00 (Mensual)</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="I547" s="3" t="inlineStr">
@@ -26255,7 +26247,7 @@
     <row r="548" ht="22" customHeight="1">
       <c r="A548" s="2" t="inlineStr">
         <is>
-          <t>bb8237cc7ed8d56b</t>
+          <t>2d406567ceb21bf8</t>
         </is>
       </c>
       <c r="B548" s="2" t="inlineStr">
@@ -26265,12 +26257,12 @@
       </c>
       <c r="C548" s="3" t="inlineStr">
         <is>
-          <t>Coordinador de Proyectos Mejoramientos de Vivienda</t>
+          <t>Ingeniero Civil de Diseño</t>
         </is>
       </c>
       <c r="D548" s="3" t="inlineStr">
         <is>
-          <t>Socya</t>
+          <t>ATLAS INFRASTRUCTURE DESIGN LIMITED</t>
         </is>
       </c>
       <c r="E548" s="8" t="n">
@@ -26282,10 +26274,14 @@
         </is>
       </c>
       <c r="G548" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-coordinador-de-proyectos-mejoramientos-de-vivienda-medellin-antioquia-en-medellin-7E29781CFFD4058961373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H548" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingeniero-civil-de-diseno-tiempo-completo-en-remoto-en-colombia-4CB8F30B6D8FBF7261373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H548" s="6" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="I548" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -26301,7 +26297,7 @@
     <row r="549" ht="22" customHeight="1">
       <c r="A549" s="2" t="inlineStr">
         <is>
-          <t>c41dc091e876cb10</t>
+          <t>4d4013d19591d2a5</t>
         </is>
       </c>
       <c r="B549" s="2" t="inlineStr">
@@ -26311,12 +26307,12 @@
       </c>
       <c r="C549" s="3" t="inlineStr">
         <is>
-          <t>Especialista de Milk Collection</t>
+          <t>Especialista en Salud y Seguridad en el trabajo con especialización en medio Ambiente</t>
         </is>
       </c>
       <c r="D549" s="3" t="inlineStr">
         <is>
-          <t>LACTALIS</t>
+          <t>DEXTERA S.A.S</t>
         </is>
       </c>
       <c r="E549" s="8" t="n">
@@ -26328,14 +26324,10 @@
         </is>
       </c>
       <c r="G549" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-especialista-de-milk-collection-optimizacion-y-analisis-de-datos-en-bogota-dc-B007F5172FEA6F6461373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H549" s="6" t="inlineStr">
-        <is>
-          <t>$ 6.000.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-especialista-en-salud-y-seguridad-en-el-trabajo-con-especializacion-en-medio-ambiente-en-bogota-dc-68C95C2F64D6648561373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H549" s="6" t="inlineStr"/>
       <c r="I549" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -26351,7 +26343,7 @@
     <row r="550" ht="22" customHeight="1">
       <c r="A550" s="2" t="inlineStr">
         <is>
-          <t>4f38d6c20430e4bb</t>
+          <t>cf70d2ca6e5c25de</t>
         </is>
       </c>
       <c r="B550" s="2" t="inlineStr">
@@ -26361,12 +26353,12 @@
       </c>
       <c r="C550" s="3" t="inlineStr">
         <is>
-          <t>ingeniero civil</t>
+          <t>Ingeniero civil</t>
         </is>
       </c>
       <c r="D550" s="3" t="inlineStr">
         <is>
-          <t>EVALTEC S.A.S.</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E550" s="8" t="n">
@@ -26378,10 +26370,14 @@
         </is>
       </c>
       <c r="G550" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingeniero-civil-o-areas-afines-en-medellin-0E02F682AB12631061373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H550" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingeniero-civil-con-experiencia-en-sistemas-fotovoltaicos-en-bogota-dc-8BCBCD7DF8FE589C61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H550" s="6" t="inlineStr">
+        <is>
+          <t>$ 3.300.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I550" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -26397,7 +26393,7 @@
     <row r="551" ht="22" customHeight="1">
       <c r="A551" s="2" t="inlineStr">
         <is>
-          <t>af38dd28fbbad8f4</t>
+          <t>bb8237cc7ed8d56b</t>
         </is>
       </c>
       <c r="B551" s="2" t="inlineStr">
@@ -26407,12 +26403,12 @@
       </c>
       <c r="C551" s="3" t="inlineStr">
         <is>
-          <t>Tecnólogo Auxiliar Civil</t>
+          <t>Coordinador de Proyectos Mejoramientos de Vivienda</t>
         </is>
       </c>
       <c r="D551" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>Socya</t>
         </is>
       </c>
       <c r="E551" s="8" t="n">
@@ -26424,7 +26420,7 @@
         </is>
       </c>
       <c r="G551" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnologo-auxiliar-civil-antioquia-en-liborina-B380460DDA9F98D061373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-coordinador-de-proyectos-mejoramientos-de-vivienda-medellin-antioquia-en-medellin-7E29781CFFD4058961373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H551" s="6" t="inlineStr"/>
@@ -26443,7 +26439,7 @@
     <row r="552" ht="22" customHeight="1">
       <c r="A552" s="2" t="inlineStr">
         <is>
-          <t>19e74768ce848880</t>
+          <t>c41dc091e876cb10</t>
         </is>
       </c>
       <c r="B552" s="2" t="inlineStr">
@@ -26453,12 +26449,12 @@
       </c>
       <c r="C552" s="3" t="inlineStr">
         <is>
-          <t>Coordinador HSEQ</t>
+          <t>Especialista de Milk Collection</t>
         </is>
       </c>
       <c r="D552" s="3" t="inlineStr">
         <is>
-          <t>Agencia de empleo de Comfenalco Cartagena</t>
+          <t>LACTALIS</t>
         </is>
       </c>
       <c r="E552" s="8" t="n">
@@ -26470,17 +26466,17 @@
         </is>
       </c>
       <c r="G552" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-coordinador-hseq-especialista-en-seguridad-y-salud-en-el-trabajo-salud-ocupacional-en-cartagena-de-indias-1EAF6570FC054C2661373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-especialista-de-milk-collection-optimizacion-y-analisis-de-datos-en-bogota-dc-B007F5172FEA6F6461373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H552" s="6" t="inlineStr">
         <is>
-          <t>$ 2.500.000,00 (Mensual)</t>
+          <t>$ 6.000.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I552" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J552" s="2" t="inlineStr">
@@ -26493,7 +26489,7 @@
     <row r="553" ht="22" customHeight="1">
       <c r="A553" s="2" t="inlineStr">
         <is>
-          <t>38c9a9481706de58</t>
+          <t>4f38d6c20430e4bb</t>
         </is>
       </c>
       <c r="B553" s="2" t="inlineStr">
@@ -26503,12 +26499,12 @@
       </c>
       <c r="C553" s="3" t="inlineStr">
         <is>
-          <t>Coordinador de seguridad vial y monitoreo</t>
+          <t>ingeniero civil</t>
         </is>
       </c>
       <c r="D553" s="3" t="inlineStr">
         <is>
-          <t>MEGACOMERCIAL S.A.S</t>
+          <t>EVALTEC S.A.S.</t>
         </is>
       </c>
       <c r="E553" s="8" t="n">
@@ -26520,17 +26516,13 @@
         </is>
       </c>
       <c r="G553" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-coordinador-de-seguridad-vial-y-monitoreo-abierto-a-nivel-nacional-en-bogota-dc-B9B593A780889F2A61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H553" s="6" t="inlineStr">
-        <is>
-          <t>$ 5.000.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingeniero-civil-o-areas-afines-en-medellin-0E02F682AB12631061373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H553" s="6" t="inlineStr"/>
       <c r="I553" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en infraestructura vial y transporte. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J553" s="2" t="inlineStr">
@@ -26543,7 +26535,7 @@
     <row r="554" ht="22" customHeight="1">
       <c r="A554" s="2" t="inlineStr">
         <is>
-          <t>aecc6c18fdd71383</t>
+          <t>af38dd28fbbad8f4</t>
         </is>
       </c>
       <c r="B554" s="2" t="inlineStr">
@@ -26553,12 +26545,12 @@
       </c>
       <c r="C554" s="3" t="inlineStr">
         <is>
-          <t>Coordinador de PESV</t>
+          <t>Tecnólogo Auxiliar Civil</t>
         </is>
       </c>
       <c r="D554" s="3" t="inlineStr">
         <is>
-          <t>Agencia de Empleo de Comfenalco Antioquia</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E554" s="8" t="n">
@@ -26570,17 +26562,13 @@
         </is>
       </c>
       <c r="G554" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-coordinador-de-pesv-en-medellin-67C3B78E9A85885161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H554" s="6" t="inlineStr">
-        <is>
-          <t>$ 2.800.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnologo-auxiliar-civil-antioquia-en-liborina-B380460DDA9F98D061373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H554" s="6" t="inlineStr"/>
       <c r="I554" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en infraestructura vial y transporte. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J554" s="2" t="inlineStr">
@@ -26593,7 +26581,7 @@
     <row r="555" ht="22" customHeight="1">
       <c r="A555" s="2" t="inlineStr">
         <is>
-          <t>1558fc20863bdd35</t>
+          <t>19e74768ce848880</t>
         </is>
       </c>
       <c r="B555" s="2" t="inlineStr">
@@ -26608,7 +26596,7 @@
       </c>
       <c r="D555" s="3" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE INGENIEROS CONSTRUCTORES S.A.S.</t>
+          <t>Agencia de empleo de Comfenalco Cartagena</t>
         </is>
       </c>
       <c r="E555" s="8" t="n">
@@ -26620,10 +26608,14 @@
         </is>
       </c>
       <c r="G555" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-coordinador-hseq-en-barranquilla-F4898EBB71CAF3ED61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H555" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-coordinador-hseq-especialista-en-seguridad-y-salud-en-el-trabajo-salud-ocupacional-en-cartagena-de-indias-1EAF6570FC054C2661373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H555" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.500.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I555" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -26639,7 +26631,7 @@
     <row r="556" ht="22" customHeight="1">
       <c r="A556" s="2" t="inlineStr">
         <is>
-          <t>0bf63022dc93885b</t>
+          <t>38c9a9481706de58</t>
         </is>
       </c>
       <c r="B556" s="2" t="inlineStr">
@@ -26649,12 +26641,12 @@
       </c>
       <c r="C556" s="3" t="inlineStr">
         <is>
-          <t>ingeniero civil</t>
+          <t>Coordinador de seguridad vial y monitoreo</t>
         </is>
       </c>
       <c r="D556" s="3" t="inlineStr">
         <is>
-          <t>FRANCISCO ANGULO M INGENIEROS S.A.S.</t>
+          <t>MEGACOMERCIAL S.A.S</t>
         </is>
       </c>
       <c r="E556" s="8" t="n">
@@ -26666,13 +26658,17 @@
         </is>
       </c>
       <c r="G556" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingeniero-civil-residente-de-interventoria-yo-supervision-tecnica-en-cali-D2AE78FA9B23778161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H556" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-coordinador-de-seguridad-vial-y-monitoreo-abierto-a-nivel-nacional-en-bogota-dc-B9B593A780889F2A61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H556" s="6" t="inlineStr">
+        <is>
+          <t>$ 5.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I556" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en infraestructura vial y transporte. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J556" s="2" t="inlineStr">
@@ -26685,7 +26681,7 @@
     <row r="557" ht="22" customHeight="1">
       <c r="A557" s="2" t="inlineStr">
         <is>
-          <t>baa61a6e15a2de77</t>
+          <t>aecc6c18fdd71383</t>
         </is>
       </c>
       <c r="B557" s="2" t="inlineStr">
@@ -26695,12 +26691,12 @@
       </c>
       <c r="C557" s="3" t="inlineStr">
         <is>
-          <t>Arquitecto(a) / Ingeniero(a) Civil</t>
+          <t>Coordinador de PESV</t>
         </is>
       </c>
       <c r="D557" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>Agencia de Empleo de Comfenalco Antioquia</t>
         </is>
       </c>
       <c r="E557" s="8" t="n">
@@ -26712,13 +26708,17 @@
         </is>
       </c>
       <c r="G557" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-arquitectoa-ingenieroa-civil-en-bucaramanga-8D15AF34F304555F61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H557" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-coordinador-de-pesv-en-medellin-67C3B78E9A85885161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H557" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.800.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I557" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en infraestructura vial y transporte. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J557" s="2" t="inlineStr">
@@ -26731,7 +26731,7 @@
     <row r="558" ht="22" customHeight="1">
       <c r="A558" s="2" t="inlineStr">
         <is>
-          <t>448d93b15d9b7dec</t>
+          <t>1558fc20863bdd35</t>
         </is>
       </c>
       <c r="B558" s="2" t="inlineStr">
@@ -26741,12 +26741,12 @@
       </c>
       <c r="C558" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero especialista fortinet</t>
+          <t>Coordinador HSEQ</t>
         </is>
       </c>
       <c r="D558" s="3" t="inlineStr">
         <is>
-          <t>ATCG DE COLOMBIA S.A.S</t>
+          <t>COMPAÑIA DE INGENIEROS CONSTRUCTORES S.A.S.</t>
         </is>
       </c>
       <c r="E558" s="8" t="n">
@@ -26758,13 +26758,13 @@
         </is>
       </c>
       <c r="G558" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-especialista-fortinet-1886742914", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-coordinador-hseq-en-barranquilla-F4898EBB71CAF3ED61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H558" s="6" t="inlineStr"/>
       <c r="I558" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J558" s="2" t="inlineStr">
@@ -26777,7 +26777,7 @@
     <row r="559" ht="22" customHeight="1">
       <c r="A559" s="2" t="inlineStr">
         <is>
-          <t>f2fc6f9471f81665</t>
+          <t>0bf63022dc93885b</t>
         </is>
       </c>
       <c r="B559" s="2" t="inlineStr">
@@ -26787,12 +26787,12 @@
       </c>
       <c r="C559" s="3" t="inlineStr">
         <is>
-          <t>Coordinador/a nacional de redes e infraestructura de ti - presencial bucaramanga</t>
+          <t>ingeniero civil</t>
         </is>
       </c>
       <c r="D559" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>FRANCISCO ANGULO M INGENIEROS S.A.S.</t>
         </is>
       </c>
       <c r="E559" s="8" t="n">
@@ -26804,13 +26804,13 @@
         </is>
       </c>
       <c r="G559" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-a-nacional-de-redes-e-infraestructura-de-ti-presencial-bucaramanga-1886769481", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingeniero-civil-residente-de-interventoria-yo-supervision-tecnica-en-cali-D2AE78FA9B23778161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H559" s="6" t="inlineStr"/>
       <c r="I559" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en infraestructura vial y transporte. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J559" s="2" t="inlineStr">
@@ -26823,7 +26823,7 @@
     <row r="560" ht="22" customHeight="1">
       <c r="A560" s="2" t="inlineStr">
         <is>
-          <t>53e1a775996a36c5</t>
+          <t>baa61a6e15a2de77</t>
         </is>
       </c>
       <c r="B560" s="2" t="inlineStr">
@@ -26833,12 +26833,12 @@
       </c>
       <c r="C560" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero civil</t>
+          <t>Arquitecto(a) / Ingeniero(a) Civil</t>
         </is>
       </c>
       <c r="D560" s="3" t="inlineStr">
         <is>
-          <t>Proyectos de Diseño y Construccion sas</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E560" s="8" t="n">
@@ -26850,7 +26850,7 @@
         </is>
       </c>
       <c r="G560" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-civil-1886757049", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-arquitectoa-ingenieroa-civil-en-bucaramanga-8D15AF34F304555F61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H560" s="6" t="inlineStr"/>
@@ -26869,7 +26869,7 @@
     <row r="561" ht="22" customHeight="1">
       <c r="A561" s="2" t="inlineStr">
         <is>
-          <t>1072d76e2f18ea50</t>
+          <t>448d93b15d9b7dec</t>
         </is>
       </c>
       <c r="B561" s="2" t="inlineStr">
@@ -26879,12 +26879,12 @@
       </c>
       <c r="C561" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero civil</t>
+          <t>Ingeniero especialista fortinet</t>
         </is>
       </c>
       <c r="D561" s="3" t="inlineStr">
         <is>
-          <t>R2P SOLUCIONES Y CONSTRUCCIONES SAS</t>
+          <t>ATCG DE COLOMBIA S.A.S</t>
         </is>
       </c>
       <c r="E561" s="8" t="n">
@@ -26896,7 +26896,7 @@
         </is>
       </c>
       <c r="G561" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-civil-1886758475", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-especialista-fortinet-1886742914", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H561" s="6" t="inlineStr"/>
@@ -26915,7 +26915,7 @@
     <row r="562" ht="22" customHeight="1">
       <c r="A562" s="2" t="inlineStr">
         <is>
-          <t>2c943591cc334f5a</t>
+          <t>f2fc6f9471f81665</t>
         </is>
       </c>
       <c r="B562" s="2" t="inlineStr">
@@ -26925,7 +26925,7 @@
       </c>
       <c r="C562" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo/ade ingeniera</t>
+          <t>Coordinador/a nacional de redes e infraestructura de ti - presencial bucaramanga</t>
         </is>
       </c>
       <c r="D562" s="3" t="inlineStr">
@@ -26942,13 +26942,13 @@
         </is>
       </c>
       <c r="G562" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ejecutivo-ade-ingeniera-1886752134", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-a-nacional-de-redes-e-infraestructura-de-ti-presencial-bucaramanga-1886769481", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H562" s="6" t="inlineStr"/>
       <c r="I562" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en infraestructura vial y transporte. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J562" s="2" t="inlineStr">
@@ -26961,7 +26961,7 @@
     <row r="563" ht="22" customHeight="1">
       <c r="A563" s="2" t="inlineStr">
         <is>
-          <t>7d4067502e572780</t>
+          <t>53e1a775996a36c5</t>
         </is>
       </c>
       <c r="B563" s="2" t="inlineStr">
@@ -26971,12 +26971,12 @@
       </c>
       <c r="C563" s="3" t="inlineStr">
         <is>
-          <t>Ingeniera de ventas - cali</t>
+          <t>Ingeniero civil</t>
         </is>
       </c>
       <c r="D563" s="3" t="inlineStr">
         <is>
-          <t>PIPOL EXPERT SAS</t>
+          <t>Proyectos de Diseño y Construccion sas</t>
         </is>
       </c>
       <c r="E563" s="8" t="n">
@@ -26988,7 +26988,7 @@
         </is>
       </c>
       <c r="G563" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniera-de-ventas-cali-1886754430", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-civil-1886757049", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H563" s="6" t="inlineStr"/>
@@ -27007,7 +27007,7 @@
     <row r="564" ht="22" customHeight="1">
       <c r="A564" s="2" t="inlineStr">
         <is>
-          <t>a3a688084650de1c</t>
+          <t>1072d76e2f18ea50</t>
         </is>
       </c>
       <c r="B564" s="2" t="inlineStr">
@@ -27017,12 +27017,12 @@
       </c>
       <c r="C564" s="3" t="inlineStr">
         <is>
-          <t>Ingeniera comercial electrica - cali</t>
+          <t>Ingeniero civil</t>
         </is>
       </c>
       <c r="D564" s="3" t="inlineStr">
         <is>
-          <t>PIPOL EXPERT SAS</t>
+          <t>R2P SOLUCIONES Y CONSTRUCCIONES SAS</t>
         </is>
       </c>
       <c r="E564" s="8" t="n">
@@ -27034,7 +27034,7 @@
         </is>
       </c>
       <c r="G564" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniera-comercial-electrica-cali-1886752104", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-civil-1886758475", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H564" s="6" t="inlineStr"/>
@@ -27053,7 +27053,7 @@
     <row r="565" ht="22" customHeight="1">
       <c r="A565" s="2" t="inlineStr">
         <is>
-          <t>359d47915a2e74e6</t>
+          <t>2c943591cc334f5a</t>
         </is>
       </c>
       <c r="B565" s="2" t="inlineStr">
@@ -27063,12 +27063,12 @@
       </c>
       <c r="C565" s="3" t="inlineStr">
         <is>
-          <t>Supervisor civil - obra</t>
+          <t>Ejecutivo/ade ingeniera</t>
         </is>
       </c>
       <c r="D565" s="3" t="inlineStr">
         <is>
-          <t>CONCONCRETO S.A.</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E565" s="8" t="n">
@@ -27080,7 +27080,7 @@
         </is>
       </c>
       <c r="G565" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/supervisor-civil-obra-1886750435", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ejecutivo-ade-ingeniera-1886752134", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H565" s="6" t="inlineStr"/>
@@ -27099,7 +27099,7 @@
     <row r="566" ht="22" customHeight="1">
       <c r="A566" s="2" t="inlineStr">
         <is>
-          <t>78244d2897084f6a</t>
+          <t>7d4067502e572780</t>
         </is>
       </c>
       <c r="B566" s="2" t="inlineStr">
@@ -27109,7 +27109,7 @@
       </c>
       <c r="C566" s="3" t="inlineStr">
         <is>
-          <t>Ingeniera comercial sector industrial - cali</t>
+          <t>Ingeniera de ventas - cali</t>
         </is>
       </c>
       <c r="D566" s="3" t="inlineStr">
@@ -27126,7 +27126,7 @@
         </is>
       </c>
       <c r="G566" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniera-comercial-sector-industrial-cali-1886753949", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniera-de-ventas-cali-1886754430", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H566" s="6" t="inlineStr"/>
@@ -27145,7 +27145,7 @@
     <row r="567" ht="22" customHeight="1">
       <c r="A567" s="2" t="inlineStr">
         <is>
-          <t>a4d1239b8910f7cf</t>
+          <t>a3a688084650de1c</t>
         </is>
       </c>
       <c r="B567" s="2" t="inlineStr">
@@ -27155,7 +27155,7 @@
       </c>
       <c r="C567" s="3" t="inlineStr">
         <is>
-          <t>Ingeniera electrica comercial - bogotá</t>
+          <t>Ingeniera comercial electrica - cali</t>
         </is>
       </c>
       <c r="D567" s="3" t="inlineStr">
@@ -27172,7 +27172,7 @@
         </is>
       </c>
       <c r="G567" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniera-electrica-comercial-bogota-1886756984", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniera-comercial-electrica-cali-1886752104", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H567" s="6" t="inlineStr"/>
@@ -27191,7 +27191,7 @@
     <row r="568" ht="22" customHeight="1">
       <c r="A568" s="2" t="inlineStr">
         <is>
-          <t>366f049dd1eaf173</t>
+          <t>359d47915a2e74e6</t>
         </is>
       </c>
       <c r="B568" s="2" t="inlineStr">
@@ -27201,12 +27201,12 @@
       </c>
       <c r="C568" s="3" t="inlineStr">
         <is>
-          <t>Civil engineering-in-training</t>
+          <t>Supervisor civil - obra</t>
         </is>
       </c>
       <c r="D568" s="3" t="inlineStr">
         <is>
-          <t>WSP COLOMBIA SAS</t>
+          <t>CONCONCRETO S.A.</t>
         </is>
       </c>
       <c r="E568" s="8" t="n">
@@ -27218,7 +27218,7 @@
         </is>
       </c>
       <c r="G568" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/civil-engineeringintraining-1886759044", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/supervisor-civil-obra-1886750435", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H568" s="6" t="inlineStr"/>
@@ -27237,7 +27237,7 @@
     <row r="569" ht="22" customHeight="1">
       <c r="A569" s="2" t="inlineStr">
         <is>
-          <t>555a755e56fc6a80</t>
+          <t>78244d2897084f6a</t>
         </is>
       </c>
       <c r="B569" s="2" t="inlineStr">
@@ -27247,12 +27247,12 @@
       </c>
       <c r="C569" s="3" t="inlineStr">
         <is>
-          <t>Civil engineering-in-training</t>
+          <t>Ingeniera comercial sector industrial - cali</t>
         </is>
       </c>
       <c r="D569" s="3" t="inlineStr">
         <is>
-          <t>WSP COLOMBIA SAS</t>
+          <t>PIPOL EXPERT SAS</t>
         </is>
       </c>
       <c r="E569" s="8" t="n">
@@ -27264,7 +27264,7 @@
         </is>
       </c>
       <c r="G569" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/civil-engineeringintraining-1886758755", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniera-comercial-sector-industrial-cali-1886753949", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H569" s="6" t="inlineStr"/>
@@ -27283,7 +27283,7 @@
     <row r="570" ht="22" customHeight="1">
       <c r="A570" s="2" t="inlineStr">
         <is>
-          <t>776483d4ec602e40</t>
+          <t>a4d1239b8910f7cf</t>
         </is>
       </c>
       <c r="B570" s="2" t="inlineStr">
@@ -27293,12 +27293,12 @@
       </c>
       <c r="C570" s="3" t="inlineStr">
         <is>
-          <t>Consultor senior sap pm - remoto colombia</t>
+          <t>Ingeniera electrica comercial - bogotá</t>
         </is>
       </c>
       <c r="D570" s="3" t="inlineStr">
         <is>
-          <t>TALYCAP GLOBAL SAS</t>
+          <t>PIPOL EXPERT SAS</t>
         </is>
       </c>
       <c r="E570" s="8" t="n">
@@ -27310,7 +27310,7 @@
         </is>
       </c>
       <c r="G570" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-senior-sap-pm-remoto-colombia-1886747903", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniera-electrica-comercial-bogota-1886756984", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H570" s="6" t="inlineStr"/>
@@ -27329,7 +27329,7 @@
     <row r="571" ht="22" customHeight="1">
       <c r="A571" s="2" t="inlineStr">
         <is>
-          <t>b1cfe269bbc00011</t>
+          <t>366f049dd1eaf173</t>
         </is>
       </c>
       <c r="B571" s="2" t="inlineStr">
@@ -27339,12 +27339,12 @@
       </c>
       <c r="C571" s="3" t="inlineStr">
         <is>
-          <t>Coordinador de interventoría</t>
+          <t>Civil engineering-in-training</t>
         </is>
       </c>
       <c r="D571" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>WSP COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E571" s="8" t="n">
@@ -27356,7 +27356,7 @@
         </is>
       </c>
       <c r="G571" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-de-interventoria-1886751671", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/civil-engineeringintraining-1886759044", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H571" s="6" t="inlineStr"/>
@@ -27375,7 +27375,7 @@
     <row r="572" ht="22" customHeight="1">
       <c r="A572" s="2" t="inlineStr">
         <is>
-          <t>b7a3423e1ee1e624</t>
+          <t>555a755e56fc6a80</t>
         </is>
       </c>
       <c r="B572" s="2" t="inlineStr">
@@ -27385,12 +27385,12 @@
       </c>
       <c r="C572" s="3" t="inlineStr">
         <is>
-          <t>Especialista en urbanismo - proyecto vial</t>
+          <t>Civil engineering-in-training</t>
         </is>
       </c>
       <c r="D572" s="3" t="inlineStr">
         <is>
-          <t>INGEPLAN.CO SAS EMPRESA DE BENEFICIO E INTERES COLECTIVO BIC</t>
+          <t>WSP COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E572" s="8" t="n">
@@ -27402,7 +27402,7 @@
         </is>
       </c>
       <c r="G572" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-urbanismo-proyecto-vial-1886755827", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/civil-engineeringintraining-1886758755", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H572" s="6" t="inlineStr"/>
@@ -27421,7 +27421,7 @@
     <row r="573" ht="22" customHeight="1">
       <c r="A573" s="2" t="inlineStr">
         <is>
-          <t>fcb39d755657052e</t>
+          <t>776483d4ec602e40</t>
         </is>
       </c>
       <c r="B573" s="2" t="inlineStr">
@@ -27431,12 +27431,12 @@
       </c>
       <c r="C573" s="3" t="inlineStr">
         <is>
-          <t>Coordinador hseq</t>
+          <t>Consultor senior sap pm - remoto colombia</t>
         </is>
       </c>
       <c r="D573" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>TALYCAP GLOBAL SAS</t>
         </is>
       </c>
       <c r="E573" s="8" t="n">
@@ -27448,13 +27448,13 @@
         </is>
       </c>
       <c r="G573" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-hseq-1886747304", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-senior-sap-pm-remoto-colombia-1886747903", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H573" s="6" t="inlineStr"/>
       <c r="I573" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J573" s="2" t="inlineStr">
@@ -27467,7 +27467,7 @@
     <row r="574" ht="22" customHeight="1">
       <c r="A574" s="2" t="inlineStr">
         <is>
-          <t>9e2f0c16f1a50983</t>
+          <t>b1cfe269bbc00011</t>
         </is>
       </c>
       <c r="B574" s="2" t="inlineStr">
@@ -27477,7 +27477,7 @@
       </c>
       <c r="C574" s="3" t="inlineStr">
         <is>
-          <t>Coordinador hseq</t>
+          <t>Coordinador de interventoría</t>
         </is>
       </c>
       <c r="D574" s="3" t="inlineStr">
@@ -27494,13 +27494,13 @@
         </is>
       </c>
       <c r="G574" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-hseq-1886764155", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-de-interventoria-1886751671", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H574" s="6" t="inlineStr"/>
       <c r="I574" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J574" s="2" t="inlineStr">
@@ -27513,7 +27513,7 @@
     <row r="575" ht="22" customHeight="1">
       <c r="A575" s="2" t="inlineStr">
         <is>
-          <t>9d4d87a631d5e8b8</t>
+          <t>b7a3423e1ee1e624</t>
         </is>
       </c>
       <c r="B575" s="2" t="inlineStr">
@@ -27523,12 +27523,12 @@
       </c>
       <c r="C575" s="3" t="inlineStr">
         <is>
-          <t>Coordinador hseq</t>
+          <t>Especialista en urbanismo - proyecto vial</t>
         </is>
       </c>
       <c r="D575" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>INGEPLAN.CO SAS EMPRESA DE BENEFICIO E INTERES COLECTIVO BIC</t>
         </is>
       </c>
       <c r="E575" s="8" t="n">
@@ -27540,13 +27540,13 @@
         </is>
       </c>
       <c r="G575" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-hseq-1886760733", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-urbanismo-proyecto-vial-1886755827", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H575" s="6" t="inlineStr"/>
       <c r="I575" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J575" s="2" t="inlineStr">
@@ -27559,7 +27559,7 @@
     <row r="576" ht="22" customHeight="1">
       <c r="A576" s="2" t="inlineStr">
         <is>
-          <t>62d6690ef260f268</t>
+          <t>fcb39d755657052e</t>
         </is>
       </c>
       <c r="B576" s="2" t="inlineStr">
@@ -27569,12 +27569,12 @@
       </c>
       <c r="C576" s="3" t="inlineStr">
         <is>
-          <t>Coordinador hseq cartagena</t>
+          <t>Coordinador hseq</t>
         </is>
       </c>
       <c r="D576" s="3" t="inlineStr">
         <is>
-          <t>APPLUS NORCONTROL COLOMBIA LTDA</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E576" s="8" t="n">
@@ -27586,7 +27586,7 @@
         </is>
       </c>
       <c r="G576" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-hseq-cartagena-1886754661", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-hseq-1886747304", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H576" s="6" t="inlineStr"/>
@@ -27605,7 +27605,7 @@
     <row r="577" ht="22" customHeight="1">
       <c r="A577" s="2" t="inlineStr">
         <is>
-          <t>6e57e2acbfc11d12</t>
+          <t>9e2f0c16f1a50983</t>
         </is>
       </c>
       <c r="B577" s="2" t="inlineStr">
@@ -27615,7 +27615,7 @@
       </c>
       <c r="C577" s="3" t="inlineStr">
         <is>
-          <t>Especialista sig</t>
+          <t>Coordinador hseq</t>
         </is>
       </c>
       <c r="D577" s="3" t="inlineStr">
@@ -27632,13 +27632,13 @@
         </is>
       </c>
       <c r="G577" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-sig-1886757094", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-hseq-1886764155", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H577" s="6" t="inlineStr"/>
       <c r="I577" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J577" s="2" t="inlineStr">
@@ -27651,7 +27651,7 @@
     <row r="578" ht="22" customHeight="1">
       <c r="A578" s="2" t="inlineStr">
         <is>
-          <t>11494a184e6f9290</t>
+          <t>9d4d87a631d5e8b8</t>
         </is>
       </c>
       <c r="B578" s="2" t="inlineStr">
@@ -27661,7 +27661,7 @@
       </c>
       <c r="C578" s="3" t="inlineStr">
         <is>
-          <t>Especialista en ingeniería civil - coordinador técnico</t>
+          <t>Coordinador hseq</t>
         </is>
       </c>
       <c r="D578" s="3" t="inlineStr">
@@ -27678,13 +27678,13 @@
         </is>
       </c>
       <c r="G578" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-ingenieria-civil-coordinador-tecnico-honduras-1886745304", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-hseq-1886760733", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H578" s="6" t="inlineStr"/>
       <c r="I578" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J578" s="2" t="inlineStr">
@@ -27697,7 +27697,7 @@
     <row r="579" ht="22" customHeight="1">
       <c r="A579" s="2" t="inlineStr">
         <is>
-          <t>327c6d2b54619849</t>
+          <t>62d6690ef260f268</t>
         </is>
       </c>
       <c r="B579" s="2" t="inlineStr">
@@ -27707,12 +27707,12 @@
       </c>
       <c r="C579" s="3" t="inlineStr">
         <is>
-          <t>Especialista en psiquiatría</t>
+          <t>Coordinador hseq cartagena</t>
         </is>
       </c>
       <c r="D579" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>APPLUS NORCONTROL COLOMBIA LTDA</t>
         </is>
       </c>
       <c r="E579" s="8" t="n">
@@ -27724,13 +27724,13 @@
         </is>
       </c>
       <c r="G579" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-psiquiatria-1886757353", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-hseq-cartagena-1886754661", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H579" s="6" t="inlineStr"/>
       <c r="I579" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J579" s="2" t="inlineStr">
@@ -27743,7 +27743,7 @@
     <row r="580" ht="22" customHeight="1">
       <c r="A580" s="2" t="inlineStr">
         <is>
-          <t>b637f33f588eb5ae</t>
+          <t>6e57e2acbfc11d12</t>
         </is>
       </c>
       <c r="B580" s="2" t="inlineStr">
@@ -27753,7 +27753,7 @@
       </c>
       <c r="C580" s="3" t="inlineStr">
         <is>
-          <t>Especialista en diseño hospitalario</t>
+          <t>Especialista sig</t>
         </is>
       </c>
       <c r="D580" s="3" t="inlineStr">
@@ -27770,7 +27770,7 @@
         </is>
       </c>
       <c r="G580" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-diseno-hospitalario-disponibilidad-viajar-a-peru-1886747220", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-sig-1886757094", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H580" s="6" t="inlineStr"/>
@@ -27789,7 +27789,7 @@
     <row r="581" ht="22" customHeight="1">
       <c r="A581" s="2" t="inlineStr">
         <is>
-          <t>adcc2b47284b5d4d</t>
+          <t>11494a184e6f9290</t>
         </is>
       </c>
       <c r="B581" s="2" t="inlineStr">
@@ -27799,12 +27799,12 @@
       </c>
       <c r="C581" s="3" t="inlineStr">
         <is>
-          <t>Analista de diseño e ingeniería de empaque - sector farmaceutico</t>
+          <t>Especialista en ingeniería civil - coordinador técnico</t>
         </is>
       </c>
       <c r="D581" s="3" t="inlineStr">
         <is>
-          <t>LABORATORIOS BUSSIE</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E581" s="8" t="n">
@@ -27816,7 +27816,7 @@
         </is>
       </c>
       <c r="G581" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-diseno-e-ingenieria-de-empaque-sector-farmaceutico-1886755492", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-ingenieria-civil-coordinador-tecnico-honduras-1886745304", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H581" s="6" t="inlineStr"/>
@@ -27835,7 +27835,7 @@
     <row r="582" ht="22" customHeight="1">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>3ec3d2d34753ff04</t>
+          <t>327c6d2b54619849</t>
         </is>
       </c>
       <c r="B582" s="2" t="inlineStr">
@@ -27845,12 +27845,12 @@
       </c>
       <c r="C582" s="3" t="inlineStr">
         <is>
-          <t>Especialista de diseño y arquitectura</t>
+          <t>Especialista en psiquiatría</t>
         </is>
       </c>
       <c r="D582" s="3" t="inlineStr">
         <is>
-          <t>INTER RAPIDISIMO</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E582" s="8" t="n">
@@ -27862,7 +27862,7 @@
         </is>
       </c>
       <c r="G582" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-de-diseno-y-arquitectura-1886761909", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-psiquiatria-1886757353", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H582" s="6" t="inlineStr"/>
@@ -27881,7 +27881,7 @@
     <row r="583" ht="22" customHeight="1">
       <c r="A583" s="2" t="inlineStr">
         <is>
-          <t>4e917305e90b3efa</t>
+          <t>b637f33f588eb5ae</t>
         </is>
       </c>
       <c r="B583" s="2" t="inlineStr">
@@ -27891,12 +27891,12 @@
       </c>
       <c r="C583" s="3" t="inlineStr">
         <is>
-          <t>Especialista en geología</t>
+          <t>Especialista en diseño hospitalario</t>
         </is>
       </c>
       <c r="D583" s="3" t="inlineStr">
         <is>
-          <t>INGEPLAN.CO SAS EMPRESA DE BENEFICIO E INTERES COLECTIVO BIC</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E583" s="8" t="n">
@@ -27908,7 +27908,7 @@
         </is>
       </c>
       <c r="G583" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-geologia-1886761263", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-diseno-hospitalario-disponibilidad-viajar-a-peru-1886747220", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H583" s="6" t="inlineStr"/>
@@ -27927,7 +27927,7 @@
     <row r="584" ht="22" customHeight="1">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>1aef5476d70bbe42</t>
+          <t>adcc2b47284b5d4d</t>
         </is>
       </c>
       <c r="B584" s="2" t="inlineStr">
@@ -27937,12 +27937,12 @@
       </c>
       <c r="C584" s="3" t="inlineStr">
         <is>
-          <t>Especialista en geología</t>
+          <t>Analista de diseño e ingeniería de empaque - sector farmaceutico</t>
         </is>
       </c>
       <c r="D584" s="3" t="inlineStr">
         <is>
-          <t>INGEPLAN.CO SAS EMPRESA DE BENEFICIO E INTERES COLECTIVO BIC</t>
+          <t>LABORATORIOS BUSSIE</t>
         </is>
       </c>
       <c r="E584" s="8" t="n">
@@ -27954,7 +27954,7 @@
         </is>
       </c>
       <c r="G584" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-geologia-1886755729", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-diseno-e-ingenieria-de-empaque-sector-farmaceutico-1886755492", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H584" s="6" t="inlineStr"/>
@@ -27973,7 +27973,7 @@
     <row r="585" ht="22" customHeight="1">
       <c r="A585" s="2" t="inlineStr">
         <is>
-          <t>b46df3b678599255</t>
+          <t>3ec3d2d34753ff04</t>
         </is>
       </c>
       <c r="B585" s="2" t="inlineStr">
@@ -27983,12 +27983,12 @@
       </c>
       <c r="C585" s="3" t="inlineStr">
         <is>
-          <t>Especialista en estructuras</t>
+          <t>Especialista de diseño y arquitectura</t>
         </is>
       </c>
       <c r="D585" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>INTER RAPIDISIMO</t>
         </is>
       </c>
       <c r="E585" s="8" t="n">
@@ -28000,7 +28000,7 @@
         </is>
       </c>
       <c r="G585" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-estructuras-1886757080", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-de-diseno-y-arquitectura-1886761909", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H585" s="6" t="inlineStr"/>
@@ -28019,7 +28019,7 @@
     <row r="586" ht="22" customHeight="1">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>935035bdfa2ae0b7</t>
+          <t>4e917305e90b3efa</t>
         </is>
       </c>
       <c r="B586" s="2" t="inlineStr">
@@ -28029,7 +28029,7 @@
       </c>
       <c r="C586" s="3" t="inlineStr">
         <is>
-          <t>Especialista en gestión del riesgo</t>
+          <t>Especialista en geología</t>
         </is>
       </c>
       <c r="D586" s="3" t="inlineStr">
@@ -28046,7 +28046,7 @@
         </is>
       </c>
       <c r="G586" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-gestion-del-riesgo-1886755709", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-geologia-1886761263", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H586" s="6" t="inlineStr"/>
@@ -28065,7 +28065,7 @@
     <row r="587" ht="22" customHeight="1">
       <c r="A587" s="2" t="inlineStr">
         <is>
-          <t>14a1c964238340ba</t>
+          <t>1aef5476d70bbe42</t>
         </is>
       </c>
       <c r="B587" s="2" t="inlineStr">
@@ -28075,12 +28075,12 @@
       </c>
       <c r="C587" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero civil nivel v</t>
+          <t>Especialista en geología</t>
         </is>
       </c>
       <c r="D587" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>INGEPLAN.CO SAS EMPRESA DE BENEFICIO E INTERES COLECTIVO BIC</t>
         </is>
       </c>
       <c r="E587" s="8" t="n">
@@ -28092,7 +28092,7 @@
         </is>
       </c>
       <c r="G587" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-civil-nivel-v-1886758046", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-geologia-1886755729", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H587" s="6" t="inlineStr"/>
@@ -28111,7 +28111,7 @@
     <row r="588" ht="22" customHeight="1">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>740f61bdbaa69d0e</t>
+          <t>b46df3b678599255</t>
         </is>
       </c>
       <c r="B588" s="2" t="inlineStr">
@@ -28121,12 +28121,12 @@
       </c>
       <c r="C588" s="3" t="inlineStr">
         <is>
-          <t>Coordinador de proyectos bilingüe</t>
+          <t>Especialista en estructuras</t>
         </is>
       </c>
       <c r="D588" s="3" t="inlineStr">
         <is>
-          <t>EyS IT SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E588" s="8" t="n">
@@ -28138,7 +28138,7 @@
         </is>
       </c>
       <c r="G588" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-de-proyectos-bilingue-1886749343", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-estructuras-1886757080", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H588" s="6" t="inlineStr"/>
@@ -28157,7 +28157,7 @@
     <row r="589" ht="22" customHeight="1">
       <c r="A589" s="2" t="inlineStr">
         <is>
-          <t>63ef229552018ccd</t>
+          <t>935035bdfa2ae0b7</t>
         </is>
       </c>
       <c r="B589" s="2" t="inlineStr">
@@ -28167,12 +28167,12 @@
       </c>
       <c r="C589" s="3" t="inlineStr">
         <is>
-          <t>Coordinador de proyectos</t>
+          <t>Especialista en gestión del riesgo</t>
         </is>
       </c>
       <c r="D589" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>INGEPLAN.CO SAS EMPRESA DE BENEFICIO E INTERES COLECTIVO BIC</t>
         </is>
       </c>
       <c r="E589" s="8" t="n">
@@ -28184,7 +28184,7 @@
         </is>
       </c>
       <c r="G589" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-de-proyectos-1886748647", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-gestion-del-riesgo-1886755709", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H589" s="6" t="inlineStr"/>
@@ -28203,7 +28203,7 @@
     <row r="590" ht="22" customHeight="1">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>03750e25a7e1c016</t>
+          <t>14a1c964238340ba</t>
         </is>
       </c>
       <c r="B590" s="2" t="inlineStr">
@@ -28213,12 +28213,12 @@
       </c>
       <c r="C590" s="3" t="inlineStr">
         <is>
-          <t>Coordinador de proyectos inmobiliarios</t>
+          <t>Ingeniero civil nivel v</t>
         </is>
       </c>
       <c r="D590" s="3" t="inlineStr">
         <is>
-          <t>GRUPO AR S.A.</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E590" s="8" t="n">
@@ -28230,7 +28230,7 @@
         </is>
       </c>
       <c r="G590" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-de-proyectos-inmobiliarios-1886745877", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-civil-nivel-v-1886758046", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H590" s="6" t="inlineStr"/>
@@ -28249,7 +28249,7 @@
     <row r="591" ht="22" customHeight="1">
       <c r="A591" s="2" t="inlineStr">
         <is>
-          <t>5627e52731a73f27</t>
+          <t>740f61bdbaa69d0e</t>
         </is>
       </c>
       <c r="B591" s="2" t="inlineStr">
@@ -28259,12 +28259,12 @@
       </c>
       <c r="C591" s="3" t="inlineStr">
         <is>
-          <t>Coordinador de proyectos inmobiliarios</t>
+          <t>Coordinador de proyectos bilingüe</t>
         </is>
       </c>
       <c r="D591" s="3" t="inlineStr">
         <is>
-          <t>GRUPO AR S.A.</t>
+          <t>EyS IT SAS</t>
         </is>
       </c>
       <c r="E591" s="8" t="n">
@@ -28276,7 +28276,7 @@
         </is>
       </c>
       <c r="G591" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-de-proyectos-inmobiliarios-1886704948", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-de-proyectos-bilingue-1886749343", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H591" s="6" t="inlineStr"/>
@@ -28295,7 +28295,7 @@
     <row r="592" ht="22" customHeight="1">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>b6af0024900baff6</t>
+          <t>63ef229552018ccd</t>
         </is>
       </c>
       <c r="B592" s="2" t="inlineStr">
@@ -28305,12 +28305,12 @@
       </c>
       <c r="C592" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero residente - ingeniero civil-cordoba</t>
+          <t>Coordinador de proyectos</t>
         </is>
       </c>
       <c r="D592" s="3" t="inlineStr">
         <is>
-          <t>OBCIPOL SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E592" s="8" t="n">
@@ -28322,7 +28322,7 @@
         </is>
       </c>
       <c r="G592" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-residente-ingeniero-civilcordoba-1886763488", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-de-proyectos-1886748647", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H592" s="6" t="inlineStr"/>
@@ -28341,7 +28341,7 @@
     <row r="593" ht="22" customHeight="1">
       <c r="A593" s="2" t="inlineStr">
         <is>
-          <t>2a0453695fa88728</t>
+          <t>03750e25a7e1c016</t>
         </is>
       </c>
       <c r="B593" s="2" t="inlineStr">
@@ -28351,12 +28351,12 @@
       </c>
       <c r="C593" s="3" t="inlineStr">
         <is>
-          <t>Profesional ingenieria mecanica</t>
+          <t>Coordinador de proyectos inmobiliarios</t>
         </is>
       </c>
       <c r="D593" s="3" t="inlineStr">
         <is>
-          <t>INZIGNIA CONSTRUCTION S.A</t>
+          <t>GRUPO AR S.A.</t>
         </is>
       </c>
       <c r="E593" s="8" t="n">
@@ -28368,7 +28368,7 @@
         </is>
       </c>
       <c r="G593" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/profesional-ingenieria-mecanica-1886767282", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-de-proyectos-inmobiliarios-1886745877", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H593" s="6" t="inlineStr"/>
@@ -28387,7 +28387,7 @@
     <row r="594" ht="22" customHeight="1">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>edfe98c543194667</t>
+          <t>5627e52731a73f27</t>
         </is>
       </c>
       <c r="B594" s="2" t="inlineStr">
@@ -28397,12 +28397,12 @@
       </c>
       <c r="C594" s="3" t="inlineStr">
         <is>
-          <t>Jefe de sst - nemocón - 1625991634-135</t>
+          <t>Coordinador de proyectos inmobiliarios</t>
         </is>
       </c>
       <c r="D594" s="3" t="inlineStr">
         <is>
-          <t>AGENCIA DE EMPLEO Y FOMENTO EMPRESARIAL COMPENSAR</t>
+          <t>GRUPO AR S.A.</t>
         </is>
       </c>
       <c r="E594" s="8" t="n">
@@ -28414,13 +28414,13 @@
         </is>
       </c>
       <c r="G594" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/jefe-de-sst-nemocon-1625991634135-1886754873", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-de-proyectos-inmobiliarios-1886704948", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H594" s="6" t="inlineStr"/>
       <c r="I594" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J594" s="2" t="inlineStr">
@@ -28433,7 +28433,7 @@
     <row r="595" ht="22" customHeight="1">
       <c r="A595" s="2" t="inlineStr">
         <is>
-          <t>6233e93ceb1dbeed</t>
+          <t>b6af0024900baff6</t>
         </is>
       </c>
       <c r="B595" s="2" t="inlineStr">
@@ -28443,12 +28443,12 @@
       </c>
       <c r="C595" s="3" t="inlineStr">
         <is>
-          <t>Jefe de sst- nemocón</t>
+          <t>Ingeniero residente - ingeniero civil-cordoba</t>
         </is>
       </c>
       <c r="D595" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>OBCIPOL SAS</t>
         </is>
       </c>
       <c r="E595" s="8" t="n">
@@ -28460,13 +28460,13 @@
         </is>
       </c>
       <c r="G595" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/jefe-de-sst-nemocon-1886757757", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-residente-ingeniero-civilcordoba-1886763488", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J595" s="2" t="inlineStr">
@@ -28479,7 +28479,7 @@
     <row r="596" ht="22" customHeight="1">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>ce75aab7a32f36a3</t>
+          <t>2a0453695fa88728</t>
         </is>
       </c>
       <c r="B596" s="2" t="inlineStr">
@@ -28489,12 +28489,12 @@
       </c>
       <c r="C596" s="3" t="inlineStr">
         <is>
-          <t>Coordinador talento humano y sst - bogota- 1626427532-7</t>
+          <t>Profesional ingenieria mecanica</t>
         </is>
       </c>
       <c r="D596" s="3" t="inlineStr">
         <is>
-          <t>AGENCIA DE EMPLEO Y FOMENTO EMPRESARIAL COMPENSAR</t>
+          <t>INZIGNIA CONSTRUCTION S.A</t>
         </is>
       </c>
       <c r="E596" s="8" t="n">
@@ -28506,13 +28506,13 @@
         </is>
       </c>
       <c r="G596" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-talento-humano-y-sst-bogota-16264275327-1886753531", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/profesional-ingenieria-mecanica-1886767282", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H596" s="6" t="inlineStr"/>
       <c r="I596" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J596" s="2" t="inlineStr">
@@ -28525,7 +28525,7 @@
     <row r="597" ht="22" customHeight="1">
       <c r="A597" s="2" t="inlineStr">
         <is>
-          <t>850731f7bb6cd73f</t>
+          <t>edfe98c543194667</t>
         </is>
       </c>
       <c r="B597" s="2" t="inlineStr">
@@ -28535,12 +28535,12 @@
       </c>
       <c r="C597" s="3" t="inlineStr">
         <is>
-          <t>Coordinador(a) de sst y medio ambiente</t>
+          <t>Jefe de sst - nemocón - 1625991634-135</t>
         </is>
       </c>
       <c r="D597" s="3" t="inlineStr">
         <is>
-          <t>ATIEMPO S.A.S</t>
+          <t>AGENCIA DE EMPLEO Y FOMENTO EMPRESARIAL COMPENSAR</t>
         </is>
       </c>
       <c r="E597" s="8" t="n">
@@ -28552,7 +28552,7 @@
         </is>
       </c>
       <c r="G597" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinadora-de-sst-y-medio-ambiente-1886759848", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/jefe-de-sst-nemocon-1625991634135-1886754873", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H597" s="6" t="inlineStr"/>
@@ -28571,7 +28571,7 @@
     <row r="598" ht="22" customHeight="1">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>abaf8e513787b3f3</t>
+          <t>6233e93ceb1dbeed</t>
         </is>
       </c>
       <c r="B598" s="2" t="inlineStr">
@@ -28581,7 +28581,7 @@
       </c>
       <c r="C598" s="3" t="inlineStr">
         <is>
-          <t>Coordinador pesv</t>
+          <t>Jefe de sst- nemocón</t>
         </is>
       </c>
       <c r="D598" s="3" t="inlineStr">
@@ -28598,13 +28598,13 @@
         </is>
       </c>
       <c r="G598" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-pesv-1886769643", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/jefe-de-sst-nemocon-1886757757", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H598" s="6" t="inlineStr"/>
       <c r="I598" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en infraestructura vial y transporte. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J598" s="2" t="inlineStr">
@@ -28617,7 +28617,7 @@
     <row r="599" ht="22" customHeight="1">
       <c r="A599" s="2" t="inlineStr">
         <is>
-          <t>9dcdf501e5912b88</t>
+          <t>ce75aab7a32f36a3</t>
         </is>
       </c>
       <c r="B599" s="2" t="inlineStr">
@@ -28627,7 +28627,7 @@
       </c>
       <c r="C599" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de obras civiles /girardot ref. 339166-82241</t>
+          <t>Coordinador talento humano y sst - bogota- 1626427532-7</t>
         </is>
       </c>
       <c r="D599" s="3" t="inlineStr">
@@ -28644,13 +28644,13 @@
         </is>
       </c>
       <c r="G599" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-obras-civiles-girardot-ref-33916682241-1886747302", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-talento-humano-y-sst-bogota-16264275327-1886753531", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H599" s="6" t="inlineStr"/>
       <c r="I599" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J599" s="2" t="inlineStr">
@@ -28663,7 +28663,7 @@
     <row r="600" ht="22" customHeight="1">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>693b8a076a888f67</t>
+          <t>850731f7bb6cd73f</t>
         </is>
       </c>
       <c r="B600" s="2" t="inlineStr">
@@ -28673,12 +28673,12 @@
       </c>
       <c r="C600" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero civil - especializacion en estructuras</t>
+          <t>Coordinador(a) de sst y medio ambiente</t>
         </is>
       </c>
       <c r="D600" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>ATIEMPO S.A.S</t>
         </is>
       </c>
       <c r="E600" s="8" t="n">
@@ -28690,13 +28690,13 @@
         </is>
       </c>
       <c r="G600" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-civil-especializacion-en-estructuras-1886766956", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinadora-de-sst-y-medio-ambiente-1886759848", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H600" s="6" t="inlineStr"/>
       <c r="I600" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J600" s="2" t="inlineStr">
@@ -28709,7 +28709,7 @@
     <row r="601" ht="22" customHeight="1">
       <c r="A601" s="2" t="inlineStr">
         <is>
-          <t>13bc527565632878</t>
+          <t>abaf8e513787b3f3</t>
         </is>
       </c>
       <c r="B601" s="2" t="inlineStr">
@@ -28719,7 +28719,7 @@
       </c>
       <c r="C601" s="3" t="inlineStr">
         <is>
-          <t>Tecnico en contratacion de obra civil bogota</t>
+          <t>Coordinador pesv</t>
         </is>
       </c>
       <c r="D601" s="3" t="inlineStr">
@@ -28736,13 +28736,13 @@
         </is>
       </c>
       <c r="G601" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-en-contratacion-de-obra-civil-bogota-1886759693", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-pesv-1886769643", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H601" s="6" t="inlineStr"/>
       <c r="I601" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en infraestructura vial y transporte. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J601" s="2" t="inlineStr">
@@ -28755,7 +28755,7 @@
     <row r="602" ht="22" customHeight="1">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>6ccccd3a1ba05f7f</t>
+          <t>9dcdf501e5912b88</t>
         </is>
       </c>
       <c r="B602" s="2" t="inlineStr">
@@ -28765,12 +28765,12 @@
       </c>
       <c r="C602" s="3" t="inlineStr">
         <is>
-          <t>14561-especialista interventoria-bogota</t>
+          <t>Tecnico de obras civiles /girardot ref. 339166-82241</t>
         </is>
       </c>
       <c r="D602" s="3" t="inlineStr">
         <is>
-          <t>APPLUS NORCONTROL COLOMBIA LTDA</t>
+          <t>AGENCIA DE EMPLEO Y FOMENTO EMPRESARIAL COMPENSAR</t>
         </is>
       </c>
       <c r="E602" s="8" t="n">
@@ -28782,7 +28782,7 @@
         </is>
       </c>
       <c r="G602" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/14561especialista-interventoriabogota-1886768886", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-obras-civiles-girardot-ref-33916682241-1886747302", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H602" s="6" t="inlineStr"/>
@@ -28801,7 +28801,7 @@
     <row r="603" ht="22" customHeight="1">
       <c r="A603" s="2" t="inlineStr">
         <is>
-          <t>8ad0c11c4f07472e</t>
+          <t>693b8a076a888f67</t>
         </is>
       </c>
       <c r="B603" s="2" t="inlineStr">
@@ -28811,12 +28811,12 @@
       </c>
       <c r="C603" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero Civil / Terracerías</t>
+          <t>Ingeniero civil - especializacion en estructuras</t>
         </is>
       </c>
       <c r="D603" s="3" t="inlineStr">
         <is>
-          <t>EOSOL</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E603" s="8" t="n">
@@ -28828,7 +28828,7 @@
         </is>
       </c>
       <c r="G603" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-civil-terracer%C3%ADas-at-eosol-4445793534", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-civil-especializacion-en-estructuras-1886766956", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H603" s="6" t="inlineStr"/>
@@ -28847,7 +28847,7 @@
     <row r="604" ht="22" customHeight="1">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>ed46085f88d06bf5</t>
+          <t>13bc527565632878</t>
         </is>
       </c>
       <c r="B604" s="2" t="inlineStr">
@@ -28857,12 +28857,12 @@
       </c>
       <c r="C604" s="3" t="inlineStr">
         <is>
-          <t>Supervisor Civil</t>
+          <t>Tecnico en contratacion de obra civil bogota</t>
         </is>
       </c>
       <c r="D604" s="3" t="inlineStr">
         <is>
-          <t>EOSOL</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E604" s="8" t="n">
@@ -28874,7 +28874,7 @@
         </is>
       </c>
       <c r="G604" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/supervisor-civil-at-eosol-4442238964", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-en-contratacion-de-obra-civil-bogota-1886759693", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H604" s="6" t="inlineStr"/>
@@ -28893,7 +28893,7 @@
     <row r="605" ht="22" customHeight="1">
       <c r="A605" s="2" t="inlineStr">
         <is>
-          <t>dc949850c44ae2c9</t>
+          <t>6ccccd3a1ba05f7f</t>
         </is>
       </c>
       <c r="B605" s="2" t="inlineStr">
@@ -28903,12 +28903,12 @@
       </c>
       <c r="C605" s="3" t="inlineStr">
         <is>
-          <t>Civil Engineer</t>
+          <t>14561-especialista interventoria-bogota</t>
         </is>
       </c>
       <c r="D605" s="3" t="inlineStr">
         <is>
-          <t>Cresta</t>
+          <t>APPLUS NORCONTROL COLOMBIA LTDA</t>
         </is>
       </c>
       <c r="E605" s="8" t="n">
@@ -28920,7 +28920,7 @@
         </is>
       </c>
       <c r="G605" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-engineer-at-cresta-4465582487", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/14561especialista-interventoriabogota-1886768886", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H605" s="6" t="inlineStr"/>
@@ -28939,7 +28939,7 @@
     <row r="606" ht="22" customHeight="1">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>4ad1a5acabdb8ad3</t>
+          <t>8ad0c11c4f07472e</t>
         </is>
       </c>
       <c r="B606" s="2" t="inlineStr">
@@ -28949,12 +28949,12 @@
       </c>
       <c r="C606" s="3" t="inlineStr">
         <is>
-          <t>Civil BIM Specialist</t>
+          <t>Ingeniero Civil / Terracerías</t>
         </is>
       </c>
       <c r="D606" s="3" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>EOSOL</t>
         </is>
       </c>
       <c r="E606" s="8" t="n">
@@ -28966,7 +28966,7 @@
         </is>
       </c>
       <c r="G606" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-bim-specialist-at-eng-4469886677", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-civil-terracer%C3%ADas-at-eosol-4445793534", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H606" s="6" t="inlineStr"/>
@@ -28985,7 +28985,7 @@
     <row r="607" ht="22" customHeight="1">
       <c r="A607" s="2" t="inlineStr">
         <is>
-          <t>5ebaba0a0c9927fb</t>
+          <t>ed46085f88d06bf5</t>
         </is>
       </c>
       <c r="B607" s="2" t="inlineStr">
@@ -28995,12 +28995,12 @@
       </c>
       <c r="C607" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero/a Civil-Estructuras Hormigón/Acero</t>
+          <t>Supervisor Civil</t>
         </is>
       </c>
       <c r="D607" s="3" t="inlineStr">
         <is>
-          <t>IDOM Consulting, Engineering, Architecture</t>
+          <t>EOSOL</t>
         </is>
       </c>
       <c r="E607" s="8" t="n">
@@ -29012,7 +29012,7 @@
         </is>
       </c>
       <c r="G607" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-a-civil-estructuras-hormig%C3%B3n-acero-at-idom-consulting-engineering-architecture-4462998187", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/supervisor-civil-at-eosol-4442238964", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H607" s="6" t="inlineStr"/>
@@ -29031,7 +29031,7 @@
     <row r="608" ht="22" customHeight="1">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>5c954c66c2c9d655</t>
+          <t>dc949850c44ae2c9</t>
         </is>
       </c>
       <c r="B608" s="2" t="inlineStr">
@@ -29041,12 +29041,12 @@
       </c>
       <c r="C608" s="3" t="inlineStr">
         <is>
-          <t>Civil Engineering-in-Training</t>
+          <t>Civil Engineer</t>
         </is>
       </c>
       <c r="D608" s="3" t="inlineStr">
         <is>
-          <t>WSP en Colombia</t>
+          <t>Cresta</t>
         </is>
       </c>
       <c r="E608" s="8" t="n">
@@ -29058,7 +29058,7 @@
         </is>
       </c>
       <c r="G608" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-engineering-in-training-french-at-wsp-en-colombia-4458430104", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-engineer-at-cresta-4465582487", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H608" s="6" t="inlineStr"/>
@@ -29077,7 +29077,7 @@
     <row r="609" ht="22" customHeight="1">
       <c r="A609" s="2" t="inlineStr">
         <is>
-          <t>571ae2aa81fa07b5</t>
+          <t>4ad1a5acabdb8ad3</t>
         </is>
       </c>
       <c r="B609" s="2" t="inlineStr">
@@ -29087,12 +29087,12 @@
       </c>
       <c r="C609" s="3" t="inlineStr">
         <is>
-          <t>Civil Engineering-in-Training</t>
+          <t>Civil BIM Specialist</t>
         </is>
       </c>
       <c r="D609" s="3" t="inlineStr">
         <is>
-          <t>WSP en Colombia</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="E609" s="8" t="n">
@@ -29104,7 +29104,7 @@
         </is>
       </c>
       <c r="G609" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-engineering-in-training-at-wsp-en-colombia-4458027784", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-bim-specialist-at-eng-4469886677", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H609" s="6" t="inlineStr"/>
@@ -29123,7 +29123,7 @@
     <row r="610" ht="22" customHeight="1">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>d94bcf92627b7b99</t>
+          <t>5ebaba0a0c9927fb</t>
         </is>
       </c>
       <c r="B610" s="2" t="inlineStr">
@@ -29133,12 +29133,12 @@
       </c>
       <c r="C610" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero civil</t>
+          <t>Ingeniero/a Civil-Estructuras Hormigón/Acero</t>
         </is>
       </c>
       <c r="D610" s="3" t="inlineStr">
         <is>
-          <t>HMV Ingenieros</t>
+          <t>IDOM Consulting, Engineering, Architecture</t>
         </is>
       </c>
       <c r="E610" s="8" t="n">
@@ -29150,7 +29150,7 @@
         </is>
       </c>
       <c r="G610" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-civil-at-hmv-ingenieros-4461715824", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-a-civil-estructuras-hormig%C3%B3n-acero-at-idom-consulting-engineering-architecture-4462998187", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H610" s="6" t="inlineStr"/>
@@ -29169,7 +29169,7 @@
     <row r="611" ht="22" customHeight="1">
       <c r="A611" s="2" t="inlineStr">
         <is>
-          <t>1be0a8e56fa4736b</t>
+          <t>5c954c66c2c9d655</t>
         </is>
       </c>
       <c r="B611" s="2" t="inlineStr">
@@ -29179,12 +29179,12 @@
       </c>
       <c r="C611" s="3" t="inlineStr">
         <is>
-          <t>Civil Engineer</t>
+          <t>Civil Engineering-in-Training</t>
         </is>
       </c>
       <c r="D611" s="3" t="inlineStr">
         <is>
-          <t>Wood</t>
+          <t>WSP en Colombia</t>
         </is>
       </c>
       <c r="E611" s="8" t="n">
@@ -29196,7 +29196,7 @@
         </is>
       </c>
       <c r="G611" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-engineer-at-wood-4418961778", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-engineering-in-training-french-at-wsp-en-colombia-4458430104", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H611" s="6" t="inlineStr"/>
@@ -29215,7 +29215,7 @@
     <row r="612" ht="22" customHeight="1">
       <c r="A612" s="2" t="inlineStr">
         <is>
-          <t>825c4e246cbd6b6b</t>
+          <t>571ae2aa81fa07b5</t>
         </is>
       </c>
       <c r="B612" s="2" t="inlineStr">
@@ -29225,12 +29225,12 @@
       </c>
       <c r="C612" s="3" t="inlineStr">
         <is>
-          <t>Civil Engineering Expert</t>
+          <t>Civil Engineering-in-Training</t>
         </is>
       </c>
       <c r="D612" s="3" t="inlineStr">
         <is>
-          <t>Anyone AI</t>
+          <t>WSP en Colombia</t>
         </is>
       </c>
       <c r="E612" s="8" t="n">
@@ -29242,7 +29242,7 @@
         </is>
       </c>
       <c r="G612" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-engineering-expert-at-anyone-ai-4462461832", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-engineering-in-training-at-wsp-en-colombia-4458027784", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H612" s="6" t="inlineStr"/>
@@ -29261,7 +29261,7 @@
     <row r="613" ht="22" customHeight="1">
       <c r="A613" s="2" t="inlineStr">
         <is>
-          <t>76740179a82340ae</t>
+          <t>d94bcf92627b7b99</t>
         </is>
       </c>
       <c r="B613" s="2" t="inlineStr">
@@ -29271,12 +29271,12 @@
       </c>
       <c r="C613" s="3" t="inlineStr">
         <is>
-          <t>Profesional en Ingeniería Civil</t>
+          <t>Ingeniero civil</t>
         </is>
       </c>
       <c r="D613" s="3" t="inlineStr">
         <is>
-          <t>CMH Colombia</t>
+          <t>HMV Ingenieros</t>
         </is>
       </c>
       <c r="E613" s="8" t="n">
@@ -29288,7 +29288,7 @@
         </is>
       </c>
       <c r="G613" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/profesional-en-ingenier%C3%ADa-civil-at-minerales-c%C3%B3rdoba-4450022471", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-civil-at-hmv-ingenieros-4461715824", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H613" s="6" t="inlineStr"/>
@@ -29307,7 +29307,7 @@
     <row r="614" ht="22" customHeight="1">
       <c r="A614" s="2" t="inlineStr">
         <is>
-          <t>5bea04b9e734c2fc</t>
+          <t>1be0a8e56fa4736b</t>
         </is>
       </c>
       <c r="B614" s="2" t="inlineStr">
@@ -29317,12 +29317,12 @@
       </c>
       <c r="C614" s="3" t="inlineStr">
         <is>
-          <t>Coordinador HSEQ</t>
+          <t>Civil Engineer</t>
         </is>
       </c>
       <c r="D614" s="3" t="inlineStr">
         <is>
-          <t>ASSEMTEC</t>
+          <t>Wood</t>
         </is>
       </c>
       <c r="E614" s="8" t="n">
@@ -29334,13 +29334,13 @@
         </is>
       </c>
       <c r="G614" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-hseq-at-assemtec-4457664932", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-engineer-at-wood-4418961778", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H614" s="6" t="inlineStr"/>
       <c r="I614" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J614" s="2" t="inlineStr">
@@ -29353,7 +29353,7 @@
     <row r="615" ht="22" customHeight="1">
       <c r="A615" s="2" t="inlineStr">
         <is>
-          <t>6ba6bae2d7bfb226</t>
+          <t>825c4e246cbd6b6b</t>
         </is>
       </c>
       <c r="B615" s="2" t="inlineStr">
@@ -29363,12 +29363,12 @@
       </c>
       <c r="C615" s="3" t="inlineStr">
         <is>
-          <t>Inspector SST con Licencia, Coordinador de Alturas</t>
+          <t>Civil Engineering Expert</t>
         </is>
       </c>
       <c r="D615" s="3" t="inlineStr">
         <is>
-          <t>Asertempo Colombia S.A.S</t>
+          <t>Anyone AI</t>
         </is>
       </c>
       <c r="E615" s="8" t="n">
@@ -29380,13 +29380,13 @@
         </is>
       </c>
       <c r="G615" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/inspector-sst-con-licencia-coordinador-de-alturas-at-asertempo-colombia-s-a-s-4464408367", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-engineering-expert-at-anyone-ai-4462461832", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H615" s="6" t="inlineStr"/>
       <c r="I615" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J615" s="2" t="inlineStr">
@@ -29399,7 +29399,7 @@
     <row r="616" ht="22" customHeight="1">
       <c r="A616" s="2" t="inlineStr">
         <is>
-          <t>0df4a63a82189896</t>
+          <t>76740179a82340ae</t>
         </is>
       </c>
       <c r="B616" s="2" t="inlineStr">
@@ -29409,12 +29409,12 @@
       </c>
       <c r="C616" s="3" t="inlineStr">
         <is>
-          <t>Especialista en Salud y Seguridad en el trabajo con especialización en medio Ambiente</t>
+          <t>Profesional en Ingeniería Civil</t>
         </is>
       </c>
       <c r="D616" s="3" t="inlineStr">
         <is>
-          <t>Dextera IT Services</t>
+          <t>CMH Colombia</t>
         </is>
       </c>
       <c r="E616" s="8" t="n">
@@ -29426,7 +29426,7 @@
         </is>
       </c>
       <c r="G616" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/especialista-en-salud-y-seguridad-en-el-trabajo-con-especializaci%C3%B3n-en-medio-ambiente-at-dextera-it-services-4464024362", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/profesional-en-ingenier%C3%ADa-civil-at-minerales-c%C3%B3rdoba-4450022471", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H616" s="6" t="inlineStr"/>
@@ -29445,7 +29445,7 @@
     <row r="617" ht="22" customHeight="1">
       <c r="A617" s="2" t="inlineStr">
         <is>
-          <t>e8e3c75915d1945c</t>
+          <t>5bea04b9e734c2fc</t>
         </is>
       </c>
       <c r="B617" s="2" t="inlineStr">
@@ -29455,12 +29455,12 @@
       </c>
       <c r="C617" s="3" t="inlineStr">
         <is>
-          <t>Coordinador (a) profesional HSEQ</t>
+          <t>Coordinador HSEQ</t>
         </is>
       </c>
       <c r="D617" s="3" t="inlineStr">
         <is>
-          <t>SD SAS</t>
+          <t>ASSEMTEC</t>
         </is>
       </c>
       <c r="E617" s="8" t="n">
@@ -29472,7 +29472,7 @@
         </is>
       </c>
       <c r="G617" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-a-profesional-hseq-at-sd-sas-4444939872", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-hseq-at-assemtec-4457664932", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H617" s="6" t="inlineStr"/>
@@ -29491,7 +29491,7 @@
     <row r="618" ht="22" customHeight="1">
       <c r="A618" s="2" t="inlineStr">
         <is>
-          <t>fb37fc1bf485e650</t>
+          <t>6ba6bae2d7bfb226</t>
         </is>
       </c>
       <c r="B618" s="2" t="inlineStr">
@@ -29501,12 +29501,12 @@
       </c>
       <c r="C618" s="3" t="inlineStr">
         <is>
-          <t>Técnico de trazado especialista en ISTRAM</t>
+          <t>Inspector SST con Licencia, Coordinador de Alturas</t>
         </is>
       </c>
       <c r="D618" s="3" t="inlineStr">
         <is>
-          <t>EADIC</t>
+          <t>Asertempo Colombia S.A.S</t>
         </is>
       </c>
       <c r="E618" s="8" t="n">
@@ -29518,13 +29518,13 @@
         </is>
       </c>
       <c r="G618" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/t%C3%A9cnico-de-trazado-especialista-en-istram-at-eadic-4468780158", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/inspector-sst-con-licencia-coordinador-de-alturas-at-asertempo-colombia-s-a-s-4464408367", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H618" s="6" t="inlineStr"/>
       <c r="I618" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J618" s="2" t="inlineStr">
@@ -29537,7 +29537,7 @@
     <row r="619" ht="22" customHeight="1">
       <c r="A619" s="2" t="inlineStr">
         <is>
-          <t>0f01a66eb85a1ffd</t>
+          <t>0df4a63a82189896</t>
         </is>
       </c>
       <c r="B619" s="2" t="inlineStr">
@@ -29547,12 +29547,12 @@
       </c>
       <c r="C619" s="3" t="inlineStr">
         <is>
-          <t>AUXILIAR MODELADOR BIM Y DIBUJANTE EN INGENIERÍA CIVIL</t>
+          <t>Especialista en Salud y Seguridad en el trabajo con especialización en medio Ambiente</t>
         </is>
       </c>
       <c r="D619" s="3" t="inlineStr">
         <is>
-          <t>Antea Group España y Latinoamérica</t>
+          <t>Dextera IT Services</t>
         </is>
       </c>
       <c r="E619" s="8" t="n">
@@ -29564,7 +29564,7 @@
         </is>
       </c>
       <c r="G619" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/auxiliar-modelador-bim-y-dibujante-en-ingenier%C3%ADa-civil-at-antea-group-espa%C3%B1a-y-latinoam%C3%A9rica-4467605615", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/especialista-en-salud-y-seguridad-en-el-trabajo-con-especializaci%C3%B3n-en-medio-ambiente-at-dextera-it-services-4464024362", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H619" s="6" t="inlineStr"/>
@@ -29583,7 +29583,7 @@
     <row r="620" ht="22" customHeight="1">
       <c r="A620" s="2" t="inlineStr">
         <is>
-          <t>cba614af5ce1fc3a</t>
+          <t>e8e3c75915d1945c</t>
         </is>
       </c>
       <c r="B620" s="2" t="inlineStr">
@@ -29593,12 +29593,12 @@
       </c>
       <c r="C620" s="3" t="inlineStr">
         <is>
-          <t>Principal Pavement Engineer - Linear Infrastructure &amp; Site Civils</t>
+          <t>Coordinador (a) profesional HSEQ</t>
         </is>
       </c>
       <c r="D620" s="3" t="inlineStr">
         <is>
-          <t>AECOM</t>
+          <t>SD SAS</t>
         </is>
       </c>
       <c r="E620" s="8" t="n">
@@ -29610,13 +29610,13 @@
         </is>
       </c>
       <c r="G620" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/principal-pavement-engineer-linear-infrastructure-site-civils-at-aecom-4403657428", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-a-profesional-hseq-at-sd-sas-4444939872", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H620" s="6" t="inlineStr"/>
       <c r="I620" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J620" s="2" t="inlineStr">
@@ -29629,7 +29629,7 @@
     <row r="621" ht="22" customHeight="1">
       <c r="A621" s="2" t="inlineStr">
         <is>
-          <t>2bafc4e5eb29746b</t>
+          <t>fb37fc1bf485e650</t>
         </is>
       </c>
       <c r="B621" s="2" t="inlineStr">
@@ -29639,12 +29639,12 @@
       </c>
       <c r="C621" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero/a Geotécnico/a Senior</t>
+          <t>Técnico de trazado especialista en ISTRAM</t>
         </is>
       </c>
       <c r="D621" s="3" t="inlineStr">
         <is>
-          <t>IDOM Consulting, Engineering, Architecture</t>
+          <t>EADIC</t>
         </is>
       </c>
       <c r="E621" s="8" t="n">
@@ -29656,7 +29656,7 @@
         </is>
       </c>
       <c r="G621" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-a-geot%C3%A9cnico-a-senior-at-idom-consulting-engineering-architecture-4467729578", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/t%C3%A9cnico-de-trazado-especialista-en-istram-at-eadic-4468780158", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H621" s="6" t="inlineStr"/>
@@ -29675,7 +29675,7 @@
     <row r="622" ht="22" customHeight="1">
       <c r="A622" s="2" t="inlineStr">
         <is>
-          <t>f3290f3c2a2d0061</t>
+          <t>0f01a66eb85a1ffd</t>
         </is>
       </c>
       <c r="B622" s="2" t="inlineStr">
@@ -29685,12 +29685,12 @@
       </c>
       <c r="C622" s="3" t="inlineStr">
         <is>
-          <t>Engenheiro Civil - Lisboa</t>
+          <t>AUXILIAR MODELADOR BIM Y DIBUJANTE EN INGENIERÍA CIVIL</t>
         </is>
       </c>
       <c r="D622" s="3" t="inlineStr">
         <is>
-          <t>DDN GERENCIAMENTO</t>
+          <t>Antea Group España y Latinoamérica</t>
         </is>
       </c>
       <c r="E622" s="8" t="n">
@@ -29702,7 +29702,7 @@
         </is>
       </c>
       <c r="G622" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/engenheiro-civil-lisboa-at-ddn-gerenciamento-4468408791", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/auxiliar-modelador-bim-y-dibujante-en-ingenier%C3%ADa-civil-at-antea-group-espa%C3%B1a-y-latinoam%C3%A9rica-4467605615", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H622" s="6" t="inlineStr"/>
@@ -29721,7 +29721,7 @@
     <row r="623" ht="22" customHeight="1">
       <c r="A623" s="2" t="inlineStr">
         <is>
-          <t>d2feccf91b9b1f0b</t>
+          <t>cba614af5ce1fc3a</t>
         </is>
       </c>
       <c r="B623" s="2" t="inlineStr">
@@ -29731,12 +29731,12 @@
       </c>
       <c r="C623" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero/a Civil especialista en Talleres y Patios Ferroviarios</t>
+          <t>Principal Pavement Engineer - Linear Infrastructure &amp; Site Civils</t>
         </is>
       </c>
       <c r="D623" s="3" t="inlineStr">
         <is>
-          <t>IDOM Consulting, Engineering, Architecture</t>
+          <t>AECOM</t>
         </is>
       </c>
       <c r="E623" s="8" t="n">
@@ -29748,7 +29748,7 @@
         </is>
       </c>
       <c r="G623" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-a-civil-especialista-en-talleres-y-patios-ferroviarios-at-idom-consulting-engineering-architecture-4443713908", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/principal-pavement-engineer-linear-infrastructure-site-civils-at-aecom-4403657428", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H623" s="6" t="inlineStr"/>
@@ -29767,7 +29767,7 @@
     <row r="624" ht="22" customHeight="1">
       <c r="A624" s="2" t="inlineStr">
         <is>
-          <t>152ea7f07f195fc8</t>
+          <t>2bafc4e5eb29746b</t>
         </is>
       </c>
       <c r="B624" s="2" t="inlineStr">
@@ -29777,12 +29777,12 @@
       </c>
       <c r="C624" s="3" t="inlineStr">
         <is>
-          <t>COORDINADOR DE INTERVENTORÍA-NIVEL 1 SECTOR HIDROCARBUROS</t>
+          <t>Ingeniero/a Geotécnico/a Senior</t>
         </is>
       </c>
       <c r="D624" s="3" t="inlineStr">
         <is>
-          <t>Centro de Empleo y Talento</t>
+          <t>IDOM Consulting, Engineering, Architecture</t>
         </is>
       </c>
       <c r="E624" s="8" t="n">
@@ -29794,7 +29794,7 @@
         </is>
       </c>
       <c r="G624" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-de-interventor%C3%ADa-nivel-1-sector-hidrocarburos-at-centro-de-empleo-y-talento-4468030406", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-a-geot%C3%A9cnico-a-senior-at-idom-consulting-engineering-architecture-4467729578", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H624" s="6" t="inlineStr"/>
@@ -29813,7 +29813,7 @@
     <row r="625" ht="22" customHeight="1">
       <c r="A625" s="2" t="inlineStr">
         <is>
-          <t>b3dd7e9d8f53fb27</t>
+          <t>f3290f3c2a2d0061</t>
         </is>
       </c>
       <c r="B625" s="2" t="inlineStr">
@@ -29823,12 +29823,12 @@
       </c>
       <c r="C625" s="3" t="inlineStr">
         <is>
-          <t>Consultor (Desarrollador) Senior Appian</t>
+          <t>Engenheiro Civil - Lisboa</t>
         </is>
       </c>
       <c r="D625" s="3" t="inlineStr">
         <is>
-          <t>VASS LATAM</t>
+          <t>DDN GERENCIAMENTO</t>
         </is>
       </c>
       <c r="E625" s="8" t="n">
@@ -29840,7 +29840,7 @@
         </is>
       </c>
       <c r="G625" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/consultor-desarrollador-senior-appian-at-vass-latam-4458249659", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/engenheiro-civil-lisboa-at-ddn-gerenciamento-4468408791", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H625" s="6" t="inlineStr"/>
@@ -29859,7 +29859,7 @@
     <row r="626" ht="22" customHeight="1">
       <c r="A626" s="2" t="inlineStr">
         <is>
-          <t>0f895f69320d7d8d</t>
+          <t>d2feccf91b9b1f0b</t>
         </is>
       </c>
       <c r="B626" s="2" t="inlineStr">
@@ -29869,12 +29869,12 @@
       </c>
       <c r="C626" s="3" t="inlineStr">
         <is>
-          <t>Coordinador hse Cartagena</t>
+          <t>Ingeniero/a Civil especialista en Talleres y Patios Ferroviarios</t>
         </is>
       </c>
       <c r="D626" s="3" t="inlineStr">
         <is>
-          <t>TRANSPORTES MONTEJO SAS</t>
+          <t>IDOM Consulting, Engineering, Architecture</t>
         </is>
       </c>
       <c r="E626" s="8" t="n">
@@ -29886,13 +29886,13 @@
         </is>
       </c>
       <c r="G626" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-hse-cartagena-at-transportes-montejo-sas-4458746462", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-a-civil-especialista-en-talleres-y-patios-ferroviarios-at-idom-consulting-engineering-architecture-4443713908", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H626" s="6" t="inlineStr"/>
       <c r="I626" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J626" s="2" t="inlineStr">
@@ -29905,7 +29905,7 @@
     <row r="627" ht="22" customHeight="1">
       <c r="A627" s="2" t="inlineStr">
         <is>
-          <t>b86d50ad2dd5f642</t>
+          <t>152ea7f07f195fc8</t>
         </is>
       </c>
       <c r="B627" s="2" t="inlineStr">
@@ -29915,12 +29915,12 @@
       </c>
       <c r="C627" s="3" t="inlineStr">
         <is>
-          <t>Coordinador Regional SIG/ SST</t>
+          <t>COORDINADOR DE INTERVENTORÍA-NIVEL 1 SECTOR HIDROCARBUROS</t>
         </is>
       </c>
       <c r="D627" s="3" t="inlineStr">
         <is>
-          <t>Interaseo S.A.S. E.S.P.</t>
+          <t>Centro de Empleo y Talento</t>
         </is>
       </c>
       <c r="E627" s="8" t="n">
@@ -29932,13 +29932,13 @@
         </is>
       </c>
       <c r="G627" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-regional-sig-sst-at-interaseo-s-a-s-e-s-p-4459088040", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-de-interventor%C3%ADa-nivel-1-sector-hidrocarburos-at-centro-de-empleo-y-talento-4468030406", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H627" s="6" t="inlineStr"/>
       <c r="I627" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J627" s="2" t="inlineStr">
@@ -29951,7 +29951,7 @@
     <row r="628" ht="22" customHeight="1">
       <c r="A628" s="2" t="inlineStr">
         <is>
-          <t>506296811a5a9cbb</t>
+          <t>b3dd7e9d8f53fb27</t>
         </is>
       </c>
       <c r="B628" s="2" t="inlineStr">
@@ -29961,12 +29961,12 @@
       </c>
       <c r="C628" s="3" t="inlineStr">
         <is>
-          <t>Coordinador/a de SST</t>
+          <t>Consultor (Desarrollador) Senior Appian</t>
         </is>
       </c>
       <c r="D628" s="3" t="inlineStr">
         <is>
-          <t>Estelar Food S.A.S</t>
+          <t>VASS LATAM</t>
         </is>
       </c>
       <c r="E628" s="8" t="n">
@@ -29978,13 +29978,13 @@
         </is>
       </c>
       <c r="G628" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-a-de-sst-at-estelar-food-s-a-s-4462115593", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/consultor-desarrollador-senior-appian-at-vass-latam-4458249659", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H628" s="6" t="inlineStr"/>
       <c r="I628" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J628" s="2" t="inlineStr">
@@ -29997,7 +29997,7 @@
     <row r="629" ht="22" customHeight="1">
       <c r="A629" s="2" t="inlineStr">
         <is>
-          <t>0e4b8eed7f32714e</t>
+          <t>0f895f69320d7d8d</t>
         </is>
       </c>
       <c r="B629" s="2" t="inlineStr">
@@ -30007,12 +30007,12 @@
       </c>
       <c r="C629" s="3" t="inlineStr">
         <is>
-          <t>coordinador de Seguridad y Salud en el Trabajo</t>
+          <t>Coordinador hse Cartagena</t>
         </is>
       </c>
       <c r="D629" s="3" t="inlineStr">
         <is>
-          <t>Asertempo Colombia S.A.S</t>
+          <t>TRANSPORTES MONTEJO SAS</t>
         </is>
       </c>
       <c r="E629" s="8" t="n">
@@ -30024,7 +30024,7 @@
         </is>
       </c>
       <c r="G629" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-de-seguridad-y-salud-en-el-trabajo-at-asertempo-colombia-s-a-s-4461723686", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-hse-cartagena-at-transportes-montejo-sas-4458746462", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H629" s="6" t="inlineStr"/>
@@ -30043,7 +30043,7 @@
     <row r="630" ht="22" customHeight="1">
       <c r="A630" s="2" t="inlineStr">
         <is>
-          <t>aa2882af3c61095b</t>
+          <t>b86d50ad2dd5f642</t>
         </is>
       </c>
       <c r="B630" s="2" t="inlineStr">
@@ -30053,12 +30053,12 @@
       </c>
       <c r="C630" s="3" t="inlineStr">
         <is>
-          <t>Coordinador (a) SST / APH - Marmato</t>
+          <t>Coordinador Regional SIG/ SST</t>
         </is>
       </c>
       <c r="D630" s="3" t="inlineStr">
         <is>
-          <t>Aris Mining Colombia</t>
+          <t>Interaseo S.A.S. E.S.P.</t>
         </is>
       </c>
       <c r="E630" s="8" t="n">
@@ -30070,7 +30070,7 @@
         </is>
       </c>
       <c r="G630" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-a-sst-aph-marmato-at-aris-mining-colombia-4448929810", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-regional-sig-sst-at-interaseo-s-a-s-e-s-p-4459088040", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H630" s="6" t="inlineStr"/>
@@ -30089,7 +30089,7 @@
     <row r="631" ht="22" customHeight="1">
       <c r="A631" s="2" t="inlineStr">
         <is>
-          <t>26cff43f13982962</t>
+          <t>506296811a5a9cbb</t>
         </is>
       </c>
       <c r="B631" s="2" t="inlineStr">
@@ -30099,12 +30099,12 @@
       </c>
       <c r="C631" s="3" t="inlineStr">
         <is>
-          <t>Consultor(a) Senior SOX TI</t>
+          <t>Coordinador/a de SST</t>
         </is>
       </c>
       <c r="D631" s="3" t="inlineStr">
         <is>
-          <t>Hitss Colombia</t>
+          <t>Estelar Food S.A.S</t>
         </is>
       </c>
       <c r="E631" s="8" t="n">
@@ -30116,13 +30116,13 @@
         </is>
       </c>
       <c r="G631" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/consultor-a-senior-sox-ti-at-hitss-colombia-4460766744", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-a-de-sst-at-estelar-food-s-a-s-4462115593", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H631" s="6" t="inlineStr"/>
       <c r="I631" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J631" s="2" t="inlineStr">
@@ -30135,7 +30135,7 @@
     <row r="632" ht="22" customHeight="1">
       <c r="A632" s="2" t="inlineStr">
         <is>
-          <t>87e367215ed55502</t>
+          <t>0e4b8eed7f32714e</t>
         </is>
       </c>
       <c r="B632" s="2" t="inlineStr">
@@ -30145,12 +30145,12 @@
       </c>
       <c r="C632" s="3" t="inlineStr">
         <is>
-          <t>Consultor(a) Senior Auditoría Interna</t>
+          <t>coordinador de Seguridad y Salud en el Trabajo</t>
         </is>
       </c>
       <c r="D632" s="3" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>Asertempo Colombia S.A.S</t>
         </is>
       </c>
       <c r="E632" s="8" t="n">
@@ -30162,13 +30162,13 @@
         </is>
       </c>
       <c r="G632" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/consultor-a-senior-auditor%C3%ADa-interna-at-deloitte-4462090075", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-de-seguridad-y-salud-en-el-trabajo-at-asertempo-colombia-s-a-s-4461723686", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H632" s="6" t="inlineStr"/>
       <c r="I632" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J632" s="2" t="inlineStr">
@@ -30181,7 +30181,7 @@
     <row r="633" ht="22" customHeight="1">
       <c r="A633" s="2" t="inlineStr">
         <is>
-          <t>e2e525b51bbd0e5e</t>
+          <t>aa2882af3c61095b</t>
         </is>
       </c>
       <c r="B633" s="2" t="inlineStr">
@@ -30191,12 +30191,12 @@
       </c>
       <c r="C633" s="3" t="inlineStr">
         <is>
-          <t>Coordinador/a de Salud y Bienestar (HSE) Latam</t>
+          <t>Coordinador (a) SST / APH - Marmato</t>
         </is>
       </c>
       <c r="D633" s="3" t="inlineStr">
         <is>
-          <t>Aqualia</t>
+          <t>Aris Mining Colombia</t>
         </is>
       </c>
       <c r="E633" s="8" t="n">
@@ -30208,7 +30208,7 @@
         </is>
       </c>
       <c r="G633" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-a-de-salud-y-bienestar-hse-latam-at-aqualia-4463977352", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-a-sst-aph-marmato-at-aris-mining-colombia-4448929810", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H633" s="6" t="inlineStr"/>
@@ -30227,7 +30227,7 @@
     <row r="634" ht="22" customHeight="1">
       <c r="A634" s="2" t="inlineStr">
         <is>
-          <t>8ef614b651dfe9d9</t>
+          <t>26cff43f13982962</t>
         </is>
       </c>
       <c r="B634" s="2" t="inlineStr">
@@ -30237,12 +30237,12 @@
       </c>
       <c r="C634" s="3" t="inlineStr">
         <is>
-          <t>Lead Civil Site Engineer</t>
+          <t>Consultor(a) Senior SOX TI</t>
         </is>
       </c>
       <c r="D634" s="3" t="inlineStr">
         <is>
-          <t>AECOM</t>
+          <t>Hitss Colombia</t>
         </is>
       </c>
       <c r="E634" s="8" t="n">
@@ -30254,7 +30254,7 @@
         </is>
       </c>
       <c r="G634" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/lead-civil-site-engineer-at-aecom-4468059409", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/consultor-a-senior-sox-ti-at-hitss-colombia-4460766744", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H634" s="6" t="inlineStr"/>
@@ -30273,7 +30273,7 @@
     <row r="635" ht="22" customHeight="1">
       <c r="A635" s="2" t="inlineStr">
         <is>
-          <t>b339389a0d32a94f</t>
+          <t>87e367215ed55502</t>
         </is>
       </c>
       <c r="B635" s="2" t="inlineStr">
@@ -30283,12 +30283,12 @@
       </c>
       <c r="C635" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero civil</t>
+          <t>Consultor(a) Senior Auditoría Interna</t>
         </is>
       </c>
       <c r="D635" s="3" t="inlineStr">
         <is>
-          <t>constructora cumbrera</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="E635" s="8" t="n">
@@ -30300,7 +30300,7 @@
         </is>
       </c>
       <c r="G635" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-civil-4463108593", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/consultor-a-senior-auditor%C3%ADa-interna-at-deloitte-4462090075", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H635" s="6" t="inlineStr"/>
@@ -30319,7 +30319,7 @@
     <row r="636" ht="22" customHeight="1">
       <c r="A636" s="2" t="inlineStr">
         <is>
-          <t>93623c0212e39cb9</t>
+          <t>e2e525b51bbd0e5e</t>
         </is>
       </c>
       <c r="B636" s="2" t="inlineStr">
@@ -30329,12 +30329,12 @@
       </c>
       <c r="C636" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero(a) Civil</t>
+          <t>Coordinador/a de Salud y Bienestar (HSE) Latam</t>
         </is>
       </c>
       <c r="D636" s="3" t="inlineStr">
         <is>
-          <t>CMH Colombia</t>
+          <t>Aqualia</t>
         </is>
       </c>
       <c r="E636" s="8" t="n">
@@ -30346,13 +30346,13 @@
         </is>
       </c>
       <c r="G636" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-a-civil-at-minerales-c%C3%B3rdoba-4417533007", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-a-de-salud-y-bienestar-hse-latam-at-aqualia-4463977352", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H636" s="6" t="inlineStr"/>
       <c r="I636" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J636" s="2" t="inlineStr">
@@ -30365,7 +30365,7 @@
     <row r="637" ht="22" customHeight="1">
       <c r="A637" s="2" t="inlineStr">
         <is>
-          <t>cd06fbe3d5b74888</t>
+          <t>8ef614b651dfe9d9</t>
         </is>
       </c>
       <c r="B637" s="2" t="inlineStr">
@@ -30375,12 +30375,12 @@
       </c>
       <c r="C637" s="3" t="inlineStr">
         <is>
-          <t>Oficial Obra Civil</t>
+          <t>Lead Civil Site Engineer</t>
         </is>
       </c>
       <c r="D637" s="3" t="inlineStr">
         <is>
-          <t>Equans Colombia</t>
+          <t>AECOM</t>
         </is>
       </c>
       <c r="E637" s="8" t="n">
@@ -30392,7 +30392,7 @@
         </is>
       </c>
       <c r="G637" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/oficial-obra-civil-bogota-y-cundinamarca-at-equans-colombia-4470218146", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/lead-civil-site-engineer-at-aecom-4468059409", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H637" s="6" t="inlineStr"/>
@@ -30408,9 +30408,147 @@
       </c>
       <c r="K637" s="3" t="inlineStr"/>
     </row>
+    <row r="638" ht="22" customHeight="1">
+      <c r="A638" s="2" t="inlineStr">
+        <is>
+          <t>b339389a0d32a94f</t>
+        </is>
+      </c>
+      <c r="B638" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 05:09</t>
+        </is>
+      </c>
+      <c r="C638" s="3" t="inlineStr">
+        <is>
+          <t>Ingeniero civil</t>
+        </is>
+      </c>
+      <c r="D638" s="3" t="inlineStr">
+        <is>
+          <t>constructora cumbrera</t>
+        </is>
+      </c>
+      <c r="E638" s="8" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F638" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G638" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-civil-4463108593", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H638" s="6" t="inlineStr"/>
+      <c r="I638" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J638" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K638" s="3" t="inlineStr"/>
+    </row>
+    <row r="639" ht="22" customHeight="1">
+      <c r="A639" s="2" t="inlineStr">
+        <is>
+          <t>93623c0212e39cb9</t>
+        </is>
+      </c>
+      <c r="B639" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 05:09</t>
+        </is>
+      </c>
+      <c r="C639" s="3" t="inlineStr">
+        <is>
+          <t>Ingeniero(a) Civil</t>
+        </is>
+      </c>
+      <c r="D639" s="3" t="inlineStr">
+        <is>
+          <t>CMH Colombia</t>
+        </is>
+      </c>
+      <c r="E639" s="8" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F639" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G639" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-a-civil-at-minerales-c%C3%B3rdoba-4417533007", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H639" s="6" t="inlineStr"/>
+      <c r="I639" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J639" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K639" s="3" t="inlineStr"/>
+    </row>
+    <row r="640" ht="22" customHeight="1">
+      <c r="A640" s="2" t="inlineStr">
+        <is>
+          <t>cd06fbe3d5b74888</t>
+        </is>
+      </c>
+      <c r="B640" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 05:09</t>
+        </is>
+      </c>
+      <c r="C640" s="3" t="inlineStr">
+        <is>
+          <t>Oficial Obra Civil</t>
+        </is>
+      </c>
+      <c r="D640" s="3" t="inlineStr">
+        <is>
+          <t>Equans Colombia</t>
+        </is>
+      </c>
+      <c r="E640" s="8" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F640" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G640" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/oficial-obra-civil-bogota-y-cundinamarca-at-equans-colombia-4470218146", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H640" s="6" t="inlineStr"/>
+      <c r="I640" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J640" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K640" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J836" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J839" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Nueva,Por revisar,Postulado,Descartado,Entrevista"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
chore(tracker): actualizacion diaria de vacantes 2026-10-19
</commit_message>
<xml_diff>
--- a/output/profile_1_civil_vias_sst_tracker.xlsx
+++ b/output/profile_1_civil_vias_sst_tracker.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K640"/>
+  <dimension ref="A1:K648"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -25537,26 +25537,26 @@
     <row r="533" ht="22" customHeight="1">
       <c r="A533" s="2" t="inlineStr">
         <is>
-          <t>4426b2c17306f519</t>
+          <t>f77356fba7f7ea68</t>
         </is>
       </c>
       <c r="B533" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 05:09</t>
+          <t>2026-10-19 17:27</t>
         </is>
       </c>
       <c r="C533" s="3" t="inlineStr">
         <is>
-          <t>Residente de Seguridad y Salud en el trabajo</t>
+          <t>Analista de Seguridad y Salud en el Trabajo</t>
         </is>
       </c>
       <c r="D533" s="3" t="inlineStr">
         <is>
-          <t>Cal y Mayor y Asociados S.C</t>
-        </is>
-      </c>
-      <c r="E533" s="8" t="n">
-        <v>0.48</v>
+          <t>Takami S.A</t>
+        </is>
+      </c>
+      <c r="E533" s="7" t="n">
+        <v>0.5</v>
       </c>
       <c r="F533" s="2" t="inlineStr">
         <is>
@@ -25564,17 +25564,13 @@
         </is>
       </c>
       <c r="G533" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-residente-de-seguridad-y-salud-en-el-trabajo-sst-sst-en-bogota-dc-D67E64C3D53E0D6961373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H533" s="6" t="inlineStr">
-        <is>
-          <t>$ 4.200.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analista-de-seguridad-y-salud-en-el-trabajo-analista-sst-en-bogota-dc-0FC1FA07D486E6FB61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H533" s="6" t="inlineStr"/>
       <c r="I533" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J533" s="2" t="inlineStr">
@@ -25587,26 +25583,26 @@
     <row r="534" ht="22" customHeight="1">
       <c r="A534" s="2" t="inlineStr">
         <is>
-          <t>83015d6afb890f1d</t>
+          <t>23251498ce710db0</t>
         </is>
       </c>
       <c r="B534" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 05:09</t>
+          <t>2026-10-19 17:27</t>
         </is>
       </c>
       <c r="C534" s="3" t="inlineStr">
         <is>
-          <t>Analista/profesional HSEQ / SST Sesquile o Alrededores</t>
+          <t>Director de Proyecto</t>
         </is>
       </c>
       <c r="D534" s="3" t="inlineStr">
         <is>
-          <t>ACTIVOS S A S</t>
-        </is>
-      </c>
-      <c r="E534" s="8" t="n">
-        <v>0.48</v>
+          <t>GESTION DE RECURSOS TEMPORALES S.A.S. "GR TEMPORALES S.A.S."</t>
+        </is>
+      </c>
+      <c r="E534" s="7" t="n">
+        <v>0.5</v>
       </c>
       <c r="F534" s="2" t="inlineStr">
         <is>
@@ -25614,17 +25610,17 @@
         </is>
       </c>
       <c r="G534" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analistaprofesional-hseq-sst-sesquile-o-alrededores-sector-consumo-masivo-en-sesquile-632A9566338A59E361373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-director-de-proyecto-obras-y-montajes-en-medellin-109E3C7C5CB623BA61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H534" s="6" t="inlineStr">
         <is>
-          <t>$ 4.000.000,00 (Mensual)</t>
+          <t>$ 5.000.000,00 (Mensual)</t>
         </is>
       </c>
       <c r="I534" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J534" s="2" t="inlineStr">
@@ -25637,26 +25633,26 @@
     <row r="535" ht="22" customHeight="1">
       <c r="A535" s="2" t="inlineStr">
         <is>
-          <t>bc0b38b5129e0905</t>
+          <t>c3249bf92df00c21</t>
         </is>
       </c>
       <c r="B535" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 05:09</t>
+          <t>2026-10-19 17:27</t>
         </is>
       </c>
       <c r="C535" s="3" t="inlineStr">
         <is>
-          <t>Profesional en seguridad y salud en el trabajo SST</t>
+          <t>Analista de seguridad y salud en el trabajo</t>
         </is>
       </c>
       <c r="D535" s="3" t="inlineStr">
         <is>
-          <t>Seguridad y Vigilancia Exito de Colombia</t>
-        </is>
-      </c>
-      <c r="E535" s="8" t="n">
-        <v>0.48</v>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E535" s="7" t="n">
+        <v>0.5</v>
       </c>
       <c r="F535" s="2" t="inlineStr">
         <is>
@@ -25664,17 +25660,13 @@
         </is>
       </c>
       <c r="G535" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-profesional-en-seguridad-y-salud-en-el-trabajo-sst-con-experiencia-y-conocimiento-en-pesv-en-bogota-dc-A7CA6F8805D1C53B61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H535" s="6" t="inlineStr">
-        <is>
-          <t>$ 3.200.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-seguridad-y-salud-en-el-trabajo-1886781980", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H535" s="6" t="inlineStr"/>
       <c r="I535" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J535" s="2" t="inlineStr">
@@ -25687,26 +25679,26 @@
     <row r="536" ht="22" customHeight="1">
       <c r="A536" s="2" t="inlineStr">
         <is>
-          <t>e15ce00dbe5c21b5</t>
+          <t>172a040b143ea0cf</t>
         </is>
       </c>
       <c r="B536" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 05:09</t>
+          <t>2026-10-19 17:27</t>
         </is>
       </c>
       <c r="C536" s="3" t="inlineStr">
         <is>
-          <t>Tecnólogo HSEQ / Seguridad y Salud en el Trabajo</t>
+          <t>Analista sst</t>
         </is>
       </c>
       <c r="D536" s="3" t="inlineStr">
         <is>
-          <t>Lighgen Ingeniería Ltda</t>
-        </is>
-      </c>
-      <c r="E536" s="8" t="n">
-        <v>0.48</v>
+          <t>Diseños y Aplicaciones de Ingeniería civil sas</t>
+        </is>
+      </c>
+      <c r="E536" s="7" t="n">
+        <v>0.5</v>
       </c>
       <c r="F536" s="2" t="inlineStr">
         <is>
@@ -25714,13 +25706,13 @@
         </is>
       </c>
       <c r="G536" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnologo-hseq-seguridad-y-salud-en-el-trabajo-con-experiencia-2-anos-en-bogota-dc-87DB3FCAFEA8E12861373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-sst-1886779165", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H536" s="6" t="inlineStr"/>
       <c r="I536" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J536" s="2" t="inlineStr">
@@ -25733,26 +25725,26 @@
     <row r="537" ht="22" customHeight="1">
       <c r="A537" s="2" t="inlineStr">
         <is>
-          <t>1f3bf8b16a58f0b4</t>
+          <t>718395b7e6fbf0fd</t>
         </is>
       </c>
       <c r="B537" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 05:09</t>
+          <t>2026-10-19 17:27</t>
         </is>
       </c>
       <c r="C537" s="3" t="inlineStr">
         <is>
-          <t>Inspector (a) de vias y urbanismo</t>
+          <t>Lider calidad y sst</t>
         </is>
       </c>
       <c r="D537" s="3" t="inlineStr">
         <is>
-          <t>METRO LINEA 1 S.A.S.</t>
-        </is>
-      </c>
-      <c r="E537" s="8" t="n">
-        <v>0.48</v>
+          <t>Confidencial</t>
+        </is>
+      </c>
+      <c r="E537" s="7" t="n">
+        <v>0.5</v>
       </c>
       <c r="F537" s="2" t="inlineStr">
         <is>
@@ -25760,13 +25752,13 @@
         </is>
       </c>
       <c r="G537" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/inspector-a-de-vias-y-urbanismo-1886728733", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/lider-calidad-y-sst-1886780115", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H537" s="6" t="inlineStr"/>
       <c r="I537" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia técnica en infraestructura vial, diseño geométrico y pavimentos. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J537" s="2" t="inlineStr">
@@ -25779,26 +25771,26 @@
     <row r="538" ht="22" customHeight="1">
       <c r="A538" s="2" t="inlineStr">
         <is>
-          <t>8fd843a922654d9e</t>
+          <t>c7d5298917a12bd3</t>
         </is>
       </c>
       <c r="B538" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 05:09</t>
+          <t>2026-10-19 17:27</t>
         </is>
       </c>
       <c r="C538" s="3" t="inlineStr">
         <is>
-          <t>Oficial de obra</t>
+          <t>Analista SST</t>
         </is>
       </c>
       <c r="D538" s="3" t="inlineStr">
         <is>
-          <t>TERMOTECNICA COINDUSTRIAL SAS</t>
-        </is>
-      </c>
-      <c r="E538" s="8" t="n">
-        <v>0.48</v>
+          <t>Grupo Núcleos de Madera</t>
+        </is>
+      </c>
+      <c r="E538" s="7" t="n">
+        <v>0.5</v>
       </c>
       <c r="F538" s="2" t="inlineStr">
         <is>
@@ -25806,13 +25798,13 @@
         </is>
       </c>
       <c r="G538" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/oficial-de-obra-puentevias-1886766237", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/analista-sst-at-grupo-n%C3%BAcleos-de-madera-4480993859", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H538" s="6" t="inlineStr"/>
       <c r="I538" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia técnica en infraestructura vial, diseño geométrico y pavimentos. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J538" s="2" t="inlineStr">
@@ -25825,26 +25817,26 @@
     <row r="539" ht="22" customHeight="1">
       <c r="A539" s="2" t="inlineStr">
         <is>
-          <t>03eab73111095faa</t>
+          <t>4a81f35509c76a9b</t>
         </is>
       </c>
       <c r="B539" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 05:09</t>
+          <t>2026-10-19 17:27</t>
         </is>
       </c>
       <c r="C539" s="3" t="inlineStr">
         <is>
-          <t>Residente estructuras</t>
+          <t>LIDER HSE</t>
         </is>
       </c>
       <c r="D539" s="3" t="inlineStr">
         <is>
-          <t>CONCONCRETO S.A.</t>
-        </is>
-      </c>
-      <c r="E539" s="8" t="n">
-        <v>0.48</v>
+          <t>Atento</t>
+        </is>
+      </c>
+      <c r="E539" s="7" t="n">
+        <v>0.5</v>
       </c>
       <c r="F539" s="2" t="inlineStr">
         <is>
@@ -25852,13 +25844,13 @@
         </is>
       </c>
       <c r="G539" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/residente-estructuras-experiencia-en-infraestructura-vial-y-talud-1886757305", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/lider-hse-at-atento-4478228863", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H539" s="6" t="inlineStr"/>
       <c r="I539" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia técnica en infraestructura vial, diseño geométrico y pavimentos. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J539" s="2" t="inlineStr">
@@ -25871,26 +25863,26 @@
     <row r="540" ht="22" customHeight="1">
       <c r="A540" s="2" t="inlineStr">
         <is>
-          <t>c5911c7562546e3c</t>
+          <t>ee66cc010a275e08</t>
         </is>
       </c>
       <c r="B540" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22 05:09</t>
+          <t>2026-10-19 17:27</t>
         </is>
       </c>
       <c r="C540" s="3" t="inlineStr">
         <is>
-          <t>Profesional con experiencia en el sector de transporte marítimo y/o por vías navegables</t>
+          <t>Senior Civil Engineer</t>
         </is>
       </c>
       <c r="D540" s="3" t="inlineStr">
         <is>
-          <t>ICONTEC</t>
-        </is>
-      </c>
-      <c r="E540" s="8" t="n">
-        <v>0.48</v>
+          <t>WSP Chile y Argentina</t>
+        </is>
+      </c>
+      <c r="E540" s="7" t="n">
+        <v>0.5</v>
       </c>
       <c r="F540" s="2" t="inlineStr">
         <is>
@@ -25898,13 +25890,13 @@
         </is>
       </c>
       <c r="G540" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/profesional-con-experiencia-en-el-sector-de-transporte-maritimo-y-o-por-vias-navegables-1886761682", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/senior-civil-engineer-at-wsp-chile-y-argentina-4480250388", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H540" s="6" t="inlineStr"/>
       <c r="I540" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia técnica en infraestructura vial, diseño geométrico y pavimentos. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 50/100 - Afinidad Moderada] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J540" s="2" t="inlineStr">
@@ -25917,7 +25909,7 @@
     <row r="541" ht="22" customHeight="1">
       <c r="A541" s="2" t="inlineStr">
         <is>
-          <t>c2903e245a44de39</t>
+          <t>4426b2c17306f519</t>
         </is>
       </c>
       <c r="B541" s="2" t="inlineStr">
@@ -25927,12 +25919,12 @@
       </c>
       <c r="C541" s="3" t="inlineStr">
         <is>
-          <t>Encargado de obra</t>
+          <t>Residente de Seguridad y Salud en el trabajo</t>
         </is>
       </c>
       <c r="D541" s="3" t="inlineStr">
         <is>
-          <t>TERMOTECNICA COINDUSTRIAL SAS</t>
+          <t>Cal y Mayor y Asociados S.C</t>
         </is>
       </c>
       <c r="E541" s="8" t="n">
@@ -25944,13 +25936,17 @@
         </is>
       </c>
       <c r="G541" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/encargado-de-obra-puentes-vias-1886762620", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H541" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-residente-de-seguridad-y-salud-en-el-trabajo-sst-sst-en-bogota-dc-D67E64C3D53E0D6961373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H541" s="6" t="inlineStr">
+        <is>
+          <t>$ 4.200.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I541" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia técnica en infraestructura vial, diseño geométrico y pavimentos. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J541" s="2" t="inlineStr">
@@ -25963,7 +25959,7 @@
     <row r="542" ht="22" customHeight="1">
       <c r="A542" s="2" t="inlineStr">
         <is>
-          <t>a5bd833e8b837d34</t>
+          <t>83015d6afb890f1d</t>
         </is>
       </c>
       <c r="B542" s="2" t="inlineStr">
@@ -25973,12 +25969,12 @@
       </c>
       <c r="C542" s="3" t="inlineStr">
         <is>
-          <t>Residente en seguridad y salud en el trabajo</t>
+          <t>Analista/profesional HSEQ / SST Sesquile o Alrededores</t>
         </is>
       </c>
       <c r="D542" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>ACTIVOS S A S</t>
         </is>
       </c>
       <c r="E542" s="8" t="n">
@@ -25990,10 +25986,14 @@
         </is>
       </c>
       <c r="G542" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/residente-en-seguridad-y-salud-en-el-trabajo-sst-1886762728", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H542" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-analistaprofesional-hseq-sst-sesquile-o-alrededores-sector-consumo-masivo-en-sesquile-632A9566338A59E361373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H542" s="6" t="inlineStr">
+        <is>
+          <t>$ 4.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I542" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -26009,7 +26009,7 @@
     <row r="543" ht="22" customHeight="1">
       <c r="A543" s="2" t="inlineStr">
         <is>
-          <t>55e7967f3b4afa02</t>
+          <t>bc0b38b5129e0905</t>
         </is>
       </c>
       <c r="B543" s="2" t="inlineStr">
@@ -26019,12 +26019,12 @@
       </c>
       <c r="C543" s="3" t="inlineStr">
         <is>
-          <t>Tecnólogo/a en Seguridad y Salud en el Trabajo</t>
+          <t>Profesional en seguridad y salud en el trabajo SST</t>
         </is>
       </c>
       <c r="D543" s="3" t="inlineStr">
         <is>
-          <t>EOSOL</t>
+          <t>Seguridad y Vigilancia Exito de Colombia</t>
         </is>
       </c>
       <c r="E543" s="8" t="n">
@@ -26036,10 +26036,14 @@
         </is>
       </c>
       <c r="G543" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/tecn%C3%B3logo-a-en-seguridad-y-salud-en-el-trabajo-sst-at-eosol-4464868638", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H543" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-profesional-en-seguridad-y-salud-en-el-trabajo-sst-con-experiencia-y-conocimiento-en-pesv-en-bogota-dc-A7CA6F8805D1C53B61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H543" s="6" t="inlineStr">
+        <is>
+          <t>$ 3.200.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I543" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -26055,7 +26059,7 @@
     <row r="544" ht="22" customHeight="1">
       <c r="A544" s="2" t="inlineStr">
         <is>
-          <t>6df905e482fe09b1</t>
+          <t>e15ce00dbe5c21b5</t>
         </is>
       </c>
       <c r="B544" s="2" t="inlineStr">
@@ -26065,12 +26069,12 @@
       </c>
       <c r="C544" s="3" t="inlineStr">
         <is>
-          <t>Aprendiz SENA - Técnico(a) de Salud Ocupacional o Seguridad y Salud en el Trabajo - Ginebra</t>
+          <t>Tecnólogo HSEQ / Seguridad y Salud en el Trabajo</t>
         </is>
       </c>
       <c r="D544" s="3" t="inlineStr">
         <is>
-          <t>Cargill</t>
+          <t>Lighgen Ingeniería Ltda</t>
         </is>
       </c>
       <c r="E544" s="8" t="n">
@@ -26082,7 +26086,7 @@
         </is>
       </c>
       <c r="G544" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/aprendiz-sena-t%C3%A9cnico-a-de-salud-ocupacional-o-seguridad-y-salud-en-el-trabajo-ginebra-at-cargill-4466994159", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnologo-hseq-seguridad-y-salud-en-el-trabajo-con-experiencia-2-anos-en-bogota-dc-87DB3FCAFEA8E12861373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H544" s="6" t="inlineStr"/>
@@ -26101,7 +26105,7 @@
     <row r="545" ht="22" customHeight="1">
       <c r="A545" s="2" t="inlineStr">
         <is>
-          <t>06656fbb2d452086</t>
+          <t>1f3bf8b16a58f0b4</t>
         </is>
       </c>
       <c r="B545" s="2" t="inlineStr">
@@ -26111,12 +26115,12 @@
       </c>
       <c r="C545" s="3" t="inlineStr">
         <is>
-          <t>Residente de Seguridad y Salud en el trabajo</t>
+          <t>Inspector (a) de vias y urbanismo</t>
         </is>
       </c>
       <c r="D545" s="3" t="inlineStr">
         <is>
-          <t>Grupo Cal y Mayor</t>
+          <t>METRO LINEA 1 S.A.S.</t>
         </is>
       </c>
       <c r="E545" s="8" t="n">
@@ -26128,13 +26132,13 @@
         </is>
       </c>
       <c r="G545" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/residente-de-seguridad-y-salud-en-el-trabajo-sst-at-cal-y-mayor-4468610572", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/inspector-a-de-vias-y-urbanismo-1886728733", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H545" s="6" t="inlineStr"/>
       <c r="I545" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia técnica en infraestructura vial, diseño geométrico y pavimentos. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J545" s="2" t="inlineStr">
@@ -26147,7 +26151,7 @@
     <row r="546" ht="22" customHeight="1">
       <c r="A546" s="2" t="inlineStr">
         <is>
-          <t>7796e088dce85b5a</t>
+          <t>8fd843a922654d9e</t>
         </is>
       </c>
       <c r="B546" s="2" t="inlineStr">
@@ -26157,16 +26161,16 @@
       </c>
       <c r="C546" s="3" t="inlineStr">
         <is>
-          <t>Civil Engineer (Fire Sprinkler Design))</t>
+          <t>Oficial de obra</t>
         </is>
       </c>
       <c r="D546" s="3" t="inlineStr">
         <is>
-          <t>Hyremote</t>
+          <t>TERMOTECNICA COINDUSTRIAL SAS</t>
         </is>
       </c>
       <c r="E546" s="8" t="n">
-        <v>0.45</v>
+        <v>0.48</v>
       </c>
       <c r="F546" s="2" t="inlineStr">
         <is>
@@ -26174,17 +26178,13 @@
         </is>
       </c>
       <c r="G546" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-civil-engineer-fire-sprinkler-design-english-c1-remote-en-bogota-dc-A2EE61A321FC0D3361373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H546" s="6" t="inlineStr">
-        <is>
-          <t>$ 4.499.993,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/oficial-de-obra-puentevias-1886766237", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H546" s="6" t="inlineStr"/>
       <c r="I546" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia técnica en infraestructura vial, diseño geométrico y pavimentos. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J546" s="2" t="inlineStr">
@@ -26197,7 +26197,7 @@
     <row r="547" ht="22" customHeight="1">
       <c r="A547" s="2" t="inlineStr">
         <is>
-          <t>48463526ca7c8ada</t>
+          <t>03eab73111095faa</t>
         </is>
       </c>
       <c r="B547" s="2" t="inlineStr">
@@ -26207,16 +26207,16 @@
       </c>
       <c r="C547" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero Civil Especialista en Hidrología e Hidráulica</t>
+          <t>Residente estructuras</t>
         </is>
       </c>
       <c r="D547" s="3" t="inlineStr">
         <is>
-          <t>ATLAS INFRASTRUCTURE DESIGN LIMITED</t>
+          <t>CONCONCRETO S.A.</t>
         </is>
       </c>
       <c r="E547" s="8" t="n">
-        <v>0.45</v>
+        <v>0.48</v>
       </c>
       <c r="F547" s="2" t="inlineStr">
         <is>
@@ -26224,17 +26224,13 @@
         </is>
       </c>
       <c r="G547" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingeniero-civil-especialista-en-hidrologia-e-hidraulica-tiempo-completo-en-remoto-y-de-larga-duracion-en-colombia-027FB718364F4C7761373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H547" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/residente-estructuras-experiencia-en-infraestructura-vial-y-talud-1886757305", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H547" s="6" t="inlineStr"/>
       <c r="I547" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia técnica en infraestructura vial, diseño geométrico y pavimentos. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J547" s="2" t="inlineStr">
@@ -26247,7 +26243,7 @@
     <row r="548" ht="22" customHeight="1">
       <c r="A548" s="2" t="inlineStr">
         <is>
-          <t>2d406567ceb21bf8</t>
+          <t>c5911c7562546e3c</t>
         </is>
       </c>
       <c r="B548" s="2" t="inlineStr">
@@ -26257,16 +26253,16 @@
       </c>
       <c r="C548" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero Civil de Diseño</t>
+          <t>Profesional con experiencia en el sector de transporte marítimo y/o por vías navegables</t>
         </is>
       </c>
       <c r="D548" s="3" t="inlineStr">
         <is>
-          <t>ATLAS INFRASTRUCTURE DESIGN LIMITED</t>
+          <t>ICONTEC</t>
         </is>
       </c>
       <c r="E548" s="8" t="n">
-        <v>0.45</v>
+        <v>0.48</v>
       </c>
       <c r="F548" s="2" t="inlineStr">
         <is>
@@ -26274,17 +26270,13 @@
         </is>
       </c>
       <c r="G548" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingeniero-civil-de-diseno-tiempo-completo-en-remoto-en-colombia-4CB8F30B6D8FBF7261373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H548" s="6" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/profesional-con-experiencia-en-el-sector-de-transporte-maritimo-y-o-por-vias-navegables-1886761682", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H548" s="6" t="inlineStr"/>
       <c r="I548" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia técnica en infraestructura vial, diseño geométrico y pavimentos. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J548" s="2" t="inlineStr">
@@ -26297,7 +26289,7 @@
     <row r="549" ht="22" customHeight="1">
       <c r="A549" s="2" t="inlineStr">
         <is>
-          <t>4d4013d19591d2a5</t>
+          <t>c2903e245a44de39</t>
         </is>
       </c>
       <c r="B549" s="2" t="inlineStr">
@@ -26307,16 +26299,16 @@
       </c>
       <c r="C549" s="3" t="inlineStr">
         <is>
-          <t>Especialista en Salud y Seguridad en el trabajo con especialización en medio Ambiente</t>
+          <t>Encargado de obra</t>
         </is>
       </c>
       <c r="D549" s="3" t="inlineStr">
         <is>
-          <t>DEXTERA S.A.S</t>
+          <t>TERMOTECNICA COINDUSTRIAL SAS</t>
         </is>
       </c>
       <c r="E549" s="8" t="n">
-        <v>0.45</v>
+        <v>0.48</v>
       </c>
       <c r="F549" s="2" t="inlineStr">
         <is>
@@ -26324,13 +26316,13 @@
         </is>
       </c>
       <c r="G549" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-especialista-en-salud-y-seguridad-en-el-trabajo-con-especializacion-en-medio-ambiente-en-bogota-dc-68C95C2F64D6648561373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/encargado-de-obra-puentes-vias-1886762620", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H549" s="6" t="inlineStr"/>
       <c r="I549" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia técnica en infraestructura vial, diseño geométrico y pavimentos. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J549" s="2" t="inlineStr">
@@ -26343,7 +26335,7 @@
     <row r="550" ht="22" customHeight="1">
       <c r="A550" s="2" t="inlineStr">
         <is>
-          <t>cf70d2ca6e5c25de</t>
+          <t>a5bd833e8b837d34</t>
         </is>
       </c>
       <c r="B550" s="2" t="inlineStr">
@@ -26353,16 +26345,16 @@
       </c>
       <c r="C550" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero civil</t>
+          <t>Residente en seguridad y salud en el trabajo</t>
         </is>
       </c>
       <c r="D550" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E550" s="8" t="n">
-        <v>0.45</v>
+        <v>0.48</v>
       </c>
       <c r="F550" s="2" t="inlineStr">
         <is>
@@ -26370,17 +26362,13 @@
         </is>
       </c>
       <c r="G550" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingeniero-civil-con-experiencia-en-sistemas-fotovoltaicos-en-bogota-dc-8BCBCD7DF8FE589C61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H550" s="6" t="inlineStr">
-        <is>
-          <t>$ 3.300.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/residente-en-seguridad-y-salud-en-el-trabajo-sst-1886762728", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H550" s="6" t="inlineStr"/>
       <c r="I550" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J550" s="2" t="inlineStr">
@@ -26393,7 +26381,7 @@
     <row r="551" ht="22" customHeight="1">
       <c r="A551" s="2" t="inlineStr">
         <is>
-          <t>bb8237cc7ed8d56b</t>
+          <t>55e7967f3b4afa02</t>
         </is>
       </c>
       <c r="B551" s="2" t="inlineStr">
@@ -26403,16 +26391,16 @@
       </c>
       <c r="C551" s="3" t="inlineStr">
         <is>
-          <t>Coordinador de Proyectos Mejoramientos de Vivienda</t>
+          <t>Tecnólogo/a en Seguridad y Salud en el Trabajo</t>
         </is>
       </c>
       <c r="D551" s="3" t="inlineStr">
         <is>
-          <t>Socya</t>
+          <t>EOSOL</t>
         </is>
       </c>
       <c r="E551" s="8" t="n">
-        <v>0.45</v>
+        <v>0.48</v>
       </c>
       <c r="F551" s="2" t="inlineStr">
         <is>
@@ -26420,13 +26408,13 @@
         </is>
       </c>
       <c r="G551" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-coordinador-de-proyectos-mejoramientos-de-vivienda-medellin-antioquia-en-medellin-7E29781CFFD4058961373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/tecn%C3%B3logo-a-en-seguridad-y-salud-en-el-trabajo-sst-at-eosol-4464868638", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H551" s="6" t="inlineStr"/>
       <c r="I551" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J551" s="2" t="inlineStr">
@@ -26439,7 +26427,7 @@
     <row r="552" ht="22" customHeight="1">
       <c r="A552" s="2" t="inlineStr">
         <is>
-          <t>c41dc091e876cb10</t>
+          <t>6df905e482fe09b1</t>
         </is>
       </c>
       <c r="B552" s="2" t="inlineStr">
@@ -26449,16 +26437,16 @@
       </c>
       <c r="C552" s="3" t="inlineStr">
         <is>
-          <t>Especialista de Milk Collection</t>
+          <t>Aprendiz SENA - Técnico(a) de Salud Ocupacional o Seguridad y Salud en el Trabajo - Ginebra</t>
         </is>
       </c>
       <c r="D552" s="3" t="inlineStr">
         <is>
-          <t>LACTALIS</t>
+          <t>Cargill</t>
         </is>
       </c>
       <c r="E552" s="8" t="n">
-        <v>0.45</v>
+        <v>0.48</v>
       </c>
       <c r="F552" s="2" t="inlineStr">
         <is>
@@ -26466,17 +26454,13 @@
         </is>
       </c>
       <c r="G552" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-especialista-de-milk-collection-optimizacion-y-analisis-de-datos-en-bogota-dc-B007F5172FEA6F6461373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H552" s="6" t="inlineStr">
-        <is>
-          <t>$ 6.000.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/aprendiz-sena-t%C3%A9cnico-a-de-salud-ocupacional-o-seguridad-y-salud-en-el-trabajo-ginebra-at-cargill-4466994159", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H552" s="6" t="inlineStr"/>
       <c r="I552" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J552" s="2" t="inlineStr">
@@ -26489,7 +26473,7 @@
     <row r="553" ht="22" customHeight="1">
       <c r="A553" s="2" t="inlineStr">
         <is>
-          <t>4f38d6c20430e4bb</t>
+          <t>06656fbb2d452086</t>
         </is>
       </c>
       <c r="B553" s="2" t="inlineStr">
@@ -26499,16 +26483,16 @@
       </c>
       <c r="C553" s="3" t="inlineStr">
         <is>
-          <t>ingeniero civil</t>
+          <t>Residente de Seguridad y Salud en el trabajo</t>
         </is>
       </c>
       <c r="D553" s="3" t="inlineStr">
         <is>
-          <t>EVALTEC S.A.S.</t>
+          <t>Grupo Cal y Mayor</t>
         </is>
       </c>
       <c r="E553" s="8" t="n">
-        <v>0.45</v>
+        <v>0.48</v>
       </c>
       <c r="F553" s="2" t="inlineStr">
         <is>
@@ -26516,13 +26500,13 @@
         </is>
       </c>
       <c r="G553" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingeniero-civil-o-areas-afines-en-medellin-0E02F682AB12631061373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/residente-de-seguridad-y-salud-en-el-trabajo-sst-at-cal-y-mayor-4468610572", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H553" s="6" t="inlineStr"/>
       <c r="I553" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 48/100 - Baja Afinidad] Alta coincidencia en gestión de Seguridad y Salud en el Trabajo (SST). Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J553" s="2" t="inlineStr">
@@ -26535,7 +26519,7 @@
     <row r="554" ht="22" customHeight="1">
       <c r="A554" s="2" t="inlineStr">
         <is>
-          <t>af38dd28fbbad8f4</t>
+          <t>7796e088dce85b5a</t>
         </is>
       </c>
       <c r="B554" s="2" t="inlineStr">
@@ -26545,12 +26529,12 @@
       </c>
       <c r="C554" s="3" t="inlineStr">
         <is>
-          <t>Tecnólogo Auxiliar Civil</t>
+          <t>Civil Engineer (Fire Sprinkler Design))</t>
         </is>
       </c>
       <c r="D554" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>Hyremote</t>
         </is>
       </c>
       <c r="E554" s="8" t="n">
@@ -26562,10 +26546,14 @@
         </is>
       </c>
       <c r="G554" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnologo-auxiliar-civil-antioquia-en-liborina-B380460DDA9F98D061373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H554" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-civil-engineer-fire-sprinkler-design-english-c1-remote-en-bogota-dc-A2EE61A321FC0D3361373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H554" s="6" t="inlineStr">
+        <is>
+          <t>$ 4.499.993,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I554" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -26581,7 +26569,7 @@
     <row r="555" ht="22" customHeight="1">
       <c r="A555" s="2" t="inlineStr">
         <is>
-          <t>19e74768ce848880</t>
+          <t>48463526ca7c8ada</t>
         </is>
       </c>
       <c r="B555" s="2" t="inlineStr">
@@ -26591,12 +26579,12 @@
       </c>
       <c r="C555" s="3" t="inlineStr">
         <is>
-          <t>Coordinador HSEQ</t>
+          <t>Ingeniero Civil Especialista en Hidrología e Hidráulica</t>
         </is>
       </c>
       <c r="D555" s="3" t="inlineStr">
         <is>
-          <t>Agencia de empleo de Comfenalco Cartagena</t>
+          <t>ATLAS INFRASTRUCTURE DESIGN LIMITED</t>
         </is>
       </c>
       <c r="E555" s="8" t="n">
@@ -26608,17 +26596,17 @@
         </is>
       </c>
       <c r="G555" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-coordinador-hseq-especialista-en-seguridad-y-salud-en-el-trabajo-salud-ocupacional-en-cartagena-de-indias-1EAF6570FC054C2661373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingeniero-civil-especialista-en-hidrologia-e-hidraulica-tiempo-completo-en-remoto-y-de-larga-duracion-en-colombia-027FB718364F4C7761373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H555" s="6" t="inlineStr">
         <is>
-          <t>$ 2.500.000,00 (Mensual)</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="I555" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J555" s="2" t="inlineStr">
@@ -26631,7 +26619,7 @@
     <row r="556" ht="22" customHeight="1">
       <c r="A556" s="2" t="inlineStr">
         <is>
-          <t>38c9a9481706de58</t>
+          <t>2d406567ceb21bf8</t>
         </is>
       </c>
       <c r="B556" s="2" t="inlineStr">
@@ -26641,12 +26629,12 @@
       </c>
       <c r="C556" s="3" t="inlineStr">
         <is>
-          <t>Coordinador de seguridad vial y monitoreo</t>
+          <t>Ingeniero Civil de Diseño</t>
         </is>
       </c>
       <c r="D556" s="3" t="inlineStr">
         <is>
-          <t>MEGACOMERCIAL S.A.S</t>
+          <t>ATLAS INFRASTRUCTURE DESIGN LIMITED</t>
         </is>
       </c>
       <c r="E556" s="8" t="n">
@@ -26658,17 +26646,17 @@
         </is>
       </c>
       <c r="G556" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-coordinador-de-seguridad-vial-y-monitoreo-abierto-a-nivel-nacional-en-bogota-dc-B9B593A780889F2A61373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingeniero-civil-de-diseno-tiempo-completo-en-remoto-en-colombia-4CB8F30B6D8FBF7261373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H556" s="6" t="inlineStr">
         <is>
-          <t>$ 5.000.000,00 (Mensual)</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="I556" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en infraestructura vial y transporte. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J556" s="2" t="inlineStr">
@@ -26681,7 +26669,7 @@
     <row r="557" ht="22" customHeight="1">
       <c r="A557" s="2" t="inlineStr">
         <is>
-          <t>aecc6c18fdd71383</t>
+          <t>4d4013d19591d2a5</t>
         </is>
       </c>
       <c r="B557" s="2" t="inlineStr">
@@ -26691,12 +26679,12 @@
       </c>
       <c r="C557" s="3" t="inlineStr">
         <is>
-          <t>Coordinador de PESV</t>
+          <t>Especialista en Salud y Seguridad en el trabajo con especialización en medio Ambiente</t>
         </is>
       </c>
       <c r="D557" s="3" t="inlineStr">
         <is>
-          <t>Agencia de Empleo de Comfenalco Antioquia</t>
+          <t>DEXTERA S.A.S</t>
         </is>
       </c>
       <c r="E557" s="8" t="n">
@@ -26708,17 +26696,13 @@
         </is>
       </c>
       <c r="G557" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-coordinador-de-pesv-en-medellin-67C3B78E9A85885161373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H557" s="6" t="inlineStr">
-        <is>
-          <t>$ 2.800.000,00 (Mensual)</t>
-        </is>
-      </c>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-especialista-en-salud-y-seguridad-en-el-trabajo-con-especializacion-en-medio-ambiente-en-bogota-dc-68C95C2F64D6648561373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H557" s="6" t="inlineStr"/>
       <c r="I557" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en infraestructura vial y transporte. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J557" s="2" t="inlineStr">
@@ -26731,7 +26715,7 @@
     <row r="558" ht="22" customHeight="1">
       <c r="A558" s="2" t="inlineStr">
         <is>
-          <t>1558fc20863bdd35</t>
+          <t>cf70d2ca6e5c25de</t>
         </is>
       </c>
       <c r="B558" s="2" t="inlineStr">
@@ -26741,12 +26725,12 @@
       </c>
       <c r="C558" s="3" t="inlineStr">
         <is>
-          <t>Coordinador HSEQ</t>
+          <t>Ingeniero civil</t>
         </is>
       </c>
       <c r="D558" s="3" t="inlineStr">
         <is>
-          <t>COMPAÑIA DE INGENIEROS CONSTRUCTORES S.A.S.</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E558" s="8" t="n">
@@ -26758,13 +26742,17 @@
         </is>
       </c>
       <c r="G558" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-coordinador-hseq-en-barranquilla-F4898EBB71CAF3ED61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H558" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingeniero-civil-con-experiencia-en-sistemas-fotovoltaicos-en-bogota-dc-8BCBCD7DF8FE589C61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H558" s="6" t="inlineStr">
+        <is>
+          <t>$ 3.300.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I558" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J558" s="2" t="inlineStr">
@@ -26777,7 +26765,7 @@
     <row r="559" ht="22" customHeight="1">
       <c r="A559" s="2" t="inlineStr">
         <is>
-          <t>0bf63022dc93885b</t>
+          <t>bb8237cc7ed8d56b</t>
         </is>
       </c>
       <c r="B559" s="2" t="inlineStr">
@@ -26787,12 +26775,12 @@
       </c>
       <c r="C559" s="3" t="inlineStr">
         <is>
-          <t>ingeniero civil</t>
+          <t>Coordinador de Proyectos Mejoramientos de Vivienda</t>
         </is>
       </c>
       <c r="D559" s="3" t="inlineStr">
         <is>
-          <t>FRANCISCO ANGULO M INGENIEROS S.A.S.</t>
+          <t>Socya</t>
         </is>
       </c>
       <c r="E559" s="8" t="n">
@@ -26804,7 +26792,7 @@
         </is>
       </c>
       <c r="G559" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingeniero-civil-residente-de-interventoria-yo-supervision-tecnica-en-cali-D2AE78FA9B23778161373E686DCF3405", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-coordinador-de-proyectos-mejoramientos-de-vivienda-medellin-antioquia-en-medellin-7E29781CFFD4058961373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H559" s="6" t="inlineStr"/>
@@ -26823,7 +26811,7 @@
     <row r="560" ht="22" customHeight="1">
       <c r="A560" s="2" t="inlineStr">
         <is>
-          <t>baa61a6e15a2de77</t>
+          <t>c41dc091e876cb10</t>
         </is>
       </c>
       <c r="B560" s="2" t="inlineStr">
@@ -26833,12 +26821,12 @@
       </c>
       <c r="C560" s="3" t="inlineStr">
         <is>
-          <t>Arquitecto(a) / Ingeniero(a) Civil</t>
+          <t>Especialista de Milk Collection</t>
         </is>
       </c>
       <c r="D560" s="3" t="inlineStr">
         <is>
-          <t>Importante empresa del sector</t>
+          <t>LACTALIS</t>
         </is>
       </c>
       <c r="E560" s="8" t="n">
@@ -26850,10 +26838,14 @@
         </is>
       </c>
       <c r="G560" s="5">
-        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-arquitectoa-ingenieroa-civil-en-bucaramanga-8D15AF34F304555F61373E686DCF3405", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H560" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-especialista-de-milk-collection-optimizacion-y-analisis-de-datos-en-bogota-dc-B007F5172FEA6F6461373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H560" s="6" t="inlineStr">
+        <is>
+          <t>$ 6.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I560" s="3" t="inlineStr">
         <is>
           <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
@@ -26869,7 +26861,7 @@
     <row r="561" ht="22" customHeight="1">
       <c r="A561" s="2" t="inlineStr">
         <is>
-          <t>448d93b15d9b7dec</t>
+          <t>4f38d6c20430e4bb</t>
         </is>
       </c>
       <c r="B561" s="2" t="inlineStr">
@@ -26879,12 +26871,12 @@
       </c>
       <c r="C561" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero especialista fortinet</t>
+          <t>ingeniero civil</t>
         </is>
       </c>
       <c r="D561" s="3" t="inlineStr">
         <is>
-          <t>ATCG DE COLOMBIA S.A.S</t>
+          <t>EVALTEC S.A.S.</t>
         </is>
       </c>
       <c r="E561" s="8" t="n">
@@ -26896,7 +26888,7 @@
         </is>
       </c>
       <c r="G561" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-especialista-fortinet-1886742914", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingeniero-civil-o-areas-afines-en-medellin-0E02F682AB12631061373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H561" s="6" t="inlineStr"/>
@@ -26915,7 +26907,7 @@
     <row r="562" ht="22" customHeight="1">
       <c r="A562" s="2" t="inlineStr">
         <is>
-          <t>f2fc6f9471f81665</t>
+          <t>af38dd28fbbad8f4</t>
         </is>
       </c>
       <c r="B562" s="2" t="inlineStr">
@@ -26925,12 +26917,12 @@
       </c>
       <c r="C562" s="3" t="inlineStr">
         <is>
-          <t>Coordinador/a nacional de redes e infraestructura de ti - presencial bucaramanga</t>
+          <t>Tecnólogo Auxiliar Civil</t>
         </is>
       </c>
       <c r="D562" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E562" s="8" t="n">
@@ -26942,13 +26934,13 @@
         </is>
       </c>
       <c r="G562" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-a-nacional-de-redes-e-infraestructura-de-ti-presencial-bucaramanga-1886769481", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-tecnologo-auxiliar-civil-antioquia-en-liborina-B380460DDA9F98D061373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H562" s="6" t="inlineStr"/>
       <c r="I562" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en infraestructura vial y transporte. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J562" s="2" t="inlineStr">
@@ -26961,7 +26953,7 @@
     <row r="563" ht="22" customHeight="1">
       <c r="A563" s="2" t="inlineStr">
         <is>
-          <t>53e1a775996a36c5</t>
+          <t>19e74768ce848880</t>
         </is>
       </c>
       <c r="B563" s="2" t="inlineStr">
@@ -26971,12 +26963,12 @@
       </c>
       <c r="C563" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero civil</t>
+          <t>Coordinador HSEQ</t>
         </is>
       </c>
       <c r="D563" s="3" t="inlineStr">
         <is>
-          <t>Proyectos de Diseño y Construccion sas</t>
+          <t>Agencia de empleo de Comfenalco Cartagena</t>
         </is>
       </c>
       <c r="E563" s="8" t="n">
@@ -26988,13 +26980,17 @@
         </is>
       </c>
       <c r="G563" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-civil-1886757049", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H563" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-coordinador-hseq-especialista-en-seguridad-y-salud-en-el-trabajo-salud-ocupacional-en-cartagena-de-indias-1EAF6570FC054C2661373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H563" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.500.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I563" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J563" s="2" t="inlineStr">
@@ -27007,7 +27003,7 @@
     <row r="564" ht="22" customHeight="1">
       <c r="A564" s="2" t="inlineStr">
         <is>
-          <t>1072d76e2f18ea50</t>
+          <t>38c9a9481706de58</t>
         </is>
       </c>
       <c r="B564" s="2" t="inlineStr">
@@ -27017,12 +27013,12 @@
       </c>
       <c r="C564" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero civil</t>
+          <t>Coordinador de seguridad vial y monitoreo</t>
         </is>
       </c>
       <c r="D564" s="3" t="inlineStr">
         <is>
-          <t>R2P SOLUCIONES Y CONSTRUCCIONES SAS</t>
+          <t>MEGACOMERCIAL S.A.S</t>
         </is>
       </c>
       <c r="E564" s="8" t="n">
@@ -27034,13 +27030,17 @@
         </is>
       </c>
       <c r="G564" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-civil-1886758475", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H564" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-coordinador-de-seguridad-vial-y-monitoreo-abierto-a-nivel-nacional-en-bogota-dc-B9B593A780889F2A61373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H564" s="6" t="inlineStr">
+        <is>
+          <t>$ 5.000.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I564" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en infraestructura vial y transporte. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J564" s="2" t="inlineStr">
@@ -27053,7 +27053,7 @@
     <row r="565" ht="22" customHeight="1">
       <c r="A565" s="2" t="inlineStr">
         <is>
-          <t>2c943591cc334f5a</t>
+          <t>aecc6c18fdd71383</t>
         </is>
       </c>
       <c r="B565" s="2" t="inlineStr">
@@ -27063,12 +27063,12 @@
       </c>
       <c r="C565" s="3" t="inlineStr">
         <is>
-          <t>Ejecutivo/ade ingeniera</t>
+          <t>Coordinador de PESV</t>
         </is>
       </c>
       <c r="D565" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Agencia de Empleo de Comfenalco Antioquia</t>
         </is>
       </c>
       <c r="E565" s="8" t="n">
@@ -27080,13 +27080,17 @@
         </is>
       </c>
       <c r="G565" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ejecutivo-ade-ingeniera-1886752134", "Ver Vacante")</f>
-        <v/>
-      </c>
-      <c r="H565" s="6" t="inlineStr"/>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-coordinador-de-pesv-en-medellin-67C3B78E9A85885161373E686DCF3405", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H565" s="6" t="inlineStr">
+        <is>
+          <t>$ 2.800.000,00 (Mensual)</t>
+        </is>
+      </c>
       <c r="I565" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en infraestructura vial y transporte. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J565" s="2" t="inlineStr">
@@ -27099,7 +27103,7 @@
     <row r="566" ht="22" customHeight="1">
       <c r="A566" s="2" t="inlineStr">
         <is>
-          <t>7d4067502e572780</t>
+          <t>1558fc20863bdd35</t>
         </is>
       </c>
       <c r="B566" s="2" t="inlineStr">
@@ -27109,12 +27113,12 @@
       </c>
       <c r="C566" s="3" t="inlineStr">
         <is>
-          <t>Ingeniera de ventas - cali</t>
+          <t>Coordinador HSEQ</t>
         </is>
       </c>
       <c r="D566" s="3" t="inlineStr">
         <is>
-          <t>PIPOL EXPERT SAS</t>
+          <t>COMPAÑIA DE INGENIEROS CONSTRUCTORES S.A.S.</t>
         </is>
       </c>
       <c r="E566" s="8" t="n">
@@ -27126,13 +27130,13 @@
         </is>
       </c>
       <c r="G566" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniera-de-ventas-cali-1886754430", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-coordinador-hseq-en-barranquilla-F4898EBB71CAF3ED61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H566" s="6" t="inlineStr"/>
       <c r="I566" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J566" s="2" t="inlineStr">
@@ -27145,7 +27149,7 @@
     <row r="567" ht="22" customHeight="1">
       <c r="A567" s="2" t="inlineStr">
         <is>
-          <t>a3a688084650de1c</t>
+          <t>0bf63022dc93885b</t>
         </is>
       </c>
       <c r="B567" s="2" t="inlineStr">
@@ -27155,12 +27159,12 @@
       </c>
       <c r="C567" s="3" t="inlineStr">
         <is>
-          <t>Ingeniera comercial electrica - cali</t>
+          <t>ingeniero civil</t>
         </is>
       </c>
       <c r="D567" s="3" t="inlineStr">
         <is>
-          <t>PIPOL EXPERT SAS</t>
+          <t>FRANCISCO ANGULO M INGENIEROS S.A.S.</t>
         </is>
       </c>
       <c r="E567" s="8" t="n">
@@ -27172,7 +27176,7 @@
         </is>
       </c>
       <c r="G567" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniera-comercial-electrica-cali-1886752104", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-ingeniero-civil-residente-de-interventoria-yo-supervision-tecnica-en-cali-D2AE78FA9B23778161373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H567" s="6" t="inlineStr"/>
@@ -27191,7 +27195,7 @@
     <row r="568" ht="22" customHeight="1">
       <c r="A568" s="2" t="inlineStr">
         <is>
-          <t>359d47915a2e74e6</t>
+          <t>baa61a6e15a2de77</t>
         </is>
       </c>
       <c r="B568" s="2" t="inlineStr">
@@ -27201,12 +27205,12 @@
       </c>
       <c r="C568" s="3" t="inlineStr">
         <is>
-          <t>Supervisor civil - obra</t>
+          <t>Arquitecto(a) / Ingeniero(a) Civil</t>
         </is>
       </c>
       <c r="D568" s="3" t="inlineStr">
         <is>
-          <t>CONCONCRETO S.A.</t>
+          <t>Importante empresa del sector</t>
         </is>
       </c>
       <c r="E568" s="8" t="n">
@@ -27218,7 +27222,7 @@
         </is>
       </c>
       <c r="G568" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/supervisor-civil-obra-1886750435", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.computrabajo.com/ofertas-de-trabajo/oferta-de-trabajo-de-arquitectoa-ingenieroa-civil-en-bucaramanga-8D15AF34F304555F61373E686DCF3405", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H568" s="6" t="inlineStr"/>
@@ -27237,7 +27241,7 @@
     <row r="569" ht="22" customHeight="1">
       <c r="A569" s="2" t="inlineStr">
         <is>
-          <t>78244d2897084f6a</t>
+          <t>448d93b15d9b7dec</t>
         </is>
       </c>
       <c r="B569" s="2" t="inlineStr">
@@ -27247,12 +27251,12 @@
       </c>
       <c r="C569" s="3" t="inlineStr">
         <is>
-          <t>Ingeniera comercial sector industrial - cali</t>
+          <t>Ingeniero especialista fortinet</t>
         </is>
       </c>
       <c r="D569" s="3" t="inlineStr">
         <is>
-          <t>PIPOL EXPERT SAS</t>
+          <t>ATCG DE COLOMBIA S.A.S</t>
         </is>
       </c>
       <c r="E569" s="8" t="n">
@@ -27264,7 +27268,7 @@
         </is>
       </c>
       <c r="G569" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniera-comercial-sector-industrial-cali-1886753949", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-especialista-fortinet-1886742914", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H569" s="6" t="inlineStr"/>
@@ -27283,7 +27287,7 @@
     <row r="570" ht="22" customHeight="1">
       <c r="A570" s="2" t="inlineStr">
         <is>
-          <t>a4d1239b8910f7cf</t>
+          <t>f2fc6f9471f81665</t>
         </is>
       </c>
       <c r="B570" s="2" t="inlineStr">
@@ -27293,12 +27297,12 @@
       </c>
       <c r="C570" s="3" t="inlineStr">
         <is>
-          <t>Ingeniera electrica comercial - bogotá</t>
+          <t>Coordinador/a nacional de redes e infraestructura de ti - presencial bucaramanga</t>
         </is>
       </c>
       <c r="D570" s="3" t="inlineStr">
         <is>
-          <t>PIPOL EXPERT SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E570" s="8" t="n">
@@ -27310,13 +27314,13 @@
         </is>
       </c>
       <c r="G570" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniera-electrica-comercial-bogota-1886756984", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-a-nacional-de-redes-e-infraestructura-de-ti-presencial-bucaramanga-1886769481", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H570" s="6" t="inlineStr"/>
       <c r="I570" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en infraestructura vial y transporte. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J570" s="2" t="inlineStr">
@@ -27329,7 +27333,7 @@
     <row r="571" ht="22" customHeight="1">
       <c r="A571" s="2" t="inlineStr">
         <is>
-          <t>366f049dd1eaf173</t>
+          <t>53e1a775996a36c5</t>
         </is>
       </c>
       <c r="B571" s="2" t="inlineStr">
@@ -27339,12 +27343,12 @@
       </c>
       <c r="C571" s="3" t="inlineStr">
         <is>
-          <t>Civil engineering-in-training</t>
+          <t>Ingeniero civil</t>
         </is>
       </c>
       <c r="D571" s="3" t="inlineStr">
         <is>
-          <t>WSP COLOMBIA SAS</t>
+          <t>Proyectos de Diseño y Construccion sas</t>
         </is>
       </c>
       <c r="E571" s="8" t="n">
@@ -27356,7 +27360,7 @@
         </is>
       </c>
       <c r="G571" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/civil-engineeringintraining-1886759044", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-civil-1886757049", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H571" s="6" t="inlineStr"/>
@@ -27375,7 +27379,7 @@
     <row r="572" ht="22" customHeight="1">
       <c r="A572" s="2" t="inlineStr">
         <is>
-          <t>555a755e56fc6a80</t>
+          <t>1072d76e2f18ea50</t>
         </is>
       </c>
       <c r="B572" s="2" t="inlineStr">
@@ -27385,12 +27389,12 @@
       </c>
       <c r="C572" s="3" t="inlineStr">
         <is>
-          <t>Civil engineering-in-training</t>
+          <t>Ingeniero civil</t>
         </is>
       </c>
       <c r="D572" s="3" t="inlineStr">
         <is>
-          <t>WSP COLOMBIA SAS</t>
+          <t>R2P SOLUCIONES Y CONSTRUCCIONES SAS</t>
         </is>
       </c>
       <c r="E572" s="8" t="n">
@@ -27402,7 +27406,7 @@
         </is>
       </c>
       <c r="G572" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/civil-engineeringintraining-1886758755", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-civil-1886758475", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H572" s="6" t="inlineStr"/>
@@ -27421,7 +27425,7 @@
     <row r="573" ht="22" customHeight="1">
       <c r="A573" s="2" t="inlineStr">
         <is>
-          <t>776483d4ec602e40</t>
+          <t>2c943591cc334f5a</t>
         </is>
       </c>
       <c r="B573" s="2" t="inlineStr">
@@ -27431,12 +27435,12 @@
       </c>
       <c r="C573" s="3" t="inlineStr">
         <is>
-          <t>Consultor senior sap pm - remoto colombia</t>
+          <t>Ejecutivo/ade ingeniera</t>
         </is>
       </c>
       <c r="D573" s="3" t="inlineStr">
         <is>
-          <t>TALYCAP GLOBAL SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E573" s="8" t="n">
@@ -27448,7 +27452,7 @@
         </is>
       </c>
       <c r="G573" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-senior-sap-pm-remoto-colombia-1886747903", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ejecutivo-ade-ingeniera-1886752134", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H573" s="6" t="inlineStr"/>
@@ -27467,7 +27471,7 @@
     <row r="574" ht="22" customHeight="1">
       <c r="A574" s="2" t="inlineStr">
         <is>
-          <t>b1cfe269bbc00011</t>
+          <t>7d4067502e572780</t>
         </is>
       </c>
       <c r="B574" s="2" t="inlineStr">
@@ -27477,12 +27481,12 @@
       </c>
       <c r="C574" s="3" t="inlineStr">
         <is>
-          <t>Coordinador de interventoría</t>
+          <t>Ingeniera de ventas - cali</t>
         </is>
       </c>
       <c r="D574" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>PIPOL EXPERT SAS</t>
         </is>
       </c>
       <c r="E574" s="8" t="n">
@@ -27494,7 +27498,7 @@
         </is>
       </c>
       <c r="G574" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-de-interventoria-1886751671", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniera-de-ventas-cali-1886754430", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H574" s="6" t="inlineStr"/>
@@ -27513,7 +27517,7 @@
     <row r="575" ht="22" customHeight="1">
       <c r="A575" s="2" t="inlineStr">
         <is>
-          <t>b7a3423e1ee1e624</t>
+          <t>a3a688084650de1c</t>
         </is>
       </c>
       <c r="B575" s="2" t="inlineStr">
@@ -27523,12 +27527,12 @@
       </c>
       <c r="C575" s="3" t="inlineStr">
         <is>
-          <t>Especialista en urbanismo - proyecto vial</t>
+          <t>Ingeniera comercial electrica - cali</t>
         </is>
       </c>
       <c r="D575" s="3" t="inlineStr">
         <is>
-          <t>INGEPLAN.CO SAS EMPRESA DE BENEFICIO E INTERES COLECTIVO BIC</t>
+          <t>PIPOL EXPERT SAS</t>
         </is>
       </c>
       <c r="E575" s="8" t="n">
@@ -27540,7 +27544,7 @@
         </is>
       </c>
       <c r="G575" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-urbanismo-proyecto-vial-1886755827", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniera-comercial-electrica-cali-1886752104", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H575" s="6" t="inlineStr"/>
@@ -27559,7 +27563,7 @@
     <row r="576" ht="22" customHeight="1">
       <c r="A576" s="2" t="inlineStr">
         <is>
-          <t>fcb39d755657052e</t>
+          <t>359d47915a2e74e6</t>
         </is>
       </c>
       <c r="B576" s="2" t="inlineStr">
@@ -27569,12 +27573,12 @@
       </c>
       <c r="C576" s="3" t="inlineStr">
         <is>
-          <t>Coordinador hseq</t>
+          <t>Supervisor civil - obra</t>
         </is>
       </c>
       <c r="D576" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>CONCONCRETO S.A.</t>
         </is>
       </c>
       <c r="E576" s="8" t="n">
@@ -27586,13 +27590,13 @@
         </is>
       </c>
       <c r="G576" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-hseq-1886747304", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/supervisor-civil-obra-1886750435", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H576" s="6" t="inlineStr"/>
       <c r="I576" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J576" s="2" t="inlineStr">
@@ -27605,7 +27609,7 @@
     <row r="577" ht="22" customHeight="1">
       <c r="A577" s="2" t="inlineStr">
         <is>
-          <t>9e2f0c16f1a50983</t>
+          <t>78244d2897084f6a</t>
         </is>
       </c>
       <c r="B577" s="2" t="inlineStr">
@@ -27615,12 +27619,12 @@
       </c>
       <c r="C577" s="3" t="inlineStr">
         <is>
-          <t>Coordinador hseq</t>
+          <t>Ingeniera comercial sector industrial - cali</t>
         </is>
       </c>
       <c r="D577" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>PIPOL EXPERT SAS</t>
         </is>
       </c>
       <c r="E577" s="8" t="n">
@@ -27632,13 +27636,13 @@
         </is>
       </c>
       <c r="G577" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-hseq-1886764155", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniera-comercial-sector-industrial-cali-1886753949", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H577" s="6" t="inlineStr"/>
       <c r="I577" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J577" s="2" t="inlineStr">
@@ -27651,7 +27655,7 @@
     <row r="578" ht="22" customHeight="1">
       <c r="A578" s="2" t="inlineStr">
         <is>
-          <t>9d4d87a631d5e8b8</t>
+          <t>a4d1239b8910f7cf</t>
         </is>
       </c>
       <c r="B578" s="2" t="inlineStr">
@@ -27661,12 +27665,12 @@
       </c>
       <c r="C578" s="3" t="inlineStr">
         <is>
-          <t>Coordinador hseq</t>
+          <t>Ingeniera electrica comercial - bogotá</t>
         </is>
       </c>
       <c r="D578" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>PIPOL EXPERT SAS</t>
         </is>
       </c>
       <c r="E578" s="8" t="n">
@@ -27678,13 +27682,13 @@
         </is>
       </c>
       <c r="G578" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-hseq-1886760733", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniera-electrica-comercial-bogota-1886756984", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H578" s="6" t="inlineStr"/>
       <c r="I578" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J578" s="2" t="inlineStr">
@@ -27697,7 +27701,7 @@
     <row r="579" ht="22" customHeight="1">
       <c r="A579" s="2" t="inlineStr">
         <is>
-          <t>62d6690ef260f268</t>
+          <t>366f049dd1eaf173</t>
         </is>
       </c>
       <c r="B579" s="2" t="inlineStr">
@@ -27707,12 +27711,12 @@
       </c>
       <c r="C579" s="3" t="inlineStr">
         <is>
-          <t>Coordinador hseq cartagena</t>
+          <t>Civil engineering-in-training</t>
         </is>
       </c>
       <c r="D579" s="3" t="inlineStr">
         <is>
-          <t>APPLUS NORCONTROL COLOMBIA LTDA</t>
+          <t>WSP COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E579" s="8" t="n">
@@ -27724,13 +27728,13 @@
         </is>
       </c>
       <c r="G579" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-hseq-cartagena-1886754661", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/civil-engineeringintraining-1886759044", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H579" s="6" t="inlineStr"/>
       <c r="I579" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J579" s="2" t="inlineStr">
@@ -27743,7 +27747,7 @@
     <row r="580" ht="22" customHeight="1">
       <c r="A580" s="2" t="inlineStr">
         <is>
-          <t>6e57e2acbfc11d12</t>
+          <t>555a755e56fc6a80</t>
         </is>
       </c>
       <c r="B580" s="2" t="inlineStr">
@@ -27753,12 +27757,12 @@
       </c>
       <c r="C580" s="3" t="inlineStr">
         <is>
-          <t>Especialista sig</t>
+          <t>Civil engineering-in-training</t>
         </is>
       </c>
       <c r="D580" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>WSP COLOMBIA SAS</t>
         </is>
       </c>
       <c r="E580" s="8" t="n">
@@ -27770,7 +27774,7 @@
         </is>
       </c>
       <c r="G580" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-sig-1886757094", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/civil-engineeringintraining-1886758755", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H580" s="6" t="inlineStr"/>
@@ -27789,7 +27793,7 @@
     <row r="581" ht="22" customHeight="1">
       <c r="A581" s="2" t="inlineStr">
         <is>
-          <t>11494a184e6f9290</t>
+          <t>776483d4ec602e40</t>
         </is>
       </c>
       <c r="B581" s="2" t="inlineStr">
@@ -27799,12 +27803,12 @@
       </c>
       <c r="C581" s="3" t="inlineStr">
         <is>
-          <t>Especialista en ingeniería civil - coordinador técnico</t>
+          <t>Consultor senior sap pm - remoto colombia</t>
         </is>
       </c>
       <c r="D581" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>TALYCAP GLOBAL SAS</t>
         </is>
       </c>
       <c r="E581" s="8" t="n">
@@ -27816,7 +27820,7 @@
         </is>
       </c>
       <c r="G581" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-ingenieria-civil-coordinador-tecnico-honduras-1886745304", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/consultor-senior-sap-pm-remoto-colombia-1886747903", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H581" s="6" t="inlineStr"/>
@@ -27835,7 +27839,7 @@
     <row r="582" ht="22" customHeight="1">
       <c r="A582" s="2" t="inlineStr">
         <is>
-          <t>327c6d2b54619849</t>
+          <t>b1cfe269bbc00011</t>
         </is>
       </c>
       <c r="B582" s="2" t="inlineStr">
@@ -27845,7 +27849,7 @@
       </c>
       <c r="C582" s="3" t="inlineStr">
         <is>
-          <t>Especialista en psiquiatría</t>
+          <t>Coordinador de interventoría</t>
         </is>
       </c>
       <c r="D582" s="3" t="inlineStr">
@@ -27862,7 +27866,7 @@
         </is>
       </c>
       <c r="G582" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-psiquiatria-1886757353", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-de-interventoria-1886751671", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H582" s="6" t="inlineStr"/>
@@ -27881,7 +27885,7 @@
     <row r="583" ht="22" customHeight="1">
       <c r="A583" s="2" t="inlineStr">
         <is>
-          <t>b637f33f588eb5ae</t>
+          <t>b7a3423e1ee1e624</t>
         </is>
       </c>
       <c r="B583" s="2" t="inlineStr">
@@ -27891,12 +27895,12 @@
       </c>
       <c r="C583" s="3" t="inlineStr">
         <is>
-          <t>Especialista en diseño hospitalario</t>
+          <t>Especialista en urbanismo - proyecto vial</t>
         </is>
       </c>
       <c r="D583" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>INGEPLAN.CO SAS EMPRESA DE BENEFICIO E INTERES COLECTIVO BIC</t>
         </is>
       </c>
       <c r="E583" s="8" t="n">
@@ -27908,7 +27912,7 @@
         </is>
       </c>
       <c r="G583" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-diseno-hospitalario-disponibilidad-viajar-a-peru-1886747220", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-urbanismo-proyecto-vial-1886755827", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H583" s="6" t="inlineStr"/>
@@ -27927,7 +27931,7 @@
     <row r="584" ht="22" customHeight="1">
       <c r="A584" s="2" t="inlineStr">
         <is>
-          <t>adcc2b47284b5d4d</t>
+          <t>fcb39d755657052e</t>
         </is>
       </c>
       <c r="B584" s="2" t="inlineStr">
@@ -27937,12 +27941,12 @@
       </c>
       <c r="C584" s="3" t="inlineStr">
         <is>
-          <t>Analista de diseño e ingeniería de empaque - sector farmaceutico</t>
+          <t>Coordinador hseq</t>
         </is>
       </c>
       <c r="D584" s="3" t="inlineStr">
         <is>
-          <t>LABORATORIOS BUSSIE</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E584" s="8" t="n">
@@ -27954,13 +27958,13 @@
         </is>
       </c>
       <c r="G584" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-diseno-e-ingenieria-de-empaque-sector-farmaceutico-1886755492", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-hseq-1886747304", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H584" s="6" t="inlineStr"/>
       <c r="I584" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J584" s="2" t="inlineStr">
@@ -27973,7 +27977,7 @@
     <row r="585" ht="22" customHeight="1">
       <c r="A585" s="2" t="inlineStr">
         <is>
-          <t>3ec3d2d34753ff04</t>
+          <t>9e2f0c16f1a50983</t>
         </is>
       </c>
       <c r="B585" s="2" t="inlineStr">
@@ -27983,12 +27987,12 @@
       </c>
       <c r="C585" s="3" t="inlineStr">
         <is>
-          <t>Especialista de diseño y arquitectura</t>
+          <t>Coordinador hseq</t>
         </is>
       </c>
       <c r="D585" s="3" t="inlineStr">
         <is>
-          <t>INTER RAPIDISIMO</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E585" s="8" t="n">
@@ -28000,13 +28004,13 @@
         </is>
       </c>
       <c r="G585" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-de-diseno-y-arquitectura-1886761909", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-hseq-1886764155", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H585" s="6" t="inlineStr"/>
       <c r="I585" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J585" s="2" t="inlineStr">
@@ -28019,7 +28023,7 @@
     <row r="586" ht="22" customHeight="1">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>4e917305e90b3efa</t>
+          <t>9d4d87a631d5e8b8</t>
         </is>
       </c>
       <c r="B586" s="2" t="inlineStr">
@@ -28029,12 +28033,12 @@
       </c>
       <c r="C586" s="3" t="inlineStr">
         <is>
-          <t>Especialista en geología</t>
+          <t>Coordinador hseq</t>
         </is>
       </c>
       <c r="D586" s="3" t="inlineStr">
         <is>
-          <t>INGEPLAN.CO SAS EMPRESA DE BENEFICIO E INTERES COLECTIVO BIC</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E586" s="8" t="n">
@@ -28046,13 +28050,13 @@
         </is>
       </c>
       <c r="G586" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-geologia-1886761263", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-hseq-1886760733", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H586" s="6" t="inlineStr"/>
       <c r="I586" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J586" s="2" t="inlineStr">
@@ -28065,7 +28069,7 @@
     <row r="587" ht="22" customHeight="1">
       <c r="A587" s="2" t="inlineStr">
         <is>
-          <t>1aef5476d70bbe42</t>
+          <t>62d6690ef260f268</t>
         </is>
       </c>
       <c r="B587" s="2" t="inlineStr">
@@ -28075,12 +28079,12 @@
       </c>
       <c r="C587" s="3" t="inlineStr">
         <is>
-          <t>Especialista en geología</t>
+          <t>Coordinador hseq cartagena</t>
         </is>
       </c>
       <c r="D587" s="3" t="inlineStr">
         <is>
-          <t>INGEPLAN.CO SAS EMPRESA DE BENEFICIO E INTERES COLECTIVO BIC</t>
+          <t>APPLUS NORCONTROL COLOMBIA LTDA</t>
         </is>
       </c>
       <c r="E587" s="8" t="n">
@@ -28092,13 +28096,13 @@
         </is>
       </c>
       <c r="G587" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-geologia-1886755729", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-hseq-cartagena-1886754661", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H587" s="6" t="inlineStr"/>
       <c r="I587" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J587" s="2" t="inlineStr">
@@ -28111,7 +28115,7 @@
     <row r="588" ht="22" customHeight="1">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>b46df3b678599255</t>
+          <t>6e57e2acbfc11d12</t>
         </is>
       </c>
       <c r="B588" s="2" t="inlineStr">
@@ -28121,7 +28125,7 @@
       </c>
       <c r="C588" s="3" t="inlineStr">
         <is>
-          <t>Especialista en estructuras</t>
+          <t>Especialista sig</t>
         </is>
       </c>
       <c r="D588" s="3" t="inlineStr">
@@ -28138,7 +28142,7 @@
         </is>
       </c>
       <c r="G588" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-estructuras-1886757080", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-sig-1886757094", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H588" s="6" t="inlineStr"/>
@@ -28157,7 +28161,7 @@
     <row r="589" ht="22" customHeight="1">
       <c r="A589" s="2" t="inlineStr">
         <is>
-          <t>935035bdfa2ae0b7</t>
+          <t>11494a184e6f9290</t>
         </is>
       </c>
       <c r="B589" s="2" t="inlineStr">
@@ -28167,12 +28171,12 @@
       </c>
       <c r="C589" s="3" t="inlineStr">
         <is>
-          <t>Especialista en gestión del riesgo</t>
+          <t>Especialista en ingeniería civil - coordinador técnico</t>
         </is>
       </c>
       <c r="D589" s="3" t="inlineStr">
         <is>
-          <t>INGEPLAN.CO SAS EMPRESA DE BENEFICIO E INTERES COLECTIVO BIC</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E589" s="8" t="n">
@@ -28184,7 +28188,7 @@
         </is>
       </c>
       <c r="G589" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-gestion-del-riesgo-1886755709", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-ingenieria-civil-coordinador-tecnico-honduras-1886745304", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H589" s="6" t="inlineStr"/>
@@ -28203,7 +28207,7 @@
     <row r="590" ht="22" customHeight="1">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>14a1c964238340ba</t>
+          <t>327c6d2b54619849</t>
         </is>
       </c>
       <c r="B590" s="2" t="inlineStr">
@@ -28213,7 +28217,7 @@
       </c>
       <c r="C590" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero civil nivel v</t>
+          <t>Especialista en psiquiatría</t>
         </is>
       </c>
       <c r="D590" s="3" t="inlineStr">
@@ -28230,7 +28234,7 @@
         </is>
       </c>
       <c r="G590" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-civil-nivel-v-1886758046", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-psiquiatria-1886757353", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H590" s="6" t="inlineStr"/>
@@ -28249,7 +28253,7 @@
     <row r="591" ht="22" customHeight="1">
       <c r="A591" s="2" t="inlineStr">
         <is>
-          <t>740f61bdbaa69d0e</t>
+          <t>b637f33f588eb5ae</t>
         </is>
       </c>
       <c r="B591" s="2" t="inlineStr">
@@ -28259,12 +28263,12 @@
       </c>
       <c r="C591" s="3" t="inlineStr">
         <is>
-          <t>Coordinador de proyectos bilingüe</t>
+          <t>Especialista en diseño hospitalario</t>
         </is>
       </c>
       <c r="D591" s="3" t="inlineStr">
         <is>
-          <t>EyS IT SAS</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E591" s="8" t="n">
@@ -28276,7 +28280,7 @@
         </is>
       </c>
       <c r="G591" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-de-proyectos-bilingue-1886749343", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-diseno-hospitalario-disponibilidad-viajar-a-peru-1886747220", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H591" s="6" t="inlineStr"/>
@@ -28295,7 +28299,7 @@
     <row r="592" ht="22" customHeight="1">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>63ef229552018ccd</t>
+          <t>adcc2b47284b5d4d</t>
         </is>
       </c>
       <c r="B592" s="2" t="inlineStr">
@@ -28305,12 +28309,12 @@
       </c>
       <c r="C592" s="3" t="inlineStr">
         <is>
-          <t>Coordinador de proyectos</t>
+          <t>Analista de diseño e ingeniería de empaque - sector farmaceutico</t>
         </is>
       </c>
       <c r="D592" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>LABORATORIOS BUSSIE</t>
         </is>
       </c>
       <c r="E592" s="8" t="n">
@@ -28322,7 +28326,7 @@
         </is>
       </c>
       <c r="G592" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-de-proyectos-1886748647", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/analista-de-diseno-e-ingenieria-de-empaque-sector-farmaceutico-1886755492", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H592" s="6" t="inlineStr"/>
@@ -28341,7 +28345,7 @@
     <row r="593" ht="22" customHeight="1">
       <c r="A593" s="2" t="inlineStr">
         <is>
-          <t>03750e25a7e1c016</t>
+          <t>3ec3d2d34753ff04</t>
         </is>
       </c>
       <c r="B593" s="2" t="inlineStr">
@@ -28351,12 +28355,12 @@
       </c>
       <c r="C593" s="3" t="inlineStr">
         <is>
-          <t>Coordinador de proyectos inmobiliarios</t>
+          <t>Especialista de diseño y arquitectura</t>
         </is>
       </c>
       <c r="D593" s="3" t="inlineStr">
         <is>
-          <t>GRUPO AR S.A.</t>
+          <t>INTER RAPIDISIMO</t>
         </is>
       </c>
       <c r="E593" s="8" t="n">
@@ -28368,7 +28372,7 @@
         </is>
       </c>
       <c r="G593" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-de-proyectos-inmobiliarios-1886745877", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-de-diseno-y-arquitectura-1886761909", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H593" s="6" t="inlineStr"/>
@@ -28387,7 +28391,7 @@
     <row r="594" ht="22" customHeight="1">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>5627e52731a73f27</t>
+          <t>4e917305e90b3efa</t>
         </is>
       </c>
       <c r="B594" s="2" t="inlineStr">
@@ -28397,12 +28401,12 @@
       </c>
       <c r="C594" s="3" t="inlineStr">
         <is>
-          <t>Coordinador de proyectos inmobiliarios</t>
+          <t>Especialista en geología</t>
         </is>
       </c>
       <c r="D594" s="3" t="inlineStr">
         <is>
-          <t>GRUPO AR S.A.</t>
+          <t>INGEPLAN.CO SAS EMPRESA DE BENEFICIO E INTERES COLECTIVO BIC</t>
         </is>
       </c>
       <c r="E594" s="8" t="n">
@@ -28414,7 +28418,7 @@
         </is>
       </c>
       <c r="G594" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-de-proyectos-inmobiliarios-1886704948", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-geologia-1886761263", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H594" s="6" t="inlineStr"/>
@@ -28433,7 +28437,7 @@
     <row r="595" ht="22" customHeight="1">
       <c r="A595" s="2" t="inlineStr">
         <is>
-          <t>b6af0024900baff6</t>
+          <t>1aef5476d70bbe42</t>
         </is>
       </c>
       <c r="B595" s="2" t="inlineStr">
@@ -28443,12 +28447,12 @@
       </c>
       <c r="C595" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero residente - ingeniero civil-cordoba</t>
+          <t>Especialista en geología</t>
         </is>
       </c>
       <c r="D595" s="3" t="inlineStr">
         <is>
-          <t>OBCIPOL SAS</t>
+          <t>INGEPLAN.CO SAS EMPRESA DE BENEFICIO E INTERES COLECTIVO BIC</t>
         </is>
       </c>
       <c r="E595" s="8" t="n">
@@ -28460,7 +28464,7 @@
         </is>
       </c>
       <c r="G595" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-residente-ingeniero-civilcordoba-1886763488", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-geologia-1886755729", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H595" s="6" t="inlineStr"/>
@@ -28479,7 +28483,7 @@
     <row r="596" ht="22" customHeight="1">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>2a0453695fa88728</t>
+          <t>b46df3b678599255</t>
         </is>
       </c>
       <c r="B596" s="2" t="inlineStr">
@@ -28489,12 +28493,12 @@
       </c>
       <c r="C596" s="3" t="inlineStr">
         <is>
-          <t>Profesional ingenieria mecanica</t>
+          <t>Especialista en estructuras</t>
         </is>
       </c>
       <c r="D596" s="3" t="inlineStr">
         <is>
-          <t>INZIGNIA CONSTRUCTION S.A</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E596" s="8" t="n">
@@ -28506,7 +28510,7 @@
         </is>
       </c>
       <c r="G596" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/profesional-ingenieria-mecanica-1886767282", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-estructuras-1886757080", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H596" s="6" t="inlineStr"/>
@@ -28525,7 +28529,7 @@
     <row r="597" ht="22" customHeight="1">
       <c r="A597" s="2" t="inlineStr">
         <is>
-          <t>edfe98c543194667</t>
+          <t>935035bdfa2ae0b7</t>
         </is>
       </c>
       <c r="B597" s="2" t="inlineStr">
@@ -28535,12 +28539,12 @@
       </c>
       <c r="C597" s="3" t="inlineStr">
         <is>
-          <t>Jefe de sst - nemocón - 1625991634-135</t>
+          <t>Especialista en gestión del riesgo</t>
         </is>
       </c>
       <c r="D597" s="3" t="inlineStr">
         <is>
-          <t>AGENCIA DE EMPLEO Y FOMENTO EMPRESARIAL COMPENSAR</t>
+          <t>INGEPLAN.CO SAS EMPRESA DE BENEFICIO E INTERES COLECTIVO BIC</t>
         </is>
       </c>
       <c r="E597" s="8" t="n">
@@ -28552,13 +28556,13 @@
         </is>
       </c>
       <c r="G597" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/jefe-de-sst-nemocon-1625991634135-1886754873", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/especialista-en-gestion-del-riesgo-1886755709", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H597" s="6" t="inlineStr"/>
       <c r="I597" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J597" s="2" t="inlineStr">
@@ -28571,7 +28575,7 @@
     <row r="598" ht="22" customHeight="1">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>6233e93ceb1dbeed</t>
+          <t>14a1c964238340ba</t>
         </is>
       </c>
       <c r="B598" s="2" t="inlineStr">
@@ -28581,7 +28585,7 @@
       </c>
       <c r="C598" s="3" t="inlineStr">
         <is>
-          <t>Jefe de sst- nemocón</t>
+          <t>Ingeniero civil nivel v</t>
         </is>
       </c>
       <c r="D598" s="3" t="inlineStr">
@@ -28598,13 +28602,13 @@
         </is>
       </c>
       <c r="G598" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/jefe-de-sst-nemocon-1886757757", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-civil-nivel-v-1886758046", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H598" s="6" t="inlineStr"/>
       <c r="I598" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J598" s="2" t="inlineStr">
@@ -28617,7 +28621,7 @@
     <row r="599" ht="22" customHeight="1">
       <c r="A599" s="2" t="inlineStr">
         <is>
-          <t>ce75aab7a32f36a3</t>
+          <t>740f61bdbaa69d0e</t>
         </is>
       </c>
       <c r="B599" s="2" t="inlineStr">
@@ -28627,12 +28631,12 @@
       </c>
       <c r="C599" s="3" t="inlineStr">
         <is>
-          <t>Coordinador talento humano y sst - bogota- 1626427532-7</t>
+          <t>Coordinador de proyectos bilingüe</t>
         </is>
       </c>
       <c r="D599" s="3" t="inlineStr">
         <is>
-          <t>AGENCIA DE EMPLEO Y FOMENTO EMPRESARIAL COMPENSAR</t>
+          <t>EyS IT SAS</t>
         </is>
       </c>
       <c r="E599" s="8" t="n">
@@ -28644,13 +28648,13 @@
         </is>
       </c>
       <c r="G599" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-talento-humano-y-sst-bogota-16264275327-1886753531", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-de-proyectos-bilingue-1886749343", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H599" s="6" t="inlineStr"/>
       <c r="I599" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J599" s="2" t="inlineStr">
@@ -28663,7 +28667,7 @@
     <row r="600" ht="22" customHeight="1">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>850731f7bb6cd73f</t>
+          <t>63ef229552018ccd</t>
         </is>
       </c>
       <c r="B600" s="2" t="inlineStr">
@@ -28673,12 +28677,12 @@
       </c>
       <c r="C600" s="3" t="inlineStr">
         <is>
-          <t>Coordinador(a) de sst y medio ambiente</t>
+          <t>Coordinador de proyectos</t>
         </is>
       </c>
       <c r="D600" s="3" t="inlineStr">
         <is>
-          <t>ATIEMPO S.A.S</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E600" s="8" t="n">
@@ -28690,13 +28694,13 @@
         </is>
       </c>
       <c r="G600" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinadora-de-sst-y-medio-ambiente-1886759848", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-de-proyectos-1886748647", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H600" s="6" t="inlineStr"/>
       <c r="I600" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J600" s="2" t="inlineStr">
@@ -28709,7 +28713,7 @@
     <row r="601" ht="22" customHeight="1">
       <c r="A601" s="2" t="inlineStr">
         <is>
-          <t>abaf8e513787b3f3</t>
+          <t>03750e25a7e1c016</t>
         </is>
       </c>
       <c r="B601" s="2" t="inlineStr">
@@ -28719,12 +28723,12 @@
       </c>
       <c r="C601" s="3" t="inlineStr">
         <is>
-          <t>Coordinador pesv</t>
+          <t>Coordinador de proyectos inmobiliarios</t>
         </is>
       </c>
       <c r="D601" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>GRUPO AR S.A.</t>
         </is>
       </c>
       <c r="E601" s="8" t="n">
@@ -28736,13 +28740,13 @@
         </is>
       </c>
       <c r="G601" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-pesv-1886769643", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-de-proyectos-inmobiliarios-1886745877", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H601" s="6" t="inlineStr"/>
       <c r="I601" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en infraestructura vial y transporte. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J601" s="2" t="inlineStr">
@@ -28755,7 +28759,7 @@
     <row r="602" ht="22" customHeight="1">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>9dcdf501e5912b88</t>
+          <t>5627e52731a73f27</t>
         </is>
       </c>
       <c r="B602" s="2" t="inlineStr">
@@ -28765,12 +28769,12 @@
       </c>
       <c r="C602" s="3" t="inlineStr">
         <is>
-          <t>Tecnico de obras civiles /girardot ref. 339166-82241</t>
+          <t>Coordinador de proyectos inmobiliarios</t>
         </is>
       </c>
       <c r="D602" s="3" t="inlineStr">
         <is>
-          <t>AGENCIA DE EMPLEO Y FOMENTO EMPRESARIAL COMPENSAR</t>
+          <t>GRUPO AR S.A.</t>
         </is>
       </c>
       <c r="E602" s="8" t="n">
@@ -28782,7 +28786,7 @@
         </is>
       </c>
       <c r="G602" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-obras-civiles-girardot-ref-33916682241-1886747302", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-de-proyectos-inmobiliarios-1886704948", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H602" s="6" t="inlineStr"/>
@@ -28801,7 +28805,7 @@
     <row r="603" ht="22" customHeight="1">
       <c r="A603" s="2" t="inlineStr">
         <is>
-          <t>693b8a076a888f67</t>
+          <t>b6af0024900baff6</t>
         </is>
       </c>
       <c r="B603" s="2" t="inlineStr">
@@ -28811,12 +28815,12 @@
       </c>
       <c r="C603" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero civil - especializacion en estructuras</t>
+          <t>Ingeniero residente - ingeniero civil-cordoba</t>
         </is>
       </c>
       <c r="D603" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>OBCIPOL SAS</t>
         </is>
       </c>
       <c r="E603" s="8" t="n">
@@ -28828,7 +28832,7 @@
         </is>
       </c>
       <c r="G603" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-civil-especializacion-en-estructuras-1886766956", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-residente-ingeniero-civilcordoba-1886763488", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H603" s="6" t="inlineStr"/>
@@ -28847,7 +28851,7 @@
     <row r="604" ht="22" customHeight="1">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>13bc527565632878</t>
+          <t>2a0453695fa88728</t>
         </is>
       </c>
       <c r="B604" s="2" t="inlineStr">
@@ -28857,12 +28861,12 @@
       </c>
       <c r="C604" s="3" t="inlineStr">
         <is>
-          <t>Tecnico en contratacion de obra civil bogota</t>
+          <t>Profesional ingenieria mecanica</t>
         </is>
       </c>
       <c r="D604" s="3" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>INZIGNIA CONSTRUCTION S.A</t>
         </is>
       </c>
       <c r="E604" s="8" t="n">
@@ -28874,7 +28878,7 @@
         </is>
       </c>
       <c r="G604" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-en-contratacion-de-obra-civil-bogota-1886759693", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/profesional-ingenieria-mecanica-1886767282", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H604" s="6" t="inlineStr"/>
@@ -28893,7 +28897,7 @@
     <row r="605" ht="22" customHeight="1">
       <c r="A605" s="2" t="inlineStr">
         <is>
-          <t>6ccccd3a1ba05f7f</t>
+          <t>edfe98c543194667</t>
         </is>
       </c>
       <c r="B605" s="2" t="inlineStr">
@@ -28903,12 +28907,12 @@
       </c>
       <c r="C605" s="3" t="inlineStr">
         <is>
-          <t>14561-especialista interventoria-bogota</t>
+          <t>Jefe de sst - nemocón - 1625991634-135</t>
         </is>
       </c>
       <c r="D605" s="3" t="inlineStr">
         <is>
-          <t>APPLUS NORCONTROL COLOMBIA LTDA</t>
+          <t>AGENCIA DE EMPLEO Y FOMENTO EMPRESARIAL COMPENSAR</t>
         </is>
       </c>
       <c r="E605" s="8" t="n">
@@ -28920,13 +28924,13 @@
         </is>
       </c>
       <c r="G605" s="5">
-        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/14561especialista-interventoriabogota-1886768886", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/jefe-de-sst-nemocon-1625991634135-1886754873", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H605" s="6" t="inlineStr"/>
       <c r="I605" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J605" s="2" t="inlineStr">
@@ -28939,7 +28943,7 @@
     <row r="606" ht="22" customHeight="1">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>8ad0c11c4f07472e</t>
+          <t>6233e93ceb1dbeed</t>
         </is>
       </c>
       <c r="B606" s="2" t="inlineStr">
@@ -28949,12 +28953,12 @@
       </c>
       <c r="C606" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero Civil / Terracerías</t>
+          <t>Jefe de sst- nemocón</t>
         </is>
       </c>
       <c r="D606" s="3" t="inlineStr">
         <is>
-          <t>EOSOL</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E606" s="8" t="n">
@@ -28966,13 +28970,13 @@
         </is>
       </c>
       <c r="G606" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-civil-terracer%C3%ADas-at-eosol-4445793534", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/jefe-de-sst-nemocon-1886757757", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H606" s="6" t="inlineStr"/>
       <c r="I606" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J606" s="2" t="inlineStr">
@@ -28985,7 +28989,7 @@
     <row r="607" ht="22" customHeight="1">
       <c r="A607" s="2" t="inlineStr">
         <is>
-          <t>ed46085f88d06bf5</t>
+          <t>ce75aab7a32f36a3</t>
         </is>
       </c>
       <c r="B607" s="2" t="inlineStr">
@@ -28995,12 +28999,12 @@
       </c>
       <c r="C607" s="3" t="inlineStr">
         <is>
-          <t>Supervisor Civil</t>
+          <t>Coordinador talento humano y sst - bogota- 1626427532-7</t>
         </is>
       </c>
       <c r="D607" s="3" t="inlineStr">
         <is>
-          <t>EOSOL</t>
+          <t>AGENCIA DE EMPLEO Y FOMENTO EMPRESARIAL COMPENSAR</t>
         </is>
       </c>
       <c r="E607" s="8" t="n">
@@ -29012,13 +29016,13 @@
         </is>
       </c>
       <c r="G607" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/supervisor-civil-at-eosol-4442238964", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-talento-humano-y-sst-bogota-16264275327-1886753531", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H607" s="6" t="inlineStr"/>
       <c r="I607" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J607" s="2" t="inlineStr">
@@ -29031,7 +29035,7 @@
     <row r="608" ht="22" customHeight="1">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>dc949850c44ae2c9</t>
+          <t>850731f7bb6cd73f</t>
         </is>
       </c>
       <c r="B608" s="2" t="inlineStr">
@@ -29041,12 +29045,12 @@
       </c>
       <c r="C608" s="3" t="inlineStr">
         <is>
-          <t>Civil Engineer</t>
+          <t>Coordinador(a) de sst y medio ambiente</t>
         </is>
       </c>
       <c r="D608" s="3" t="inlineStr">
         <is>
-          <t>Cresta</t>
+          <t>ATIEMPO S.A.S</t>
         </is>
       </c>
       <c r="E608" s="8" t="n">
@@ -29058,13 +29062,13 @@
         </is>
       </c>
       <c r="G608" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-engineer-at-cresta-4465582487", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinadora-de-sst-y-medio-ambiente-1886759848", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H608" s="6" t="inlineStr"/>
       <c r="I608" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J608" s="2" t="inlineStr">
@@ -29077,7 +29081,7 @@
     <row r="609" ht="22" customHeight="1">
       <c r="A609" s="2" t="inlineStr">
         <is>
-          <t>4ad1a5acabdb8ad3</t>
+          <t>abaf8e513787b3f3</t>
         </is>
       </c>
       <c r="B609" s="2" t="inlineStr">
@@ -29087,12 +29091,12 @@
       </c>
       <c r="C609" s="3" t="inlineStr">
         <is>
-          <t>Civil BIM Specialist</t>
+          <t>Coordinador pesv</t>
         </is>
       </c>
       <c r="D609" s="3" t="inlineStr">
         <is>
-          <t>ENG</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E609" s="8" t="n">
@@ -29104,13 +29108,13 @@
         </is>
       </c>
       <c r="G609" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-bim-specialist-at-eng-4469886677", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/coordinador-pesv-1886769643", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H609" s="6" t="inlineStr"/>
       <c r="I609" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en infraestructura vial y transporte. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J609" s="2" t="inlineStr">
@@ -29123,7 +29127,7 @@
     <row r="610" ht="22" customHeight="1">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>5ebaba0a0c9927fb</t>
+          <t>9dcdf501e5912b88</t>
         </is>
       </c>
       <c r="B610" s="2" t="inlineStr">
@@ -29133,12 +29137,12 @@
       </c>
       <c r="C610" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero/a Civil-Estructuras Hormigón/Acero</t>
+          <t>Tecnico de obras civiles /girardot ref. 339166-82241</t>
         </is>
       </c>
       <c r="D610" s="3" t="inlineStr">
         <is>
-          <t>IDOM Consulting, Engineering, Architecture</t>
+          <t>AGENCIA DE EMPLEO Y FOMENTO EMPRESARIAL COMPENSAR</t>
         </is>
       </c>
       <c r="E610" s="8" t="n">
@@ -29150,7 +29154,7 @@
         </is>
       </c>
       <c r="G610" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-a-civil-estructuras-hormig%C3%B3n-acero-at-idom-consulting-engineering-architecture-4462998187", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-de-obras-civiles-girardot-ref-33916682241-1886747302", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H610" s="6" t="inlineStr"/>
@@ -29169,7 +29173,7 @@
     <row r="611" ht="22" customHeight="1">
       <c r="A611" s="2" t="inlineStr">
         <is>
-          <t>5c954c66c2c9d655</t>
+          <t>693b8a076a888f67</t>
         </is>
       </c>
       <c r="B611" s="2" t="inlineStr">
@@ -29179,12 +29183,12 @@
       </c>
       <c r="C611" s="3" t="inlineStr">
         <is>
-          <t>Civil Engineering-in-Training</t>
+          <t>Ingeniero civil - especializacion en estructuras</t>
         </is>
       </c>
       <c r="D611" s="3" t="inlineStr">
         <is>
-          <t>WSP en Colombia</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E611" s="8" t="n">
@@ -29196,7 +29200,7 @@
         </is>
       </c>
       <c r="G611" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-engineering-in-training-french-at-wsp-en-colombia-4458430104", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/ingeniero-civil-especializacion-en-estructuras-1886766956", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H611" s="6" t="inlineStr"/>
@@ -29215,7 +29219,7 @@
     <row r="612" ht="22" customHeight="1">
       <c r="A612" s="2" t="inlineStr">
         <is>
-          <t>571ae2aa81fa07b5</t>
+          <t>13bc527565632878</t>
         </is>
       </c>
       <c r="B612" s="2" t="inlineStr">
@@ -29225,12 +29229,12 @@
       </c>
       <c r="C612" s="3" t="inlineStr">
         <is>
-          <t>Civil Engineering-in-Training</t>
+          <t>Tecnico en contratacion de obra civil bogota</t>
         </is>
       </c>
       <c r="D612" s="3" t="inlineStr">
         <is>
-          <t>WSP en Colombia</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="E612" s="8" t="n">
@@ -29242,7 +29246,7 @@
         </is>
       </c>
       <c r="G612" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-engineering-in-training-at-wsp-en-colombia-4458027784", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/tecnico-en-contratacion-de-obra-civil-bogota-1886759693", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H612" s="6" t="inlineStr"/>
@@ -29261,7 +29265,7 @@
     <row r="613" ht="22" customHeight="1">
       <c r="A613" s="2" t="inlineStr">
         <is>
-          <t>d94bcf92627b7b99</t>
+          <t>6ccccd3a1ba05f7f</t>
         </is>
       </c>
       <c r="B613" s="2" t="inlineStr">
@@ -29271,12 +29275,12 @@
       </c>
       <c r="C613" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero civil</t>
+          <t>14561-especialista interventoria-bogota</t>
         </is>
       </c>
       <c r="D613" s="3" t="inlineStr">
         <is>
-          <t>HMV Ingenieros</t>
+          <t>APPLUS NORCONTROL COLOMBIA LTDA</t>
         </is>
       </c>
       <c r="E613" s="8" t="n">
@@ -29288,7 +29292,7 @@
         </is>
       </c>
       <c r="G613" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-civil-at-hmv-ingenieros-4461715824", "Ver Vacante")</f>
+        <f>HYPERLINK("https://www.elempleo.com/co/ofertas-trabajo/14561especialista-interventoriabogota-1886768886", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H613" s="6" t="inlineStr"/>
@@ -29307,7 +29311,7 @@
     <row r="614" ht="22" customHeight="1">
       <c r="A614" s="2" t="inlineStr">
         <is>
-          <t>1be0a8e56fa4736b</t>
+          <t>8ad0c11c4f07472e</t>
         </is>
       </c>
       <c r="B614" s="2" t="inlineStr">
@@ -29317,12 +29321,12 @@
       </c>
       <c r="C614" s="3" t="inlineStr">
         <is>
-          <t>Civil Engineer</t>
+          <t>Ingeniero Civil / Terracerías</t>
         </is>
       </c>
       <c r="D614" s="3" t="inlineStr">
         <is>
-          <t>Wood</t>
+          <t>EOSOL</t>
         </is>
       </c>
       <c r="E614" s="8" t="n">
@@ -29334,7 +29338,7 @@
         </is>
       </c>
       <c r="G614" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-engineer-at-wood-4418961778", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-civil-terracer%C3%ADas-at-eosol-4445793534", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H614" s="6" t="inlineStr"/>
@@ -29353,7 +29357,7 @@
     <row r="615" ht="22" customHeight="1">
       <c r="A615" s="2" t="inlineStr">
         <is>
-          <t>825c4e246cbd6b6b</t>
+          <t>ed46085f88d06bf5</t>
         </is>
       </c>
       <c r="B615" s="2" t="inlineStr">
@@ -29363,12 +29367,12 @@
       </c>
       <c r="C615" s="3" t="inlineStr">
         <is>
-          <t>Civil Engineering Expert</t>
+          <t>Supervisor Civil</t>
         </is>
       </c>
       <c r="D615" s="3" t="inlineStr">
         <is>
-          <t>Anyone AI</t>
+          <t>EOSOL</t>
         </is>
       </c>
       <c r="E615" s="8" t="n">
@@ -29380,7 +29384,7 @@
         </is>
       </c>
       <c r="G615" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-engineering-expert-at-anyone-ai-4462461832", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/supervisor-civil-at-eosol-4442238964", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H615" s="6" t="inlineStr"/>
@@ -29399,7 +29403,7 @@
     <row r="616" ht="22" customHeight="1">
       <c r="A616" s="2" t="inlineStr">
         <is>
-          <t>76740179a82340ae</t>
+          <t>dc949850c44ae2c9</t>
         </is>
       </c>
       <c r="B616" s="2" t="inlineStr">
@@ -29409,12 +29413,12 @@
       </c>
       <c r="C616" s="3" t="inlineStr">
         <is>
-          <t>Profesional en Ingeniería Civil</t>
+          <t>Civil Engineer</t>
         </is>
       </c>
       <c r="D616" s="3" t="inlineStr">
         <is>
-          <t>CMH Colombia</t>
+          <t>Cresta</t>
         </is>
       </c>
       <c r="E616" s="8" t="n">
@@ -29426,7 +29430,7 @@
         </is>
       </c>
       <c r="G616" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/profesional-en-ingenier%C3%ADa-civil-at-minerales-c%C3%B3rdoba-4450022471", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-engineer-at-cresta-4465582487", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H616" s="6" t="inlineStr"/>
@@ -29445,7 +29449,7 @@
     <row r="617" ht="22" customHeight="1">
       <c r="A617" s="2" t="inlineStr">
         <is>
-          <t>5bea04b9e734c2fc</t>
+          <t>4ad1a5acabdb8ad3</t>
         </is>
       </c>
       <c r="B617" s="2" t="inlineStr">
@@ -29455,12 +29459,12 @@
       </c>
       <c r="C617" s="3" t="inlineStr">
         <is>
-          <t>Coordinador HSEQ</t>
+          <t>Civil BIM Specialist</t>
         </is>
       </c>
       <c r="D617" s="3" t="inlineStr">
         <is>
-          <t>ASSEMTEC</t>
+          <t>ENG</t>
         </is>
       </c>
       <c r="E617" s="8" t="n">
@@ -29472,13 +29476,13 @@
         </is>
       </c>
       <c r="G617" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-hseq-at-assemtec-4457664932", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-bim-specialist-at-eng-4469886677", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H617" s="6" t="inlineStr"/>
       <c r="I617" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J617" s="2" t="inlineStr">
@@ -29491,7 +29495,7 @@
     <row r="618" ht="22" customHeight="1">
       <c r="A618" s="2" t="inlineStr">
         <is>
-          <t>6ba6bae2d7bfb226</t>
+          <t>5ebaba0a0c9927fb</t>
         </is>
       </c>
       <c r="B618" s="2" t="inlineStr">
@@ -29501,12 +29505,12 @@
       </c>
       <c r="C618" s="3" t="inlineStr">
         <is>
-          <t>Inspector SST con Licencia, Coordinador de Alturas</t>
+          <t>Ingeniero/a Civil-Estructuras Hormigón/Acero</t>
         </is>
       </c>
       <c r="D618" s="3" t="inlineStr">
         <is>
-          <t>Asertempo Colombia S.A.S</t>
+          <t>IDOM Consulting, Engineering, Architecture</t>
         </is>
       </c>
       <c r="E618" s="8" t="n">
@@ -29518,13 +29522,13 @@
         </is>
       </c>
       <c r="G618" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/inspector-sst-con-licencia-coordinador-de-alturas-at-asertempo-colombia-s-a-s-4464408367", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-a-civil-estructuras-hormig%C3%B3n-acero-at-idom-consulting-engineering-architecture-4462998187", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H618" s="6" t="inlineStr"/>
       <c r="I618" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J618" s="2" t="inlineStr">
@@ -29537,7 +29541,7 @@
     <row r="619" ht="22" customHeight="1">
       <c r="A619" s="2" t="inlineStr">
         <is>
-          <t>0df4a63a82189896</t>
+          <t>5c954c66c2c9d655</t>
         </is>
       </c>
       <c r="B619" s="2" t="inlineStr">
@@ -29547,12 +29551,12 @@
       </c>
       <c r="C619" s="3" t="inlineStr">
         <is>
-          <t>Especialista en Salud y Seguridad en el trabajo con especialización en medio Ambiente</t>
+          <t>Civil Engineering-in-Training</t>
         </is>
       </c>
       <c r="D619" s="3" t="inlineStr">
         <is>
-          <t>Dextera IT Services</t>
+          <t>WSP en Colombia</t>
         </is>
       </c>
       <c r="E619" s="8" t="n">
@@ -29564,7 +29568,7 @@
         </is>
       </c>
       <c r="G619" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/especialista-en-salud-y-seguridad-en-el-trabajo-con-especializaci%C3%B3n-en-medio-ambiente-at-dextera-it-services-4464024362", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-engineering-in-training-french-at-wsp-en-colombia-4458430104", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H619" s="6" t="inlineStr"/>
@@ -29583,7 +29587,7 @@
     <row r="620" ht="22" customHeight="1">
       <c r="A620" s="2" t="inlineStr">
         <is>
-          <t>e8e3c75915d1945c</t>
+          <t>571ae2aa81fa07b5</t>
         </is>
       </c>
       <c r="B620" s="2" t="inlineStr">
@@ -29593,12 +29597,12 @@
       </c>
       <c r="C620" s="3" t="inlineStr">
         <is>
-          <t>Coordinador (a) profesional HSEQ</t>
+          <t>Civil Engineering-in-Training</t>
         </is>
       </c>
       <c r="D620" s="3" t="inlineStr">
         <is>
-          <t>SD SAS</t>
+          <t>WSP en Colombia</t>
         </is>
       </c>
       <c r="E620" s="8" t="n">
@@ -29610,13 +29614,13 @@
         </is>
       </c>
       <c r="G620" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-a-profesional-hseq-at-sd-sas-4444939872", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-engineering-in-training-at-wsp-en-colombia-4458027784", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H620" s="6" t="inlineStr"/>
       <c r="I620" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J620" s="2" t="inlineStr">
@@ -29629,7 +29633,7 @@
     <row r="621" ht="22" customHeight="1">
       <c r="A621" s="2" t="inlineStr">
         <is>
-          <t>fb37fc1bf485e650</t>
+          <t>d94bcf92627b7b99</t>
         </is>
       </c>
       <c r="B621" s="2" t="inlineStr">
@@ -29639,12 +29643,12 @@
       </c>
       <c r="C621" s="3" t="inlineStr">
         <is>
-          <t>Técnico de trazado especialista en ISTRAM</t>
+          <t>Ingeniero civil</t>
         </is>
       </c>
       <c r="D621" s="3" t="inlineStr">
         <is>
-          <t>EADIC</t>
+          <t>HMV Ingenieros</t>
         </is>
       </c>
       <c r="E621" s="8" t="n">
@@ -29656,7 +29660,7 @@
         </is>
       </c>
       <c r="G621" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/t%C3%A9cnico-de-trazado-especialista-en-istram-at-eadic-4468780158", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-civil-at-hmv-ingenieros-4461715824", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H621" s="6" t="inlineStr"/>
@@ -29675,7 +29679,7 @@
     <row r="622" ht="22" customHeight="1">
       <c r="A622" s="2" t="inlineStr">
         <is>
-          <t>0f01a66eb85a1ffd</t>
+          <t>1be0a8e56fa4736b</t>
         </is>
       </c>
       <c r="B622" s="2" t="inlineStr">
@@ -29685,12 +29689,12 @@
       </c>
       <c r="C622" s="3" t="inlineStr">
         <is>
-          <t>AUXILIAR MODELADOR BIM Y DIBUJANTE EN INGENIERÍA CIVIL</t>
+          <t>Civil Engineer</t>
         </is>
       </c>
       <c r="D622" s="3" t="inlineStr">
         <is>
-          <t>Antea Group España y Latinoamérica</t>
+          <t>Wood</t>
         </is>
       </c>
       <c r="E622" s="8" t="n">
@@ -29702,7 +29706,7 @@
         </is>
       </c>
       <c r="G622" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/auxiliar-modelador-bim-y-dibujante-en-ingenier%C3%ADa-civil-at-antea-group-espa%C3%B1a-y-latinoam%C3%A9rica-4467605615", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-engineer-at-wood-4418961778", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H622" s="6" t="inlineStr"/>
@@ -29721,7 +29725,7 @@
     <row r="623" ht="22" customHeight="1">
       <c r="A623" s="2" t="inlineStr">
         <is>
-          <t>cba614af5ce1fc3a</t>
+          <t>825c4e246cbd6b6b</t>
         </is>
       </c>
       <c r="B623" s="2" t="inlineStr">
@@ -29731,12 +29735,12 @@
       </c>
       <c r="C623" s="3" t="inlineStr">
         <is>
-          <t>Principal Pavement Engineer - Linear Infrastructure &amp; Site Civils</t>
+          <t>Civil Engineering Expert</t>
         </is>
       </c>
       <c r="D623" s="3" t="inlineStr">
         <is>
-          <t>AECOM</t>
+          <t>Anyone AI</t>
         </is>
       </c>
       <c r="E623" s="8" t="n">
@@ -29748,7 +29752,7 @@
         </is>
       </c>
       <c r="G623" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/principal-pavement-engineer-linear-infrastructure-site-civils-at-aecom-4403657428", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/civil-engineering-expert-at-anyone-ai-4462461832", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H623" s="6" t="inlineStr"/>
@@ -29767,7 +29771,7 @@
     <row r="624" ht="22" customHeight="1">
       <c r="A624" s="2" t="inlineStr">
         <is>
-          <t>2bafc4e5eb29746b</t>
+          <t>76740179a82340ae</t>
         </is>
       </c>
       <c r="B624" s="2" t="inlineStr">
@@ -29777,12 +29781,12 @@
       </c>
       <c r="C624" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero/a Geotécnico/a Senior</t>
+          <t>Profesional en Ingeniería Civil</t>
         </is>
       </c>
       <c r="D624" s="3" t="inlineStr">
         <is>
-          <t>IDOM Consulting, Engineering, Architecture</t>
+          <t>CMH Colombia</t>
         </is>
       </c>
       <c r="E624" s="8" t="n">
@@ -29794,7 +29798,7 @@
         </is>
       </c>
       <c r="G624" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-a-geot%C3%A9cnico-a-senior-at-idom-consulting-engineering-architecture-4467729578", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/profesional-en-ingenier%C3%ADa-civil-at-minerales-c%C3%B3rdoba-4450022471", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H624" s="6" t="inlineStr"/>
@@ -29813,7 +29817,7 @@
     <row r="625" ht="22" customHeight="1">
       <c r="A625" s="2" t="inlineStr">
         <is>
-          <t>f3290f3c2a2d0061</t>
+          <t>5bea04b9e734c2fc</t>
         </is>
       </c>
       <c r="B625" s="2" t="inlineStr">
@@ -29823,12 +29827,12 @@
       </c>
       <c r="C625" s="3" t="inlineStr">
         <is>
-          <t>Engenheiro Civil - Lisboa</t>
+          <t>Coordinador HSEQ</t>
         </is>
       </c>
       <c r="D625" s="3" t="inlineStr">
         <is>
-          <t>DDN GERENCIAMENTO</t>
+          <t>ASSEMTEC</t>
         </is>
       </c>
       <c r="E625" s="8" t="n">
@@ -29840,13 +29844,13 @@
         </is>
       </c>
       <c r="G625" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/engenheiro-civil-lisboa-at-ddn-gerenciamento-4468408791", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-hseq-at-assemtec-4457664932", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H625" s="6" t="inlineStr"/>
       <c r="I625" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J625" s="2" t="inlineStr">
@@ -29859,7 +29863,7 @@
     <row r="626" ht="22" customHeight="1">
       <c r="A626" s="2" t="inlineStr">
         <is>
-          <t>d2feccf91b9b1f0b</t>
+          <t>6ba6bae2d7bfb226</t>
         </is>
       </c>
       <c r="B626" s="2" t="inlineStr">
@@ -29869,12 +29873,12 @@
       </c>
       <c r="C626" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero/a Civil especialista en Talleres y Patios Ferroviarios</t>
+          <t>Inspector SST con Licencia, Coordinador de Alturas</t>
         </is>
       </c>
       <c r="D626" s="3" t="inlineStr">
         <is>
-          <t>IDOM Consulting, Engineering, Architecture</t>
+          <t>Asertempo Colombia S.A.S</t>
         </is>
       </c>
       <c r="E626" s="8" t="n">
@@ -29886,13 +29890,13 @@
         </is>
       </c>
       <c r="G626" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-a-civil-especialista-en-talleres-y-patios-ferroviarios-at-idom-consulting-engineering-architecture-4443713908", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/inspector-sst-con-licencia-coordinador-de-alturas-at-asertempo-colombia-s-a-s-4464408367", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H626" s="6" t="inlineStr"/>
       <c r="I626" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J626" s="2" t="inlineStr">
@@ -29905,7 +29909,7 @@
     <row r="627" ht="22" customHeight="1">
       <c r="A627" s="2" t="inlineStr">
         <is>
-          <t>152ea7f07f195fc8</t>
+          <t>0df4a63a82189896</t>
         </is>
       </c>
       <c r="B627" s="2" t="inlineStr">
@@ -29915,12 +29919,12 @@
       </c>
       <c r="C627" s="3" t="inlineStr">
         <is>
-          <t>COORDINADOR DE INTERVENTORÍA-NIVEL 1 SECTOR HIDROCARBUROS</t>
+          <t>Especialista en Salud y Seguridad en el trabajo con especialización en medio Ambiente</t>
         </is>
       </c>
       <c r="D627" s="3" t="inlineStr">
         <is>
-          <t>Centro de Empleo y Talento</t>
+          <t>Dextera IT Services</t>
         </is>
       </c>
       <c r="E627" s="8" t="n">
@@ -29932,7 +29936,7 @@
         </is>
       </c>
       <c r="G627" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-de-interventor%C3%ADa-nivel-1-sector-hidrocarburos-at-centro-de-empleo-y-talento-4468030406", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/especialista-en-salud-y-seguridad-en-el-trabajo-con-especializaci%C3%B3n-en-medio-ambiente-at-dextera-it-services-4464024362", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H627" s="6" t="inlineStr"/>
@@ -29951,7 +29955,7 @@
     <row r="628" ht="22" customHeight="1">
       <c r="A628" s="2" t="inlineStr">
         <is>
-          <t>b3dd7e9d8f53fb27</t>
+          <t>e8e3c75915d1945c</t>
         </is>
       </c>
       <c r="B628" s="2" t="inlineStr">
@@ -29961,12 +29965,12 @@
       </c>
       <c r="C628" s="3" t="inlineStr">
         <is>
-          <t>Consultor (Desarrollador) Senior Appian</t>
+          <t>Coordinador (a) profesional HSEQ</t>
         </is>
       </c>
       <c r="D628" s="3" t="inlineStr">
         <is>
-          <t>VASS LATAM</t>
+          <t>SD SAS</t>
         </is>
       </c>
       <c r="E628" s="8" t="n">
@@ -29978,13 +29982,13 @@
         </is>
       </c>
       <c r="G628" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/consultor-desarrollador-senior-appian-at-vass-latam-4458249659", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-a-profesional-hseq-at-sd-sas-4444939872", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H628" s="6" t="inlineStr"/>
       <c r="I628" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J628" s="2" t="inlineStr">
@@ -29997,7 +30001,7 @@
     <row r="629" ht="22" customHeight="1">
       <c r="A629" s="2" t="inlineStr">
         <is>
-          <t>0f895f69320d7d8d</t>
+          <t>fb37fc1bf485e650</t>
         </is>
       </c>
       <c r="B629" s="2" t="inlineStr">
@@ -30007,12 +30011,12 @@
       </c>
       <c r="C629" s="3" t="inlineStr">
         <is>
-          <t>Coordinador hse Cartagena</t>
+          <t>Técnico de trazado especialista en ISTRAM</t>
         </is>
       </c>
       <c r="D629" s="3" t="inlineStr">
         <is>
-          <t>TRANSPORTES MONTEJO SAS</t>
+          <t>EADIC</t>
         </is>
       </c>
       <c r="E629" s="8" t="n">
@@ -30024,13 +30028,13 @@
         </is>
       </c>
       <c r="G629" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-hse-cartagena-at-transportes-montejo-sas-4458746462", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/t%C3%A9cnico-de-trazado-especialista-en-istram-at-eadic-4468780158", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H629" s="6" t="inlineStr"/>
       <c r="I629" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J629" s="2" t="inlineStr">
@@ -30043,7 +30047,7 @@
     <row r="630" ht="22" customHeight="1">
       <c r="A630" s="2" t="inlineStr">
         <is>
-          <t>b86d50ad2dd5f642</t>
+          <t>0f01a66eb85a1ffd</t>
         </is>
       </c>
       <c r="B630" s="2" t="inlineStr">
@@ -30053,12 +30057,12 @@
       </c>
       <c r="C630" s="3" t="inlineStr">
         <is>
-          <t>Coordinador Regional SIG/ SST</t>
+          <t>AUXILIAR MODELADOR BIM Y DIBUJANTE EN INGENIERÍA CIVIL</t>
         </is>
       </c>
       <c r="D630" s="3" t="inlineStr">
         <is>
-          <t>Interaseo S.A.S. E.S.P.</t>
+          <t>Antea Group España y Latinoamérica</t>
         </is>
       </c>
       <c r="E630" s="8" t="n">
@@ -30070,13 +30074,13 @@
         </is>
       </c>
       <c r="G630" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-regional-sig-sst-at-interaseo-s-a-s-e-s-p-4459088040", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/auxiliar-modelador-bim-y-dibujante-en-ingenier%C3%ADa-civil-at-antea-group-espa%C3%B1a-y-latinoam%C3%A9rica-4467605615", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H630" s="6" t="inlineStr"/>
       <c r="I630" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J630" s="2" t="inlineStr">
@@ -30089,7 +30093,7 @@
     <row r="631" ht="22" customHeight="1">
       <c r="A631" s="2" t="inlineStr">
         <is>
-          <t>506296811a5a9cbb</t>
+          <t>cba614af5ce1fc3a</t>
         </is>
       </c>
       <c r="B631" s="2" t="inlineStr">
@@ -30099,12 +30103,12 @@
       </c>
       <c r="C631" s="3" t="inlineStr">
         <is>
-          <t>Coordinador/a de SST</t>
+          <t>Principal Pavement Engineer - Linear Infrastructure &amp; Site Civils</t>
         </is>
       </c>
       <c r="D631" s="3" t="inlineStr">
         <is>
-          <t>Estelar Food S.A.S</t>
+          <t>AECOM</t>
         </is>
       </c>
       <c r="E631" s="8" t="n">
@@ -30116,13 +30120,13 @@
         </is>
       </c>
       <c r="G631" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-a-de-sst-at-estelar-food-s-a-s-4462115593", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/principal-pavement-engineer-linear-infrastructure-site-civils-at-aecom-4403657428", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H631" s="6" t="inlineStr"/>
       <c r="I631" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J631" s="2" t="inlineStr">
@@ -30135,7 +30139,7 @@
     <row r="632" ht="22" customHeight="1">
       <c r="A632" s="2" t="inlineStr">
         <is>
-          <t>0e4b8eed7f32714e</t>
+          <t>2bafc4e5eb29746b</t>
         </is>
       </c>
       <c r="B632" s="2" t="inlineStr">
@@ -30145,12 +30149,12 @@
       </c>
       <c r="C632" s="3" t="inlineStr">
         <is>
-          <t>coordinador de Seguridad y Salud en el Trabajo</t>
+          <t>Ingeniero/a Geotécnico/a Senior</t>
         </is>
       </c>
       <c r="D632" s="3" t="inlineStr">
         <is>
-          <t>Asertempo Colombia S.A.S</t>
+          <t>IDOM Consulting, Engineering, Architecture</t>
         </is>
       </c>
       <c r="E632" s="8" t="n">
@@ -30162,13 +30166,13 @@
         </is>
       </c>
       <c r="G632" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-de-seguridad-y-salud-en-el-trabajo-at-asertempo-colombia-s-a-s-4461723686", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-a-geot%C3%A9cnico-a-senior-at-idom-consulting-engineering-architecture-4467729578", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H632" s="6" t="inlineStr"/>
       <c r="I632" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J632" s="2" t="inlineStr">
@@ -30181,7 +30185,7 @@
     <row r="633" ht="22" customHeight="1">
       <c r="A633" s="2" t="inlineStr">
         <is>
-          <t>aa2882af3c61095b</t>
+          <t>f3290f3c2a2d0061</t>
         </is>
       </c>
       <c r="B633" s="2" t="inlineStr">
@@ -30191,12 +30195,12 @@
       </c>
       <c r="C633" s="3" t="inlineStr">
         <is>
-          <t>Coordinador (a) SST / APH - Marmato</t>
+          <t>Engenheiro Civil - Lisboa</t>
         </is>
       </c>
       <c r="D633" s="3" t="inlineStr">
         <is>
-          <t>Aris Mining Colombia</t>
+          <t>DDN GERENCIAMENTO</t>
         </is>
       </c>
       <c r="E633" s="8" t="n">
@@ -30208,13 +30212,13 @@
         </is>
       </c>
       <c r="G633" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-a-sst-aph-marmato-at-aris-mining-colombia-4448929810", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/engenheiro-civil-lisboa-at-ddn-gerenciamento-4468408791", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H633" s="6" t="inlineStr"/>
       <c r="I633" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J633" s="2" t="inlineStr">
@@ -30227,7 +30231,7 @@
     <row r="634" ht="22" customHeight="1">
       <c r="A634" s="2" t="inlineStr">
         <is>
-          <t>26cff43f13982962</t>
+          <t>d2feccf91b9b1f0b</t>
         </is>
       </c>
       <c r="B634" s="2" t="inlineStr">
@@ -30237,12 +30241,12 @@
       </c>
       <c r="C634" s="3" t="inlineStr">
         <is>
-          <t>Consultor(a) Senior SOX TI</t>
+          <t>Ingeniero/a Civil especialista en Talleres y Patios Ferroviarios</t>
         </is>
       </c>
       <c r="D634" s="3" t="inlineStr">
         <is>
-          <t>Hitss Colombia</t>
+          <t>IDOM Consulting, Engineering, Architecture</t>
         </is>
       </c>
       <c r="E634" s="8" t="n">
@@ -30254,7 +30258,7 @@
         </is>
       </c>
       <c r="G634" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/consultor-a-senior-sox-ti-at-hitss-colombia-4460766744", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-a-civil-especialista-en-talleres-y-patios-ferroviarios-at-idom-consulting-engineering-architecture-4443713908", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H634" s="6" t="inlineStr"/>
@@ -30273,7 +30277,7 @@
     <row r="635" ht="22" customHeight="1">
       <c r="A635" s="2" t="inlineStr">
         <is>
-          <t>87e367215ed55502</t>
+          <t>152ea7f07f195fc8</t>
         </is>
       </c>
       <c r="B635" s="2" t="inlineStr">
@@ -30283,12 +30287,12 @@
       </c>
       <c r="C635" s="3" t="inlineStr">
         <is>
-          <t>Consultor(a) Senior Auditoría Interna</t>
+          <t>COORDINADOR DE INTERVENTORÍA-NIVEL 1 SECTOR HIDROCARBUROS</t>
         </is>
       </c>
       <c r="D635" s="3" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>Centro de Empleo y Talento</t>
         </is>
       </c>
       <c r="E635" s="8" t="n">
@@ -30300,7 +30304,7 @@
         </is>
       </c>
       <c r="G635" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/consultor-a-senior-auditor%C3%ADa-interna-at-deloitte-4462090075", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-de-interventor%C3%ADa-nivel-1-sector-hidrocarburos-at-centro-de-empleo-y-talento-4468030406", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H635" s="6" t="inlineStr"/>
@@ -30319,7 +30323,7 @@
     <row r="636" ht="22" customHeight="1">
       <c r="A636" s="2" t="inlineStr">
         <is>
-          <t>e2e525b51bbd0e5e</t>
+          <t>b3dd7e9d8f53fb27</t>
         </is>
       </c>
       <c r="B636" s="2" t="inlineStr">
@@ -30329,12 +30333,12 @@
       </c>
       <c r="C636" s="3" t="inlineStr">
         <is>
-          <t>Coordinador/a de Salud y Bienestar (HSE) Latam</t>
+          <t>Consultor (Desarrollador) Senior Appian</t>
         </is>
       </c>
       <c r="D636" s="3" t="inlineStr">
         <is>
-          <t>Aqualia</t>
+          <t>VASS LATAM</t>
         </is>
       </c>
       <c r="E636" s="8" t="n">
@@ -30346,13 +30350,13 @@
         </is>
       </c>
       <c r="G636" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-a-de-salud-y-bienestar-hse-latam-at-aqualia-4463977352", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/consultor-desarrollador-senior-appian-at-vass-latam-4458249659", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H636" s="6" t="inlineStr"/>
       <c r="I636" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J636" s="2" t="inlineStr">
@@ -30365,7 +30369,7 @@
     <row r="637" ht="22" customHeight="1">
       <c r="A637" s="2" t="inlineStr">
         <is>
-          <t>8ef614b651dfe9d9</t>
+          <t>0f895f69320d7d8d</t>
         </is>
       </c>
       <c r="B637" s="2" t="inlineStr">
@@ -30375,12 +30379,12 @@
       </c>
       <c r="C637" s="3" t="inlineStr">
         <is>
-          <t>Lead Civil Site Engineer</t>
+          <t>Coordinador hse Cartagena</t>
         </is>
       </c>
       <c r="D637" s="3" t="inlineStr">
         <is>
-          <t>AECOM</t>
+          <t>TRANSPORTES MONTEJO SAS</t>
         </is>
       </c>
       <c r="E637" s="8" t="n">
@@ -30392,13 +30396,13 @@
         </is>
       </c>
       <c r="G637" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/lead-civil-site-engineer-at-aecom-4468059409", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-hse-cartagena-at-transportes-montejo-sas-4458746462", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H637" s="6" t="inlineStr"/>
       <c r="I637" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J637" s="2" t="inlineStr">
@@ -30411,7 +30415,7 @@
     <row r="638" ht="22" customHeight="1">
       <c r="A638" s="2" t="inlineStr">
         <is>
-          <t>b339389a0d32a94f</t>
+          <t>b86d50ad2dd5f642</t>
         </is>
       </c>
       <c r="B638" s="2" t="inlineStr">
@@ -30421,12 +30425,12 @@
       </c>
       <c r="C638" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero civil</t>
+          <t>Coordinador Regional SIG/ SST</t>
         </is>
       </c>
       <c r="D638" s="3" t="inlineStr">
         <is>
-          <t>constructora cumbrera</t>
+          <t>Interaseo S.A.S. E.S.P.</t>
         </is>
       </c>
       <c r="E638" s="8" t="n">
@@ -30438,13 +30442,13 @@
         </is>
       </c>
       <c r="G638" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-civil-4463108593", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-regional-sig-sst-at-interaseo-s-a-s-e-s-p-4459088040", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H638" s="6" t="inlineStr"/>
       <c r="I638" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J638" s="2" t="inlineStr">
@@ -30457,7 +30461,7 @@
     <row r="639" ht="22" customHeight="1">
       <c r="A639" s="2" t="inlineStr">
         <is>
-          <t>93623c0212e39cb9</t>
+          <t>506296811a5a9cbb</t>
         </is>
       </c>
       <c r="B639" s="2" t="inlineStr">
@@ -30467,12 +30471,12 @@
       </c>
       <c r="C639" s="3" t="inlineStr">
         <is>
-          <t>Ingeniero(a) Civil</t>
+          <t>Coordinador/a de SST</t>
         </is>
       </c>
       <c r="D639" s="3" t="inlineStr">
         <is>
-          <t>CMH Colombia</t>
+          <t>Estelar Food S.A.S</t>
         </is>
       </c>
       <c r="E639" s="8" t="n">
@@ -30484,13 +30488,13 @@
         </is>
       </c>
       <c r="G639" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-a-civil-at-minerales-c%C3%B3rdoba-4417533007", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-a-de-sst-at-estelar-food-s-a-s-4462115593", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H639" s="6" t="inlineStr"/>
       <c r="I639" s="3" t="inlineStr">
         <is>
-          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
       <c r="J639" s="2" t="inlineStr">
@@ -30503,7 +30507,7 @@
     <row r="640" ht="22" customHeight="1">
       <c r="A640" s="2" t="inlineStr">
         <is>
-          <t>cd06fbe3d5b74888</t>
+          <t>0e4b8eed7f32714e</t>
         </is>
       </c>
       <c r="B640" s="2" t="inlineStr">
@@ -30513,12 +30517,12 @@
       </c>
       <c r="C640" s="3" t="inlineStr">
         <is>
-          <t>Oficial Obra Civil</t>
+          <t>coordinador de Seguridad y Salud en el Trabajo</t>
         </is>
       </c>
       <c r="D640" s="3" t="inlineStr">
         <is>
-          <t>Equans Colombia</t>
+          <t>Asertempo Colombia S.A.S</t>
         </is>
       </c>
       <c r="E640" s="8" t="n">
@@ -30530,25 +30534,393 @@
         </is>
       </c>
       <c r="G640" s="5">
-        <f>HYPERLINK("https://co.linkedin.com/jobs/view/oficial-obra-civil-bogota-y-cundinamarca-at-equans-colombia-4470218146", "Ver Vacante")</f>
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-de-seguridad-y-salud-en-el-trabajo-at-asertempo-colombia-s-a-s-4461723686", "Ver Vacante")</f>
         <v/>
       </c>
       <c r="H640" s="6" t="inlineStr"/>
       <c r="I640" s="3" t="inlineStr">
         <is>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J640" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K640" s="3" t="inlineStr"/>
+    </row>
+    <row r="641" ht="22" customHeight="1">
+      <c r="A641" s="2" t="inlineStr">
+        <is>
+          <t>aa2882af3c61095b</t>
+        </is>
+      </c>
+      <c r="B641" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 05:09</t>
+        </is>
+      </c>
+      <c r="C641" s="3" t="inlineStr">
+        <is>
+          <t>Coordinador (a) SST / APH - Marmato</t>
+        </is>
+      </c>
+      <c r="D641" s="3" t="inlineStr">
+        <is>
+          <t>Aris Mining Colombia</t>
+        </is>
+      </c>
+      <c r="E641" s="8" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F641" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G641" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-a-sst-aph-marmato-at-aris-mining-colombia-4448929810", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H641" s="6" t="inlineStr"/>
+      <c r="I641" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J641" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K641" s="3" t="inlineStr"/>
+    </row>
+    <row r="642" ht="22" customHeight="1">
+      <c r="A642" s="2" t="inlineStr">
+        <is>
+          <t>26cff43f13982962</t>
+        </is>
+      </c>
+      <c r="B642" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 05:09</t>
+        </is>
+      </c>
+      <c r="C642" s="3" t="inlineStr">
+        <is>
+          <t>Consultor(a) Senior SOX TI</t>
+        </is>
+      </c>
+      <c r="D642" s="3" t="inlineStr">
+        <is>
+          <t>Hitss Colombia</t>
+        </is>
+      </c>
+      <c r="E642" s="8" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F642" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G642" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/consultor-a-senior-sox-ti-at-hitss-colombia-4460766744", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H642" s="6" t="inlineStr"/>
+      <c r="I642" s="3" t="inlineStr">
+        <is>
           <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
         </is>
       </c>
-      <c r="J640" s="2" t="inlineStr">
-        <is>
-          <t>Nueva</t>
-        </is>
-      </c>
-      <c r="K640" s="3" t="inlineStr"/>
+      <c r="J642" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K642" s="3" t="inlineStr"/>
+    </row>
+    <row r="643" ht="22" customHeight="1">
+      <c r="A643" s="2" t="inlineStr">
+        <is>
+          <t>87e367215ed55502</t>
+        </is>
+      </c>
+      <c r="B643" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 05:09</t>
+        </is>
+      </c>
+      <c r="C643" s="3" t="inlineStr">
+        <is>
+          <t>Consultor(a) Senior Auditoría Interna</t>
+        </is>
+      </c>
+      <c r="D643" s="3" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+      <c r="E643" s="8" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F643" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G643" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/consultor-a-senior-auditor%C3%ADa-interna-at-deloitte-4462090075", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H643" s="6" t="inlineStr"/>
+      <c r="I643" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J643" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K643" s="3" t="inlineStr"/>
+    </row>
+    <row r="644" ht="22" customHeight="1">
+      <c r="A644" s="2" t="inlineStr">
+        <is>
+          <t>e2e525b51bbd0e5e</t>
+        </is>
+      </c>
+      <c r="B644" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 05:09</t>
+        </is>
+      </c>
+      <c r="C644" s="3" t="inlineStr">
+        <is>
+          <t>Coordinador/a de Salud y Bienestar (HSE) Latam</t>
+        </is>
+      </c>
+      <c r="D644" s="3" t="inlineStr">
+        <is>
+          <t>Aqualia</t>
+        </is>
+      </c>
+      <c r="E644" s="8" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F644" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G644" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/coordinador-a-de-salud-y-bienestar-hse-latam-at-aqualia-4463977352", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H644" s="6" t="inlineStr"/>
+      <c r="I644" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad parcial en seguridad y salud ocupacional. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J644" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K644" s="3" t="inlineStr"/>
+    </row>
+    <row r="645" ht="22" customHeight="1">
+      <c r="A645" s="2" t="inlineStr">
+        <is>
+          <t>8ef614b651dfe9d9</t>
+        </is>
+      </c>
+      <c r="B645" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 05:09</t>
+        </is>
+      </c>
+      <c r="C645" s="3" t="inlineStr">
+        <is>
+          <t>Lead Civil Site Engineer</t>
+        </is>
+      </c>
+      <c r="D645" s="3" t="inlineStr">
+        <is>
+          <t>AECOM</t>
+        </is>
+      </c>
+      <c r="E645" s="8" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F645" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G645" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/lead-civil-site-engineer-at-aecom-4468059409", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H645" s="6" t="inlineStr"/>
+      <c r="I645" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J645" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K645" s="3" t="inlineStr"/>
+    </row>
+    <row r="646" ht="22" customHeight="1">
+      <c r="A646" s="2" t="inlineStr">
+        <is>
+          <t>b339389a0d32a94f</t>
+        </is>
+      </c>
+      <c r="B646" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 05:09</t>
+        </is>
+      </c>
+      <c r="C646" s="3" t="inlineStr">
+        <is>
+          <t>Ingeniero civil</t>
+        </is>
+      </c>
+      <c r="D646" s="3" t="inlineStr">
+        <is>
+          <t>constructora cumbrera</t>
+        </is>
+      </c>
+      <c r="E646" s="8" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F646" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G646" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-civil-4463108593", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H646" s="6" t="inlineStr"/>
+      <c r="I646" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J646" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K646" s="3" t="inlineStr"/>
+    </row>
+    <row r="647" ht="22" customHeight="1">
+      <c r="A647" s="2" t="inlineStr">
+        <is>
+          <t>93623c0212e39cb9</t>
+        </is>
+      </c>
+      <c r="B647" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 05:09</t>
+        </is>
+      </c>
+      <c r="C647" s="3" t="inlineStr">
+        <is>
+          <t>Ingeniero(a) Civil</t>
+        </is>
+      </c>
+      <c r="D647" s="3" t="inlineStr">
+        <is>
+          <t>CMH Colombia</t>
+        </is>
+      </c>
+      <c r="E647" s="8" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F647" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G647" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/ingeniero-a-civil-at-minerales-c%C3%B3rdoba-4417533007", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H647" s="6" t="inlineStr"/>
+      <c r="I647" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J647" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K647" s="3" t="inlineStr"/>
+    </row>
+    <row r="648" ht="22" customHeight="1">
+      <c r="A648" s="2" t="inlineStr">
+        <is>
+          <t>cd06fbe3d5b74888</t>
+        </is>
+      </c>
+      <c r="B648" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 05:09</t>
+        </is>
+      </c>
+      <c r="C648" s="3" t="inlineStr">
+        <is>
+          <t>Oficial Obra Civil</t>
+        </is>
+      </c>
+      <c r="D648" s="3" t="inlineStr">
+        <is>
+          <t>Equans Colombia</t>
+        </is>
+      </c>
+      <c r="E648" s="8" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F648" s="2" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="G648" s="5">
+        <f>HYPERLINK("https://co.linkedin.com/jobs/view/oficial-obra-civil-bogota-y-cundinamarca-at-equans-colombia-4470218146", "Ver Vacante")</f>
+        <v/>
+      </c>
+      <c r="H648" s="6" t="inlineStr"/>
+      <c r="I648" s="3" t="inlineStr">
+        <is>
+          <t>[Afinidad: 45/100 - Baja Afinidad] Afinidad en disciplina base (Ingeniera Civil Especialista en Vías y SST) sin especialidad directa en vías/SST. Modalidad: 100% Remoto en Colombia confirmado.</t>
+        </is>
+      </c>
+      <c r="J648" s="2" t="inlineStr">
+        <is>
+          <t>Nueva</t>
+        </is>
+      </c>
+      <c r="K648" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J839" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J847" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Nueva,Por revisar,Postulado,Descartado,Entrevista"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>